<commit_message>
APRESENTAÇÃO DA VERSÃO 1.0 AMANHÃ, LASCOU
</commit_message>
<xml_diff>
--- a/Calculo_Comissoes_10_2025.xlsx
+++ b/Calculo_Comissoes_10_2025.xlsx
@@ -3953,7 +3953,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S2"/>
+  <dimension ref="A1:S3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4070,11 +4070,11 @@
         </is>
       </c>
       <c r="E2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>ISCO</t>
+          <t>YSI</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -4089,39 +4089,111 @@
         <v>25</v>
       </c>
       <c r="J2" t="n">
-        <v>0</v>
+        <v>14.6416</v>
       </c>
       <c r="K2" t="n">
         <v>10</v>
       </c>
       <c r="L2" t="inlineStr">
         <is>
-          <t>meta_fornecedor_2</t>
+          <t>meta_fornecedor_1</t>
         </is>
       </c>
       <c r="M2" t="n">
         <v>0.1</v>
       </c>
       <c r="N2" t="n">
+        <v>0.585664</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0.585664</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0.0585664</v>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>[]</t>
+        </is>
+      </c>
+      <c r="S2" t="b">
         <v>0</v>
       </c>
-      <c r="O2" t="n">
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>André Caramello</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Gerente Linha</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Hidrologia</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>2</v>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>ISCO</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+      <c r="H3" t="n">
+        <v>30</v>
+      </c>
+      <c r="I3" t="n">
+        <v>25</v>
+      </c>
+      <c r="J3" t="n">
         <v>0</v>
       </c>
-      <c r="P2" t="n">
+      <c r="K3" t="n">
+        <v>10</v>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>meta_fornecedor_2</t>
+        </is>
+      </c>
+      <c r="M3" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="N3" t="n">
         <v>0</v>
       </c>
-      <c r="Q2" t="inlineStr">
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="inlineStr">
         <is>
           <t>{}</t>
         </is>
       </c>
-      <c r="R2" t="inlineStr">
+      <c r="R3" t="inlineStr">
         <is>
           <t>[]</t>
         </is>
       </c>
-      <c r="S2" t="b">
+      <c r="S3" t="b">
         <v>0</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Primeiro Backup para apresentação do robô amanhã
</commit_message>
<xml_diff>
--- a/Calculo_Comissoes_10_2025.xlsx
+++ b/Calculo_Comissoes_10_2025.xlsx
@@ -4089,7 +4089,7 @@
         <v>25</v>
       </c>
       <c r="J2" t="n">
-        <v>14.6416</v>
+        <v>14.85573769241505</v>
       </c>
       <c r="K2" t="n">
         <v>10</v>
@@ -4103,13 +4103,13 @@
         <v>0.1</v>
       </c>
       <c r="N2" t="n">
-        <v>0.585664</v>
+        <v>0.594229507696602</v>
       </c>
       <c r="O2" t="n">
-        <v>0.585664</v>
+        <v>0.594229507696602</v>
       </c>
       <c r="P2" t="n">
-        <v>0.0585664</v>
+        <v>0.0594229507696602</v>
       </c>
       <c r="Q2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
BACKUP 2 ANTES DA APRESENTAÇÃO 10:27 DO DIA 19/12
</commit_message>
<xml_diff>
--- a/Calculo_Comissoes_10_2025.xlsx
+++ b/Calculo_Comissoes_10_2025.xlsx
@@ -14,9 +14,10 @@
     <sheet name="DEBUG_ANALISE_INFO" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="DEBUG_ANALISE_SAMPLE" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="DEBUG_FORNECEDORES" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="RECONCILIACAO" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="ESTADO" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="DEBUG_PAGAMENTOS_FINANCEIRO" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="CROSS_SELLING_DECISIONS" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="RECONCILIACAO" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="ESTADO" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="DEBUG_PAGAMENTOS_FINANCEIRO" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -25,7 +26,9 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="0"/>
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -118,11 +121,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="20">
+  <cellXfs count="22">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -159,6 +163,7 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -524,7 +529,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:BO16"/>
+  <dimension ref="A1:BP18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -593,257 +598,257 @@
           <t>percentual_elegibilidade_pe</t>
         </is>
       </c>
-      <c r="N1" s="2" t="inlineStr">
+      <c r="N1" s="3" t="inlineStr">
         <is>
           <t>fator_correcao_fc</t>
         </is>
       </c>
-      <c r="O1" s="3" t="inlineStr">
+      <c r="O1" s="4" t="inlineStr">
         <is>
           <t>peso_fat_linha</t>
         </is>
       </c>
-      <c r="P1" s="3" t="inlineStr">
+      <c r="P1" s="4" t="inlineStr">
         <is>
           <t>realizado_fat_linha</t>
         </is>
       </c>
-      <c r="Q1" s="3" t="inlineStr">
+      <c r="Q1" s="4" t="inlineStr">
         <is>
           <t>meta_fat_linha</t>
         </is>
       </c>
-      <c r="R1" s="3" t="inlineStr">
+      <c r="R1" s="4" t="inlineStr">
         <is>
           <t>ating_fat_linha</t>
         </is>
       </c>
-      <c r="S1" s="3" t="inlineStr">
+      <c r="S1" s="4" t="inlineStr">
         <is>
           <t>ating_cap_fat_linha</t>
         </is>
       </c>
-      <c r="T1" s="3" t="inlineStr">
+      <c r="T1" s="4" t="inlineStr">
         <is>
           <t>comp_fc_fat_linha</t>
         </is>
       </c>
-      <c r="U1" s="4" t="inlineStr">
+      <c r="U1" s="5" t="inlineStr">
         <is>
           <t>peso_conv_linha</t>
         </is>
       </c>
-      <c r="V1" s="4" t="inlineStr">
+      <c r="V1" s="5" t="inlineStr">
         <is>
           <t>realizado_conv_linha</t>
         </is>
       </c>
-      <c r="W1" s="4" t="inlineStr">
+      <c r="W1" s="5" t="inlineStr">
         <is>
           <t>meta_conv_linha</t>
         </is>
       </c>
-      <c r="X1" s="4" t="inlineStr">
+      <c r="X1" s="5" t="inlineStr">
         <is>
           <t>ating_conv_linha</t>
         </is>
       </c>
-      <c r="Y1" s="4" t="inlineStr">
+      <c r="Y1" s="5" t="inlineStr">
         <is>
           <t>ating_cap_conv_linha</t>
         </is>
       </c>
-      <c r="Z1" s="4" t="inlineStr">
+      <c r="Z1" s="5" t="inlineStr">
         <is>
           <t>comp_fc_conv_linha</t>
         </is>
       </c>
-      <c r="AA1" s="5" t="inlineStr">
+      <c r="AA1" s="6" t="inlineStr">
         <is>
           <t>peso_fat_ind</t>
         </is>
       </c>
-      <c r="AB1" s="5" t="inlineStr">
+      <c r="AB1" s="6" t="inlineStr">
         <is>
           <t>realizado_fat_ind</t>
         </is>
       </c>
-      <c r="AC1" s="5" t="inlineStr">
+      <c r="AC1" s="6" t="inlineStr">
         <is>
           <t>meta_fat_ind</t>
         </is>
       </c>
-      <c r="AD1" s="5" t="inlineStr">
+      <c r="AD1" s="6" t="inlineStr">
         <is>
           <t>ating_fat_ind</t>
         </is>
       </c>
-      <c r="AE1" s="5" t="inlineStr">
+      <c r="AE1" s="6" t="inlineStr">
         <is>
           <t>ating_cap_fat_ind</t>
         </is>
       </c>
-      <c r="AF1" s="5" t="inlineStr">
+      <c r="AF1" s="6" t="inlineStr">
         <is>
           <t>comp_fc_fat_ind</t>
         </is>
       </c>
-      <c r="AG1" s="6" t="inlineStr">
+      <c r="AG1" s="7" t="inlineStr">
         <is>
           <t>peso_conv_ind</t>
         </is>
       </c>
-      <c r="AH1" s="6" t="inlineStr">
+      <c r="AH1" s="7" t="inlineStr">
         <is>
           <t>realizado_conv_ind</t>
         </is>
       </c>
-      <c r="AI1" s="6" t="inlineStr">
+      <c r="AI1" s="7" t="inlineStr">
         <is>
           <t>meta_conv_ind</t>
         </is>
       </c>
-      <c r="AJ1" s="6" t="inlineStr">
+      <c r="AJ1" s="7" t="inlineStr">
         <is>
           <t>ating_conv_ind</t>
         </is>
       </c>
-      <c r="AK1" s="6" t="inlineStr">
+      <c r="AK1" s="7" t="inlineStr">
         <is>
           <t>ating_cap_conv_ind</t>
         </is>
       </c>
-      <c r="AL1" s="6" t="inlineStr">
+      <c r="AL1" s="7" t="inlineStr">
         <is>
           <t>comp_fc_conv_ind</t>
         </is>
       </c>
-      <c r="AM1" s="7" t="inlineStr">
+      <c r="AM1" s="8" t="inlineStr">
         <is>
           <t>peso_rentab</t>
         </is>
       </c>
-      <c r="AN1" s="7" t="inlineStr">
+      <c r="AN1" s="8" t="inlineStr">
         <is>
           <t>realizado_rentab</t>
         </is>
       </c>
-      <c r="AO1" s="7" t="inlineStr">
+      <c r="AO1" s="8" t="inlineStr">
         <is>
           <t>meta_rentab</t>
         </is>
       </c>
-      <c r="AP1" s="7" t="inlineStr">
+      <c r="AP1" s="8" t="inlineStr">
         <is>
           <t>ating_rentab</t>
         </is>
       </c>
-      <c r="AQ1" s="7" t="inlineStr">
+      <c r="AQ1" s="8" t="inlineStr">
         <is>
           <t>ating_cap_rentab</t>
         </is>
       </c>
-      <c r="AR1" s="7" t="inlineStr">
+      <c r="AR1" s="8" t="inlineStr">
         <is>
           <t>comp_fc_rentab</t>
         </is>
       </c>
-      <c r="AS1" s="8" t="inlineStr">
+      <c r="AS1" s="9" t="inlineStr">
         <is>
           <t>peso_retencao</t>
         </is>
       </c>
-      <c r="AT1" s="8" t="inlineStr">
+      <c r="AT1" s="9" t="inlineStr">
         <is>
           <t>realizado_retencao</t>
         </is>
       </c>
-      <c r="AU1" s="8" t="inlineStr">
+      <c r="AU1" s="9" t="inlineStr">
         <is>
           <t>meta_retencao</t>
         </is>
       </c>
-      <c r="AV1" s="8" t="inlineStr">
+      <c r="AV1" s="9" t="inlineStr">
         <is>
           <t>ating_retencao</t>
         </is>
       </c>
-      <c r="AW1" s="8" t="inlineStr">
+      <c r="AW1" s="9" t="inlineStr">
         <is>
           <t>ating_cap_retencao</t>
         </is>
       </c>
-      <c r="AX1" s="8" t="inlineStr">
+      <c r="AX1" s="9" t="inlineStr">
         <is>
           <t>comp_fc_retencao</t>
         </is>
       </c>
-      <c r="AY1" s="9" t="inlineStr">
+      <c r="AY1" s="10" t="inlineStr">
         <is>
           <t>peso_forn1</t>
         </is>
       </c>
-      <c r="AZ1" s="9" t="inlineStr">
+      <c r="AZ1" s="10" t="inlineStr">
         <is>
           <t>realizado_forn1</t>
         </is>
       </c>
-      <c r="BA1" s="9" t="inlineStr">
+      <c r="BA1" s="10" t="inlineStr">
         <is>
           <t>meta_forn1</t>
         </is>
       </c>
-      <c r="BB1" s="9" t="inlineStr">
+      <c r="BB1" s="10" t="inlineStr">
         <is>
           <t>ating_forn1</t>
         </is>
       </c>
-      <c r="BC1" s="9" t="inlineStr">
+      <c r="BC1" s="10" t="inlineStr">
         <is>
           <t>ating_cap_forn1</t>
         </is>
       </c>
-      <c r="BD1" s="9" t="inlineStr">
+      <c r="BD1" s="10" t="inlineStr">
         <is>
           <t>comp_fc_forn1</t>
         </is>
       </c>
-      <c r="BE1" s="9" t="inlineStr">
+      <c r="BE1" s="10" t="inlineStr">
         <is>
           <t>moeda_forn1</t>
         </is>
       </c>
-      <c r="BF1" s="10" t="inlineStr">
+      <c r="BF1" s="11" t="inlineStr">
         <is>
           <t>peso_forn2</t>
         </is>
       </c>
-      <c r="BG1" s="10" t="inlineStr">
+      <c r="BG1" s="11" t="inlineStr">
         <is>
           <t>realizado_forn2</t>
         </is>
       </c>
-      <c r="BH1" s="10" t="inlineStr">
+      <c r="BH1" s="11" t="inlineStr">
         <is>
           <t>meta_forn2</t>
         </is>
       </c>
-      <c r="BI1" s="10" t="inlineStr">
+      <c r="BI1" s="11" t="inlineStr">
         <is>
           <t>ating_forn2</t>
         </is>
       </c>
-      <c r="BJ1" s="10" t="inlineStr">
+      <c r="BJ1" s="11" t="inlineStr">
         <is>
           <t>ating_cap_forn2</t>
         </is>
       </c>
-      <c r="BK1" s="10" t="inlineStr">
+      <c r="BK1" s="11" t="inlineStr">
         <is>
           <t>comp_fc_forn2</t>
         </is>
       </c>
-      <c r="BL1" s="10" t="inlineStr">
+      <c r="BL1" s="11" t="inlineStr">
         <is>
           <t>moeda_forn2</t>
         </is>
@@ -861,23 +866,28 @@
       <c r="BO1" s="1" t="inlineStr">
         <is>
           <t>observacao</t>
+        </is>
+      </c>
+      <c r="BP1" s="1" t="inlineStr">
+        <is>
+          <t>cross_selling_decision</t>
         </is>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>C001</t>
+          <t>C015</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Paulo Negrão</t>
+          <t>André Camargo</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Diretor</t>
+          <t>Consultor Externo</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -909,121 +919,95 @@
         <v>30</v>
       </c>
       <c r="L2" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="M2" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="N2" s="11" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="O2" s="12" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="P2" s="12" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q2" s="12" t="n">
-        <v>100</v>
-      </c>
-      <c r="R2" s="12" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="S2" s="12" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="T2" s="12" t="n">
-        <v>0.3200000000000001</v>
-      </c>
-      <c r="U2" s="13" t="n">
+        <v>1</v>
+      </c>
+      <c r="N2" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="O2" s="13" t="inlineStr"/>
+      <c r="P2" s="13" t="inlineStr"/>
+      <c r="Q2" s="13" t="inlineStr"/>
+      <c r="R2" s="13" t="inlineStr"/>
+      <c r="S2" s="13" t="inlineStr"/>
+      <c r="T2" s="13" t="inlineStr"/>
+      <c r="U2" s="14" t="inlineStr"/>
+      <c r="V2" s="14" t="inlineStr"/>
+      <c r="W2" s="14" t="inlineStr"/>
+      <c r="X2" s="14" t="inlineStr"/>
+      <c r="Y2" s="14" t="inlineStr"/>
+      <c r="Z2" s="14" t="inlineStr"/>
+      <c r="AA2" s="15" t="inlineStr"/>
+      <c r="AB2" s="15" t="inlineStr"/>
+      <c r="AC2" s="15" t="inlineStr"/>
+      <c r="AD2" s="15" t="inlineStr"/>
+      <c r="AE2" s="15" t="inlineStr"/>
+      <c r="AF2" s="15" t="inlineStr"/>
+      <c r="AG2" s="16" t="inlineStr"/>
+      <c r="AH2" s="16" t="inlineStr"/>
+      <c r="AI2" s="16" t="inlineStr"/>
+      <c r="AJ2" s="16" t="inlineStr"/>
+      <c r="AK2" s="16" t="inlineStr"/>
+      <c r="AL2" s="16" t="inlineStr"/>
+      <c r="AM2" s="17" t="inlineStr"/>
+      <c r="AN2" s="17" t="inlineStr"/>
+      <c r="AO2" s="17" t="inlineStr"/>
+      <c r="AP2" s="17" t="inlineStr"/>
+      <c r="AQ2" s="17" t="inlineStr"/>
+      <c r="AR2" s="17" t="inlineStr"/>
+      <c r="AS2" s="18" t="inlineStr"/>
+      <c r="AT2" s="18" t="inlineStr"/>
+      <c r="AU2" s="18" t="inlineStr"/>
+      <c r="AV2" s="18" t="inlineStr"/>
+      <c r="AW2" s="18" t="inlineStr"/>
+      <c r="AX2" s="18" t="inlineStr"/>
+      <c r="AY2" s="19" t="inlineStr"/>
+      <c r="AZ2" s="19" t="inlineStr"/>
+      <c r="BA2" s="19" t="inlineStr"/>
+      <c r="BB2" s="19" t="inlineStr"/>
+      <c r="BC2" s="19" t="inlineStr"/>
+      <c r="BD2" s="19" t="inlineStr"/>
+      <c r="BE2" s="19" t="inlineStr"/>
+      <c r="BF2" s="20" t="inlineStr"/>
+      <c r="BG2" s="20" t="inlineStr"/>
+      <c r="BH2" s="20" t="inlineStr"/>
+      <c r="BI2" s="20" t="inlineStr"/>
+      <c r="BJ2" s="20" t="inlineStr"/>
+      <c r="BK2" s="20" t="inlineStr"/>
+      <c r="BL2" s="20" t="inlineStr"/>
+      <c r="BM2" t="n">
         <v>0.3</v>
       </c>
-      <c r="V2" s="13" t="n">
-        <v>30</v>
-      </c>
-      <c r="W2" s="13" t="n">
-        <v>100</v>
-      </c>
-      <c r="X2" s="13" t="n">
+      <c r="BN2" t="n">
         <v>0.3</v>
       </c>
-      <c r="Y2" s="13" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="Z2" s="13" t="n">
-        <v>0.09</v>
-      </c>
-      <c r="AA2" s="14" t="inlineStr"/>
-      <c r="AB2" s="14" t="inlineStr"/>
-      <c r="AC2" s="14" t="inlineStr"/>
-      <c r="AD2" s="14" t="inlineStr"/>
-      <c r="AE2" s="14" t="inlineStr"/>
-      <c r="AF2" s="14" t="inlineStr"/>
-      <c r="AG2" s="15" t="inlineStr"/>
-      <c r="AH2" s="15" t="inlineStr"/>
-      <c r="AI2" s="15" t="inlineStr"/>
-      <c r="AJ2" s="15" t="inlineStr"/>
-      <c r="AK2" s="15" t="inlineStr"/>
-      <c r="AL2" s="15" t="inlineStr"/>
-      <c r="AM2" s="16" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="AN2" s="16" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="AO2" s="16" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AP2" s="16" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AQ2" s="16" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AR2" s="16" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="AS2" s="17" t="inlineStr"/>
-      <c r="AT2" s="17" t="inlineStr"/>
-      <c r="AU2" s="17" t="inlineStr"/>
-      <c r="AV2" s="17" t="inlineStr"/>
-      <c r="AW2" s="17" t="inlineStr"/>
-      <c r="AX2" s="17" t="inlineStr"/>
-      <c r="AY2" s="18" t="inlineStr"/>
-      <c r="AZ2" s="18" t="inlineStr"/>
-      <c r="BA2" s="18" t="inlineStr"/>
-      <c r="BB2" s="18" t="inlineStr"/>
-      <c r="BC2" s="18" t="inlineStr"/>
-      <c r="BD2" s="18" t="inlineStr"/>
-      <c r="BE2" s="18" t="inlineStr"/>
-      <c r="BF2" s="19" t="inlineStr"/>
-      <c r="BG2" s="19" t="inlineStr"/>
-      <c r="BH2" s="19" t="inlineStr"/>
-      <c r="BI2" s="19" t="inlineStr"/>
-      <c r="BJ2" s="19" t="inlineStr"/>
-      <c r="BK2" s="19" t="inlineStr"/>
-      <c r="BL2" s="19" t="inlineStr"/>
-      <c r="BM2" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="BN2" t="n">
-        <v>0.09750000000000002</v>
+      <c r="BO2" t="inlineStr">
+        <is>
+          <t>CROSS_SELLING</t>
+        </is>
+      </c>
+      <c r="BP2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>C002</t>
+          <t>C001</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Antônio Rosa</t>
+          <t>Paulo Negrão</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Gerente Geral</t>
+          <t>Diretor</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -1058,118 +1042,123 @@
         <v>0.05</v>
       </c>
       <c r="M3" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="N3" s="11" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="O3" s="12" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="N3" s="12" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="O3" s="13" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="P3" s="13" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q3" s="13" t="n">
+        <v>100</v>
+      </c>
+      <c r="R3" s="13" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="S3" s="13" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="T3" s="13" t="n">
+        <v>0.3200000000000001</v>
+      </c>
+      <c r="U3" s="14" t="n">
         <v>0.3</v>
       </c>
-      <c r="P3" s="12" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q3" s="12" t="n">
+      <c r="V3" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="W3" s="14" t="n">
         <v>100</v>
       </c>
-      <c r="R3" s="12" t="n">
+      <c r="X3" s="14" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Y3" s="14" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Z3" s="14" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="AA3" s="15" t="inlineStr"/>
+      <c r="AB3" s="15" t="inlineStr"/>
+      <c r="AC3" s="15" t="inlineStr"/>
+      <c r="AD3" s="15" t="inlineStr"/>
+      <c r="AE3" s="15" t="inlineStr"/>
+      <c r="AF3" s="15" t="inlineStr"/>
+      <c r="AG3" s="16" t="inlineStr"/>
+      <c r="AH3" s="16" t="inlineStr"/>
+      <c r="AI3" s="16" t="inlineStr"/>
+      <c r="AJ3" s="16" t="inlineStr"/>
+      <c r="AK3" s="16" t="inlineStr"/>
+      <c r="AL3" s="16" t="inlineStr"/>
+      <c r="AM3" s="17" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="AN3" s="17" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="AO3" s="17" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AP3" s="17" t="n">
         <v>0.8</v>
       </c>
-      <c r="S3" s="12" t="n">
+      <c r="AQ3" s="17" t="n">
         <v>0.8</v>
       </c>
-      <c r="T3" s="12" t="n">
+      <c r="AR3" s="17" t="n">
         <v>0.24</v>
       </c>
-      <c r="U3" s="13" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="V3" s="13" t="n">
-        <v>30</v>
-      </c>
-      <c r="W3" s="13" t="n">
-        <v>100</v>
-      </c>
-      <c r="X3" s="13" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="Y3" s="13" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="Z3" s="13" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="AA3" s="14" t="inlineStr"/>
-      <c r="AB3" s="14" t="inlineStr"/>
-      <c r="AC3" s="14" t="inlineStr"/>
-      <c r="AD3" s="14" t="inlineStr"/>
-      <c r="AE3" s="14" t="inlineStr"/>
-      <c r="AF3" s="14" t="inlineStr"/>
-      <c r="AG3" s="15" t="inlineStr"/>
-      <c r="AH3" s="15" t="inlineStr"/>
-      <c r="AI3" s="15" t="inlineStr"/>
-      <c r="AJ3" s="15" t="inlineStr"/>
-      <c r="AK3" s="15" t="inlineStr"/>
-      <c r="AL3" s="15" t="inlineStr"/>
-      <c r="AM3" s="16" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="AN3" s="16" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="AO3" s="16" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AP3" s="16" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AQ3" s="16" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AR3" s="16" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="AS3" s="17" t="inlineStr"/>
-      <c r="AT3" s="17" t="inlineStr"/>
-      <c r="AU3" s="17" t="inlineStr"/>
-      <c r="AV3" s="17" t="inlineStr"/>
-      <c r="AW3" s="17" t="inlineStr"/>
-      <c r="AX3" s="17" t="inlineStr"/>
-      <c r="AY3" s="18" t="inlineStr"/>
-      <c r="AZ3" s="18" t="inlineStr"/>
-      <c r="BA3" s="18" t="inlineStr"/>
-      <c r="BB3" s="18" t="inlineStr"/>
-      <c r="BC3" s="18" t="inlineStr"/>
-      <c r="BD3" s="18" t="inlineStr"/>
-      <c r="BE3" s="18" t="inlineStr"/>
-      <c r="BF3" s="19" t="inlineStr"/>
-      <c r="BG3" s="19" t="inlineStr"/>
-      <c r="BH3" s="19" t="inlineStr"/>
-      <c r="BI3" s="19" t="inlineStr"/>
-      <c r="BJ3" s="19" t="inlineStr"/>
-      <c r="BK3" s="19" t="inlineStr"/>
-      <c r="BL3" s="19" t="inlineStr"/>
+      <c r="AS3" s="18" t="inlineStr"/>
+      <c r="AT3" s="18" t="inlineStr"/>
+      <c r="AU3" s="18" t="inlineStr"/>
+      <c r="AV3" s="18" t="inlineStr"/>
+      <c r="AW3" s="18" t="inlineStr"/>
+      <c r="AX3" s="18" t="inlineStr"/>
+      <c r="AY3" s="19" t="inlineStr"/>
+      <c r="AZ3" s="19" t="inlineStr"/>
+      <c r="BA3" s="19" t="inlineStr"/>
+      <c r="BB3" s="19" t="inlineStr"/>
+      <c r="BC3" s="19" t="inlineStr"/>
+      <c r="BD3" s="19" t="inlineStr"/>
+      <c r="BE3" s="19" t="inlineStr"/>
+      <c r="BF3" s="20" t="inlineStr"/>
+      <c r="BG3" s="20" t="inlineStr"/>
+      <c r="BH3" s="20" t="inlineStr"/>
+      <c r="BI3" s="20" t="inlineStr"/>
+      <c r="BJ3" s="20" t="inlineStr"/>
+      <c r="BK3" s="20" t="inlineStr"/>
+      <c r="BL3" s="20" t="inlineStr"/>
       <c r="BM3" t="n">
-        <v>0.3</v>
+        <v>0.15</v>
       </c>
       <c r="BN3" t="n">
-        <v>0.18</v>
+        <v>0.09750000000000002</v>
+      </c>
+      <c r="BP3" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>C007</t>
+          <t>C002</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Simone</t>
+          <t>Antônio Rosa</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Coordenador</t>
+          <t>Gerente Geral</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1206,116 +1195,121 @@
       <c r="M4" t="n">
         <v>0.2</v>
       </c>
-      <c r="N4" s="11" t="n">
-        <v>0.6000000000000001</v>
-      </c>
-      <c r="O4" s="12" t="n">
+      <c r="N4" s="12" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="O4" s="13" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="P4" s="13" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q4" s="13" t="n">
+        <v>100</v>
+      </c>
+      <c r="R4" s="13" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="S4" s="13" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="T4" s="13" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="U4" s="14" t="n">
         <v>0.4</v>
       </c>
-      <c r="P4" s="12" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q4" s="12" t="n">
+      <c r="V4" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="W4" s="14" t="n">
         <v>100</v>
       </c>
-      <c r="R4" s="12" t="n">
+      <c r="X4" s="14" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Y4" s="14" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Z4" s="14" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="AA4" s="15" t="inlineStr"/>
+      <c r="AB4" s="15" t="inlineStr"/>
+      <c r="AC4" s="15" t="inlineStr"/>
+      <c r="AD4" s="15" t="inlineStr"/>
+      <c r="AE4" s="15" t="inlineStr"/>
+      <c r="AF4" s="15" t="inlineStr"/>
+      <c r="AG4" s="16" t="inlineStr"/>
+      <c r="AH4" s="16" t="inlineStr"/>
+      <c r="AI4" s="16" t="inlineStr"/>
+      <c r="AJ4" s="16" t="inlineStr"/>
+      <c r="AK4" s="16" t="inlineStr"/>
+      <c r="AL4" s="16" t="inlineStr"/>
+      <c r="AM4" s="17" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="AN4" s="17" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="AO4" s="17" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AP4" s="17" t="n">
         <v>0.8</v>
       </c>
-      <c r="S4" s="12" t="n">
+      <c r="AQ4" s="17" t="n">
         <v>0.8</v>
       </c>
-      <c r="T4" s="12" t="n">
-        <v>0.3200000000000001</v>
-      </c>
-      <c r="U4" s="13" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="V4" s="13" t="n">
-        <v>30</v>
-      </c>
-      <c r="W4" s="13" t="n">
-        <v>100</v>
-      </c>
-      <c r="X4" s="13" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="Y4" s="13" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="Z4" s="13" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="AA4" s="14" t="inlineStr"/>
-      <c r="AB4" s="14" t="inlineStr"/>
-      <c r="AC4" s="14" t="inlineStr"/>
-      <c r="AD4" s="14" t="inlineStr"/>
-      <c r="AE4" s="14" t="inlineStr"/>
-      <c r="AF4" s="14" t="inlineStr"/>
-      <c r="AG4" s="15" t="inlineStr"/>
-      <c r="AH4" s="15" t="inlineStr"/>
-      <c r="AI4" s="15" t="inlineStr"/>
-      <c r="AJ4" s="15" t="inlineStr"/>
-      <c r="AK4" s="15" t="inlineStr"/>
-      <c r="AL4" s="15" t="inlineStr"/>
-      <c r="AM4" s="16" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="AN4" s="16" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="AO4" s="16" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AP4" s="16" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AQ4" s="16" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AR4" s="16" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="AS4" s="17" t="inlineStr"/>
-      <c r="AT4" s="17" t="inlineStr"/>
-      <c r="AU4" s="17" t="inlineStr"/>
-      <c r="AV4" s="17" t="inlineStr"/>
-      <c r="AW4" s="17" t="inlineStr"/>
-      <c r="AX4" s="17" t="inlineStr"/>
-      <c r="AY4" s="18" t="inlineStr"/>
-      <c r="AZ4" s="18" t="inlineStr"/>
-      <c r="BA4" s="18" t="inlineStr"/>
-      <c r="BB4" s="18" t="inlineStr"/>
-      <c r="BC4" s="18" t="inlineStr"/>
-      <c r="BD4" s="18" t="inlineStr"/>
-      <c r="BE4" s="18" t="inlineStr"/>
-      <c r="BF4" s="19" t="inlineStr"/>
-      <c r="BG4" s="19" t="inlineStr"/>
-      <c r="BH4" s="19" t="inlineStr"/>
-      <c r="BI4" s="19" t="inlineStr"/>
-      <c r="BJ4" s="19" t="inlineStr"/>
-      <c r="BK4" s="19" t="inlineStr"/>
-      <c r="BL4" s="19" t="inlineStr"/>
+      <c r="AR4" s="17" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="AS4" s="18" t="inlineStr"/>
+      <c r="AT4" s="18" t="inlineStr"/>
+      <c r="AU4" s="18" t="inlineStr"/>
+      <c r="AV4" s="18" t="inlineStr"/>
+      <c r="AW4" s="18" t="inlineStr"/>
+      <c r="AX4" s="18" t="inlineStr"/>
+      <c r="AY4" s="19" t="inlineStr"/>
+      <c r="AZ4" s="19" t="inlineStr"/>
+      <c r="BA4" s="19" t="inlineStr"/>
+      <c r="BB4" s="19" t="inlineStr"/>
+      <c r="BC4" s="19" t="inlineStr"/>
+      <c r="BD4" s="19" t="inlineStr"/>
+      <c r="BE4" s="19" t="inlineStr"/>
+      <c r="BF4" s="20" t="inlineStr"/>
+      <c r="BG4" s="20" t="inlineStr"/>
+      <c r="BH4" s="20" t="inlineStr"/>
+      <c r="BI4" s="20" t="inlineStr"/>
+      <c r="BJ4" s="20" t="inlineStr"/>
+      <c r="BK4" s="20" t="inlineStr"/>
+      <c r="BL4" s="20" t="inlineStr"/>
       <c r="BM4" t="n">
         <v>0.3</v>
       </c>
       <c r="BN4" t="n">
         <v>0.18</v>
       </c>
+      <c r="BP4" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>C010</t>
+          <t>C007</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Samanta</t>
+          <t>Simone</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Consultor Interno</t>
+          <t>Coordenador</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
@@ -1350,106 +1344,123 @@
         <v>0.05</v>
       </c>
       <c r="M5" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="N5" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="N5" s="12" t="n">
+        <v>0.6000000000000001</v>
+      </c>
+      <c r="O5" s="13" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="P5" s="13" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q5" s="13" t="n">
+        <v>100</v>
+      </c>
+      <c r="R5" s="13" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="S5" s="13" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="T5" s="13" t="n">
+        <v>0.3200000000000001</v>
+      </c>
+      <c r="U5" s="14" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="V5" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="W5" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="X5" s="14" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Y5" s="14" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Z5" s="14" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="AA5" s="15" t="inlineStr"/>
+      <c r="AB5" s="15" t="inlineStr"/>
+      <c r="AC5" s="15" t="inlineStr"/>
+      <c r="AD5" s="15" t="inlineStr"/>
+      <c r="AE5" s="15" t="inlineStr"/>
+      <c r="AF5" s="15" t="inlineStr"/>
+      <c r="AG5" s="16" t="inlineStr"/>
+      <c r="AH5" s="16" t="inlineStr"/>
+      <c r="AI5" s="16" t="inlineStr"/>
+      <c r="AJ5" s="16" t="inlineStr"/>
+      <c r="AK5" s="16" t="inlineStr"/>
+      <c r="AL5" s="16" t="inlineStr"/>
+      <c r="AM5" s="17" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="AN5" s="17" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="AO5" s="17" t="n">
         <v>0.5</v>
       </c>
-      <c r="O5" s="12" t="inlineStr"/>
-      <c r="P5" s="12" t="inlineStr"/>
-      <c r="Q5" s="12" t="inlineStr"/>
-      <c r="R5" s="12" t="inlineStr"/>
-      <c r="S5" s="12" t="inlineStr"/>
-      <c r="T5" s="12" t="inlineStr"/>
-      <c r="U5" s="13" t="inlineStr"/>
-      <c r="V5" s="13" t="inlineStr"/>
-      <c r="W5" s="13" t="inlineStr"/>
-      <c r="X5" s="13" t="inlineStr"/>
-      <c r="Y5" s="13" t="inlineStr"/>
-      <c r="Z5" s="13" t="inlineStr"/>
-      <c r="AA5" s="14" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="AB5" s="14" t="n">
-        <v>80</v>
-      </c>
-      <c r="AC5" s="14" t="n">
-        <v>100</v>
-      </c>
-      <c r="AD5" s="14" t="n">
+      <c r="AP5" s="17" t="n">
         <v>0.8</v>
       </c>
-      <c r="AE5" s="14" t="n">
+      <c r="AQ5" s="17" t="n">
         <v>0.8</v>
       </c>
-      <c r="AF5" s="14" t="n">
-        <v>0.3200000000000001</v>
-      </c>
-      <c r="AG5" s="15" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="AH5" s="15" t="n">
-        <v>30</v>
-      </c>
-      <c r="AI5" s="15" t="n">
-        <v>100</v>
-      </c>
-      <c r="AJ5" s="15" t="n">
+      <c r="AR5" s="17" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="AS5" s="18" t="inlineStr"/>
+      <c r="AT5" s="18" t="inlineStr"/>
+      <c r="AU5" s="18" t="inlineStr"/>
+      <c r="AV5" s="18" t="inlineStr"/>
+      <c r="AW5" s="18" t="inlineStr"/>
+      <c r="AX5" s="18" t="inlineStr"/>
+      <c r="AY5" s="19" t="inlineStr"/>
+      <c r="AZ5" s="19" t="inlineStr"/>
+      <c r="BA5" s="19" t="inlineStr"/>
+      <c r="BB5" s="19" t="inlineStr"/>
+      <c r="BC5" s="19" t="inlineStr"/>
+      <c r="BD5" s="19" t="inlineStr"/>
+      <c r="BE5" s="19" t="inlineStr"/>
+      <c r="BF5" s="20" t="inlineStr"/>
+      <c r="BG5" s="20" t="inlineStr"/>
+      <c r="BH5" s="20" t="inlineStr"/>
+      <c r="BI5" s="20" t="inlineStr"/>
+      <c r="BJ5" s="20" t="inlineStr"/>
+      <c r="BK5" s="20" t="inlineStr"/>
+      <c r="BL5" s="20" t="inlineStr"/>
+      <c r="BM5" t="n">
         <v>0.3</v>
       </c>
-      <c r="AK5" s="15" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="AL5" s="15" t="n">
+      <c r="BN5" t="n">
         <v>0.18</v>
       </c>
-      <c r="AM5" s="16" t="inlineStr"/>
-      <c r="AN5" s="16" t="inlineStr"/>
-      <c r="AO5" s="16" t="inlineStr"/>
-      <c r="AP5" s="16" t="inlineStr"/>
-      <c r="AQ5" s="16" t="inlineStr"/>
-      <c r="AR5" s="16" t="inlineStr"/>
-      <c r="AS5" s="17" t="inlineStr"/>
-      <c r="AT5" s="17" t="inlineStr"/>
-      <c r="AU5" s="17" t="inlineStr"/>
-      <c r="AV5" s="17" t="inlineStr"/>
-      <c r="AW5" s="17" t="inlineStr"/>
-      <c r="AX5" s="17" t="inlineStr"/>
-      <c r="AY5" s="18" t="inlineStr"/>
-      <c r="AZ5" s="18" t="inlineStr"/>
-      <c r="BA5" s="18" t="inlineStr"/>
-      <c r="BB5" s="18" t="inlineStr"/>
-      <c r="BC5" s="18" t="inlineStr"/>
-      <c r="BD5" s="18" t="inlineStr"/>
-      <c r="BE5" s="18" t="inlineStr"/>
-      <c r="BF5" s="19" t="inlineStr"/>
-      <c r="BG5" s="19" t="inlineStr"/>
-      <c r="BH5" s="19" t="inlineStr"/>
-      <c r="BI5" s="19" t="inlineStr"/>
-      <c r="BJ5" s="19" t="inlineStr"/>
-      <c r="BK5" s="19" t="inlineStr"/>
-      <c r="BL5" s="19" t="inlineStr"/>
-      <c r="BM5" t="n">
-        <v>0.225</v>
-      </c>
-      <c r="BN5" t="n">
-        <v>0.1125</v>
+      <c r="BP5" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>C020</t>
+          <t>C010</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Mateus Machado</t>
+          <t>Samanta</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Consultor Externo</t>
+          <t>Consultor Interno</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1486,100 +1497,109 @@
       <c r="M6" t="n">
         <v>0.15</v>
       </c>
-      <c r="N6" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="O6" s="12" t="inlineStr"/>
-      <c r="P6" s="12" t="inlineStr"/>
-      <c r="Q6" s="12" t="inlineStr"/>
-      <c r="R6" s="12" t="inlineStr"/>
-      <c r="S6" s="12" t="inlineStr"/>
-      <c r="T6" s="12" t="inlineStr"/>
-      <c r="U6" s="13" t="inlineStr"/>
-      <c r="V6" s="13" t="inlineStr"/>
-      <c r="W6" s="13" t="inlineStr"/>
-      <c r="X6" s="13" t="inlineStr"/>
-      <c r="Y6" s="13" t="inlineStr"/>
-      <c r="Z6" s="13" t="inlineStr"/>
-      <c r="AA6" s="14" t="n">
+      <c r="N6" s="12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="O6" s="13" t="inlineStr"/>
+      <c r="P6" s="13" t="inlineStr"/>
+      <c r="Q6" s="13" t="inlineStr"/>
+      <c r="R6" s="13" t="inlineStr"/>
+      <c r="S6" s="13" t="inlineStr"/>
+      <c r="T6" s="13" t="inlineStr"/>
+      <c r="U6" s="14" t="inlineStr"/>
+      <c r="V6" s="14" t="inlineStr"/>
+      <c r="W6" s="14" t="inlineStr"/>
+      <c r="X6" s="14" t="inlineStr"/>
+      <c r="Y6" s="14" t="inlineStr"/>
+      <c r="Z6" s="14" t="inlineStr"/>
+      <c r="AA6" s="15" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="AB6" s="15" t="n">
+        <v>80</v>
+      </c>
+      <c r="AC6" s="15" t="n">
+        <v>100</v>
+      </c>
+      <c r="AD6" s="15" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AE6" s="15" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AF6" s="15" t="n">
+        <v>0.3200000000000001</v>
+      </c>
+      <c r="AG6" s="16" t="n">
         <v>0.6</v>
       </c>
-      <c r="AB6" s="14" t="n">
-        <v>80</v>
-      </c>
-      <c r="AC6" s="14" t="inlineStr"/>
-      <c r="AD6" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE6" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF6" s="14" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="AG6" s="15" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="AH6" s="15" t="n">
+      <c r="AH6" s="16" t="n">
         <v>30</v>
       </c>
-      <c r="AI6" s="15" t="inlineStr"/>
-      <c r="AJ6" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK6" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL6" s="15" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="AM6" s="16" t="inlineStr"/>
-      <c r="AN6" s="16" t="inlineStr"/>
-      <c r="AO6" s="16" t="inlineStr"/>
-      <c r="AP6" s="16" t="inlineStr"/>
-      <c r="AQ6" s="16" t="inlineStr"/>
-      <c r="AR6" s="16" t="inlineStr"/>
-      <c r="AS6" s="17" t="inlineStr"/>
-      <c r="AT6" s="17" t="inlineStr"/>
-      <c r="AU6" s="17" t="inlineStr"/>
-      <c r="AV6" s="17" t="inlineStr"/>
-      <c r="AW6" s="17" t="inlineStr"/>
-      <c r="AX6" s="17" t="inlineStr"/>
-      <c r="AY6" s="18" t="inlineStr"/>
-      <c r="AZ6" s="18" t="inlineStr"/>
-      <c r="BA6" s="18" t="inlineStr"/>
-      <c r="BB6" s="18" t="inlineStr"/>
-      <c r="BC6" s="18" t="inlineStr"/>
-      <c r="BD6" s="18" t="inlineStr"/>
-      <c r="BE6" s="18" t="inlineStr"/>
-      <c r="BF6" s="19" t="inlineStr"/>
-      <c r="BG6" s="19" t="inlineStr"/>
-      <c r="BH6" s="19" t="inlineStr"/>
-      <c r="BI6" s="19" t="inlineStr"/>
-      <c r="BJ6" s="19" t="inlineStr"/>
-      <c r="BK6" s="19" t="inlineStr"/>
-      <c r="BL6" s="19" t="inlineStr"/>
+      <c r="AI6" s="16" t="n">
+        <v>100</v>
+      </c>
+      <c r="AJ6" s="16" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="AK6" s="16" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="AL6" s="16" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="AM6" s="17" t="inlineStr"/>
+      <c r="AN6" s="17" t="inlineStr"/>
+      <c r="AO6" s="17" t="inlineStr"/>
+      <c r="AP6" s="17" t="inlineStr"/>
+      <c r="AQ6" s="17" t="inlineStr"/>
+      <c r="AR6" s="17" t="inlineStr"/>
+      <c r="AS6" s="18" t="inlineStr"/>
+      <c r="AT6" s="18" t="inlineStr"/>
+      <c r="AU6" s="18" t="inlineStr"/>
+      <c r="AV6" s="18" t="inlineStr"/>
+      <c r="AW6" s="18" t="inlineStr"/>
+      <c r="AX6" s="18" t="inlineStr"/>
+      <c r="AY6" s="19" t="inlineStr"/>
+      <c r="AZ6" s="19" t="inlineStr"/>
+      <c r="BA6" s="19" t="inlineStr"/>
+      <c r="BB6" s="19" t="inlineStr"/>
+      <c r="BC6" s="19" t="inlineStr"/>
+      <c r="BD6" s="19" t="inlineStr"/>
+      <c r="BE6" s="19" t="inlineStr"/>
+      <c r="BF6" s="20" t="inlineStr"/>
+      <c r="BG6" s="20" t="inlineStr"/>
+      <c r="BH6" s="20" t="inlineStr"/>
+      <c r="BI6" s="20" t="inlineStr"/>
+      <c r="BJ6" s="20" t="inlineStr"/>
+      <c r="BK6" s="20" t="inlineStr"/>
+      <c r="BL6" s="20" t="inlineStr"/>
       <c r="BM6" t="n">
         <v>0.225</v>
       </c>
       <c r="BN6" t="n">
-        <v>0.225</v>
+        <v>0.1125</v>
+      </c>
+      <c r="BP6" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>C001</t>
+          <t>C020</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Paulo Negrão</t>
+          <t>Mateus Machado</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Diretor</t>
+          <t>Consultor Externo</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1594,12 +1614,12 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>Medidor de Vazão Fixo</t>
+          <t>Sonda Serie EXO</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>IQ Standard</t>
+          <t>EXO</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -1608,124 +1628,113 @@
         </is>
       </c>
       <c r="K7" t="n">
-        <v>20</v>
+        <v>30</v>
       </c>
       <c r="L7" t="n">
         <v>0.05</v>
       </c>
       <c r="M7" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="N7" s="11" t="n">
-        <v>0.5900000000000001</v>
-      </c>
-      <c r="O7" s="12" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="N7" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="O7" s="13" t="inlineStr"/>
+      <c r="P7" s="13" t="inlineStr"/>
+      <c r="Q7" s="13" t="inlineStr"/>
+      <c r="R7" s="13" t="inlineStr"/>
+      <c r="S7" s="13" t="inlineStr"/>
+      <c r="T7" s="13" t="inlineStr"/>
+      <c r="U7" s="14" t="inlineStr"/>
+      <c r="V7" s="14" t="inlineStr"/>
+      <c r="W7" s="14" t="inlineStr"/>
+      <c r="X7" s="14" t="inlineStr"/>
+      <c r="Y7" s="14" t="inlineStr"/>
+      <c r="Z7" s="14" t="inlineStr"/>
+      <c r="AA7" s="15" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="AB7" s="15" t="n">
+        <v>80</v>
+      </c>
+      <c r="AC7" s="15" t="inlineStr"/>
+      <c r="AD7" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE7" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF7" s="15" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="AG7" s="16" t="n">
         <v>0.4</v>
       </c>
-      <c r="P7" s="12" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q7" s="12" t="n">
-        <v>100</v>
-      </c>
-      <c r="R7" s="12" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="S7" s="12" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="T7" s="12" t="n">
-        <v>0.3200000000000001</v>
-      </c>
-      <c r="U7" s="13" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="V7" s="13" t="n">
+      <c r="AH7" s="16" t="n">
         <v>30</v>
       </c>
-      <c r="W7" s="13" t="n">
-        <v>100</v>
-      </c>
-      <c r="X7" s="13" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="Y7" s="13" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="Z7" s="13" t="n">
-        <v>0.09</v>
-      </c>
-      <c r="AA7" s="14" t="inlineStr"/>
-      <c r="AB7" s="14" t="inlineStr"/>
-      <c r="AC7" s="14" t="inlineStr"/>
-      <c r="AD7" s="14" t="inlineStr"/>
-      <c r="AE7" s="14" t="inlineStr"/>
-      <c r="AF7" s="14" t="inlineStr"/>
-      <c r="AG7" s="15" t="inlineStr"/>
-      <c r="AH7" s="15" t="inlineStr"/>
-      <c r="AI7" s="15" t="inlineStr"/>
-      <c r="AJ7" s="15" t="inlineStr"/>
-      <c r="AK7" s="15" t="inlineStr"/>
-      <c r="AL7" s="15" t="inlineStr"/>
-      <c r="AM7" s="16" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="AN7" s="16" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="AO7" s="16" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AP7" s="16" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="AQ7" s="16" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="AR7" s="16" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="AS7" s="17" t="inlineStr"/>
-      <c r="AT7" s="17" t="inlineStr"/>
-      <c r="AU7" s="17" t="inlineStr"/>
-      <c r="AV7" s="17" t="inlineStr"/>
-      <c r="AW7" s="17" t="inlineStr"/>
-      <c r="AX7" s="17" t="inlineStr"/>
-      <c r="AY7" s="18" t="inlineStr"/>
-      <c r="AZ7" s="18" t="inlineStr"/>
-      <c r="BA7" s="18" t="inlineStr"/>
-      <c r="BB7" s="18" t="inlineStr"/>
-      <c r="BC7" s="18" t="inlineStr"/>
-      <c r="BD7" s="18" t="inlineStr"/>
-      <c r="BE7" s="18" t="inlineStr"/>
-      <c r="BF7" s="19" t="inlineStr"/>
-      <c r="BG7" s="19" t="inlineStr"/>
-      <c r="BH7" s="19" t="inlineStr"/>
-      <c r="BI7" s="19" t="inlineStr"/>
-      <c r="BJ7" s="19" t="inlineStr"/>
-      <c r="BK7" s="19" t="inlineStr"/>
-      <c r="BL7" s="19" t="inlineStr"/>
+      <c r="AI7" s="16" t="inlineStr"/>
+      <c r="AJ7" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK7" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL7" s="16" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="AM7" s="17" t="inlineStr"/>
+      <c r="AN7" s="17" t="inlineStr"/>
+      <c r="AO7" s="17" t="inlineStr"/>
+      <c r="AP7" s="17" t="inlineStr"/>
+      <c r="AQ7" s="17" t="inlineStr"/>
+      <c r="AR7" s="17" t="inlineStr"/>
+      <c r="AS7" s="18" t="inlineStr"/>
+      <c r="AT7" s="18" t="inlineStr"/>
+      <c r="AU7" s="18" t="inlineStr"/>
+      <c r="AV7" s="18" t="inlineStr"/>
+      <c r="AW7" s="18" t="inlineStr"/>
+      <c r="AX7" s="18" t="inlineStr"/>
+      <c r="AY7" s="19" t="inlineStr"/>
+      <c r="AZ7" s="19" t="inlineStr"/>
+      <c r="BA7" s="19" t="inlineStr"/>
+      <c r="BB7" s="19" t="inlineStr"/>
+      <c r="BC7" s="19" t="inlineStr"/>
+      <c r="BD7" s="19" t="inlineStr"/>
+      <c r="BE7" s="19" t="inlineStr"/>
+      <c r="BF7" s="20" t="inlineStr"/>
+      <c r="BG7" s="20" t="inlineStr"/>
+      <c r="BH7" s="20" t="inlineStr"/>
+      <c r="BI7" s="20" t="inlineStr"/>
+      <c r="BJ7" s="20" t="inlineStr"/>
+      <c r="BK7" s="20" t="inlineStr"/>
+      <c r="BL7" s="20" t="inlineStr"/>
       <c r="BM7" t="n">
-        <v>0.1</v>
+        <v>0.225</v>
       </c>
       <c r="BN7" t="n">
-        <v>0.05900000000000001</v>
+        <v>0.225</v>
+      </c>
+      <c r="BP7" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>C002</t>
+          <t>C015</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Antônio Rosa</t>
+          <t>André Camargo</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Gerente Geral</t>
+          <t>Consultor Externo</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1757,121 +1766,95 @@
         <v>20</v>
       </c>
       <c r="L8" t="n">
-        <v>0.05</v>
+        <v>0.01</v>
       </c>
       <c r="M8" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="N8" s="11" t="n">
-        <v>0.54</v>
-      </c>
-      <c r="O8" s="12" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="P8" s="12" t="n">
-        <v>80</v>
-      </c>
-      <c r="Q8" s="12" t="n">
-        <v>100</v>
-      </c>
-      <c r="R8" s="12" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="S8" s="12" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="T8" s="12" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="U8" s="13" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="V8" s="13" t="n">
-        <v>30</v>
-      </c>
-      <c r="W8" s="13" t="n">
-        <v>100</v>
-      </c>
-      <c r="X8" s="13" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="Y8" s="13" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="Z8" s="13" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="AA8" s="14" t="inlineStr"/>
-      <c r="AB8" s="14" t="inlineStr"/>
-      <c r="AC8" s="14" t="inlineStr"/>
-      <c r="AD8" s="14" t="inlineStr"/>
-      <c r="AE8" s="14" t="inlineStr"/>
-      <c r="AF8" s="14" t="inlineStr"/>
-      <c r="AG8" s="15" t="inlineStr"/>
-      <c r="AH8" s="15" t="inlineStr"/>
-      <c r="AI8" s="15" t="inlineStr"/>
-      <c r="AJ8" s="15" t="inlineStr"/>
-      <c r="AK8" s="15" t="inlineStr"/>
-      <c r="AL8" s="15" t="inlineStr"/>
-      <c r="AM8" s="16" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="AN8" s="16" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="AO8" s="16" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AP8" s="16" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="AQ8" s="16" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="AR8" s="16" t="n">
-        <v>0.18</v>
-      </c>
-      <c r="AS8" s="17" t="inlineStr"/>
-      <c r="AT8" s="17" t="inlineStr"/>
-      <c r="AU8" s="17" t="inlineStr"/>
-      <c r="AV8" s="17" t="inlineStr"/>
-      <c r="AW8" s="17" t="inlineStr"/>
-      <c r="AX8" s="17" t="inlineStr"/>
-      <c r="AY8" s="18" t="inlineStr"/>
-      <c r="AZ8" s="18" t="inlineStr"/>
-      <c r="BA8" s="18" t="inlineStr"/>
-      <c r="BB8" s="18" t="inlineStr"/>
-      <c r="BC8" s="18" t="inlineStr"/>
-      <c r="BD8" s="18" t="inlineStr"/>
-      <c r="BE8" s="18" t="inlineStr"/>
-      <c r="BF8" s="19" t="inlineStr"/>
-      <c r="BG8" s="19" t="inlineStr"/>
-      <c r="BH8" s="19" t="inlineStr"/>
-      <c r="BI8" s="19" t="inlineStr"/>
-      <c r="BJ8" s="19" t="inlineStr"/>
-      <c r="BK8" s="19" t="inlineStr"/>
-      <c r="BL8" s="19" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="N8" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="O8" s="13" t="inlineStr"/>
+      <c r="P8" s="13" t="inlineStr"/>
+      <c r="Q8" s="13" t="inlineStr"/>
+      <c r="R8" s="13" t="inlineStr"/>
+      <c r="S8" s="13" t="inlineStr"/>
+      <c r="T8" s="13" t="inlineStr"/>
+      <c r="U8" s="14" t="inlineStr"/>
+      <c r="V8" s="14" t="inlineStr"/>
+      <c r="W8" s="14" t="inlineStr"/>
+      <c r="X8" s="14" t="inlineStr"/>
+      <c r="Y8" s="14" t="inlineStr"/>
+      <c r="Z8" s="14" t="inlineStr"/>
+      <c r="AA8" s="15" t="inlineStr"/>
+      <c r="AB8" s="15" t="inlineStr"/>
+      <c r="AC8" s="15" t="inlineStr"/>
+      <c r="AD8" s="15" t="inlineStr"/>
+      <c r="AE8" s="15" t="inlineStr"/>
+      <c r="AF8" s="15" t="inlineStr"/>
+      <c r="AG8" s="16" t="inlineStr"/>
+      <c r="AH8" s="16" t="inlineStr"/>
+      <c r="AI8" s="16" t="inlineStr"/>
+      <c r="AJ8" s="16" t="inlineStr"/>
+      <c r="AK8" s="16" t="inlineStr"/>
+      <c r="AL8" s="16" t="inlineStr"/>
+      <c r="AM8" s="17" t="inlineStr"/>
+      <c r="AN8" s="17" t="inlineStr"/>
+      <c r="AO8" s="17" t="inlineStr"/>
+      <c r="AP8" s="17" t="inlineStr"/>
+      <c r="AQ8" s="17" t="inlineStr"/>
+      <c r="AR8" s="17" t="inlineStr"/>
+      <c r="AS8" s="18" t="inlineStr"/>
+      <c r="AT8" s="18" t="inlineStr"/>
+      <c r="AU8" s="18" t="inlineStr"/>
+      <c r="AV8" s="18" t="inlineStr"/>
+      <c r="AW8" s="18" t="inlineStr"/>
+      <c r="AX8" s="18" t="inlineStr"/>
+      <c r="AY8" s="19" t="inlineStr"/>
+      <c r="AZ8" s="19" t="inlineStr"/>
+      <c r="BA8" s="19" t="inlineStr"/>
+      <c r="BB8" s="19" t="inlineStr"/>
+      <c r="BC8" s="19" t="inlineStr"/>
+      <c r="BD8" s="19" t="inlineStr"/>
+      <c r="BE8" s="19" t="inlineStr"/>
+      <c r="BF8" s="20" t="inlineStr"/>
+      <c r="BG8" s="20" t="inlineStr"/>
+      <c r="BH8" s="20" t="inlineStr"/>
+      <c r="BI8" s="20" t="inlineStr"/>
+      <c r="BJ8" s="20" t="inlineStr"/>
+      <c r="BK8" s="20" t="inlineStr"/>
+      <c r="BL8" s="20" t="inlineStr"/>
       <c r="BM8" t="n">
         <v>0.2</v>
       </c>
       <c r="BN8" t="n">
-        <v>0.108</v>
+        <v>0.2</v>
+      </c>
+      <c r="BO8" t="inlineStr">
+        <is>
+          <t>CROSS_SELLING</t>
+        </is>
+      </c>
+      <c r="BP8" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>C007</t>
+          <t>C001</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Simone</t>
+          <t>Paulo Negrão</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Coordenador</t>
+          <t>Diretor</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -1906,118 +1889,123 @@
         <v>0.05</v>
       </c>
       <c r="M9" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="N9" s="11" t="n">
-        <v>0.5600000000000001</v>
-      </c>
-      <c r="O9" s="12" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="N9" s="12" t="n">
+        <v>0.5900000000000001</v>
+      </c>
+      <c r="O9" s="13" t="n">
         <v>0.4</v>
       </c>
-      <c r="P9" s="12" t="n">
+      <c r="P9" s="13" t="n">
         <v>80</v>
       </c>
-      <c r="Q9" s="12" t="n">
+      <c r="Q9" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="R9" s="12" t="n">
+      <c r="R9" s="13" t="n">
         <v>0.8</v>
       </c>
-      <c r="S9" s="12" t="n">
+      <c r="S9" s="13" t="n">
         <v>0.8</v>
       </c>
-      <c r="T9" s="12" t="n">
+      <c r="T9" s="13" t="n">
         <v>0.3200000000000001</v>
       </c>
-      <c r="U9" s="13" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="V9" s="13" t="n">
+      <c r="U9" s="14" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="V9" s="14" t="n">
         <v>30</v>
       </c>
-      <c r="W9" s="13" t="n">
+      <c r="W9" s="14" t="n">
         <v>100</v>
       </c>
-      <c r="X9" s="13" t="n">
+      <c r="X9" s="14" t="n">
         <v>0.3</v>
       </c>
-      <c r="Y9" s="13" t="n">
+      <c r="Y9" s="14" t="n">
         <v>0.3</v>
       </c>
-      <c r="Z9" s="13" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="AA9" s="14" t="inlineStr"/>
-      <c r="AB9" s="14" t="inlineStr"/>
-      <c r="AC9" s="14" t="inlineStr"/>
-      <c r="AD9" s="14" t="inlineStr"/>
-      <c r="AE9" s="14" t="inlineStr"/>
-      <c r="AF9" s="14" t="inlineStr"/>
-      <c r="AG9" s="15" t="inlineStr"/>
-      <c r="AH9" s="15" t="inlineStr"/>
-      <c r="AI9" s="15" t="inlineStr"/>
-      <c r="AJ9" s="15" t="inlineStr"/>
-      <c r="AK9" s="15" t="inlineStr"/>
-      <c r="AL9" s="15" t="inlineStr"/>
-      <c r="AM9" s="16" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="AN9" s="16" t="n">
+      <c r="Z9" s="14" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="AA9" s="15" t="inlineStr"/>
+      <c r="AB9" s="15" t="inlineStr"/>
+      <c r="AC9" s="15" t="inlineStr"/>
+      <c r="AD9" s="15" t="inlineStr"/>
+      <c r="AE9" s="15" t="inlineStr"/>
+      <c r="AF9" s="15" t="inlineStr"/>
+      <c r="AG9" s="16" t="inlineStr"/>
+      <c r="AH9" s="16" t="inlineStr"/>
+      <c r="AI9" s="16" t="inlineStr"/>
+      <c r="AJ9" s="16" t="inlineStr"/>
+      <c r="AK9" s="16" t="inlineStr"/>
+      <c r="AL9" s="16" t="inlineStr"/>
+      <c r="AM9" s="17" t="n">
         <v>0.3</v>
       </c>
-      <c r="AO9" s="16" t="n">
+      <c r="AN9" s="17" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="AO9" s="17" t="n">
         <v>0.5</v>
       </c>
-      <c r="AP9" s="16" t="n">
+      <c r="AP9" s="17" t="n">
         <v>0.6</v>
       </c>
-      <c r="AQ9" s="16" t="n">
+      <c r="AQ9" s="17" t="n">
         <v>0.6</v>
       </c>
-      <c r="AR9" s="16" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="AS9" s="17" t="inlineStr"/>
-      <c r="AT9" s="17" t="inlineStr"/>
-      <c r="AU9" s="17" t="inlineStr"/>
-      <c r="AV9" s="17" t="inlineStr"/>
-      <c r="AW9" s="17" t="inlineStr"/>
-      <c r="AX9" s="17" t="inlineStr"/>
-      <c r="AY9" s="18" t="inlineStr"/>
-      <c r="AZ9" s="18" t="inlineStr"/>
-      <c r="BA9" s="18" t="inlineStr"/>
-      <c r="BB9" s="18" t="inlineStr"/>
-      <c r="BC9" s="18" t="inlineStr"/>
-      <c r="BD9" s="18" t="inlineStr"/>
-      <c r="BE9" s="18" t="inlineStr"/>
-      <c r="BF9" s="19" t="inlineStr"/>
-      <c r="BG9" s="19" t="inlineStr"/>
-      <c r="BH9" s="19" t="inlineStr"/>
-      <c r="BI9" s="19" t="inlineStr"/>
-      <c r="BJ9" s="19" t="inlineStr"/>
-      <c r="BK9" s="19" t="inlineStr"/>
-      <c r="BL9" s="19" t="inlineStr"/>
+      <c r="AR9" s="17" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="AS9" s="18" t="inlineStr"/>
+      <c r="AT9" s="18" t="inlineStr"/>
+      <c r="AU9" s="18" t="inlineStr"/>
+      <c r="AV9" s="18" t="inlineStr"/>
+      <c r="AW9" s="18" t="inlineStr"/>
+      <c r="AX9" s="18" t="inlineStr"/>
+      <c r="AY9" s="19" t="inlineStr"/>
+      <c r="AZ9" s="19" t="inlineStr"/>
+      <c r="BA9" s="19" t="inlineStr"/>
+      <c r="BB9" s="19" t="inlineStr"/>
+      <c r="BC9" s="19" t="inlineStr"/>
+      <c r="BD9" s="19" t="inlineStr"/>
+      <c r="BE9" s="19" t="inlineStr"/>
+      <c r="BF9" s="20" t="inlineStr"/>
+      <c r="BG9" s="20" t="inlineStr"/>
+      <c r="BH9" s="20" t="inlineStr"/>
+      <c r="BI9" s="20" t="inlineStr"/>
+      <c r="BJ9" s="20" t="inlineStr"/>
+      <c r="BK9" s="20" t="inlineStr"/>
+      <c r="BL9" s="20" t="inlineStr"/>
       <c r="BM9" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="BN9" t="n">
-        <v>0.112</v>
+        <v>0.05900000000000001</v>
+      </c>
+      <c r="BP9" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>C010</t>
+          <t>C002</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Samanta</t>
+          <t>Antônio Rosa</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Consultor Interno</t>
+          <t>Gerente Geral</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -2052,106 +2040,123 @@
         <v>0.05</v>
       </c>
       <c r="M10" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="N10" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="N10" s="12" t="n">
+        <v>0.54</v>
+      </c>
+      <c r="O10" s="13" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="P10" s="13" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q10" s="13" t="n">
+        <v>100</v>
+      </c>
+      <c r="R10" s="13" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="S10" s="13" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="T10" s="13" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="U10" s="14" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="V10" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="W10" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="X10" s="14" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Y10" s="14" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Z10" s="14" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="AA10" s="15" t="inlineStr"/>
+      <c r="AB10" s="15" t="inlineStr"/>
+      <c r="AC10" s="15" t="inlineStr"/>
+      <c r="AD10" s="15" t="inlineStr"/>
+      <c r="AE10" s="15" t="inlineStr"/>
+      <c r="AF10" s="15" t="inlineStr"/>
+      <c r="AG10" s="16" t="inlineStr"/>
+      <c r="AH10" s="16" t="inlineStr"/>
+      <c r="AI10" s="16" t="inlineStr"/>
+      <c r="AJ10" s="16" t="inlineStr"/>
+      <c r="AK10" s="16" t="inlineStr"/>
+      <c r="AL10" s="16" t="inlineStr"/>
+      <c r="AM10" s="17" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="AN10" s="17" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="AO10" s="17" t="n">
         <v>0.5</v>
       </c>
-      <c r="O10" s="12" t="inlineStr"/>
-      <c r="P10" s="12" t="inlineStr"/>
-      <c r="Q10" s="12" t="inlineStr"/>
-      <c r="R10" s="12" t="inlineStr"/>
-      <c r="S10" s="12" t="inlineStr"/>
-      <c r="T10" s="12" t="inlineStr"/>
-      <c r="U10" s="13" t="inlineStr"/>
-      <c r="V10" s="13" t="inlineStr"/>
-      <c r="W10" s="13" t="inlineStr"/>
-      <c r="X10" s="13" t="inlineStr"/>
-      <c r="Y10" s="13" t="inlineStr"/>
-      <c r="Z10" s="13" t="inlineStr"/>
-      <c r="AA10" s="14" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="AB10" s="14" t="n">
-        <v>80</v>
-      </c>
-      <c r="AC10" s="14" t="n">
-        <v>100</v>
-      </c>
-      <c r="AD10" s="14" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AE10" s="14" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AF10" s="14" t="n">
-        <v>0.3200000000000001</v>
-      </c>
-      <c r="AG10" s="15" t="n">
+      <c r="AP10" s="17" t="n">
         <v>0.6</v>
       </c>
-      <c r="AH10" s="15" t="n">
-        <v>30</v>
-      </c>
-      <c r="AI10" s="15" t="n">
-        <v>100</v>
-      </c>
-      <c r="AJ10" s="15" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="AK10" s="15" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="AL10" s="15" t="n">
+      <c r="AQ10" s="17" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="AR10" s="17" t="n">
         <v>0.18</v>
       </c>
-      <c r="AM10" s="16" t="inlineStr"/>
-      <c r="AN10" s="16" t="inlineStr"/>
-      <c r="AO10" s="16" t="inlineStr"/>
-      <c r="AP10" s="16" t="inlineStr"/>
-      <c r="AQ10" s="16" t="inlineStr"/>
-      <c r="AR10" s="16" t="inlineStr"/>
-      <c r="AS10" s="17" t="inlineStr"/>
-      <c r="AT10" s="17" t="inlineStr"/>
-      <c r="AU10" s="17" t="inlineStr"/>
-      <c r="AV10" s="17" t="inlineStr"/>
-      <c r="AW10" s="17" t="inlineStr"/>
-      <c r="AX10" s="17" t="inlineStr"/>
-      <c r="AY10" s="18" t="inlineStr"/>
-      <c r="AZ10" s="18" t="inlineStr"/>
-      <c r="BA10" s="18" t="inlineStr"/>
-      <c r="BB10" s="18" t="inlineStr"/>
-      <c r="BC10" s="18" t="inlineStr"/>
-      <c r="BD10" s="18" t="inlineStr"/>
-      <c r="BE10" s="18" t="inlineStr"/>
-      <c r="BF10" s="19" t="inlineStr"/>
-      <c r="BG10" s="19" t="inlineStr"/>
-      <c r="BH10" s="19" t="inlineStr"/>
-      <c r="BI10" s="19" t="inlineStr"/>
-      <c r="BJ10" s="19" t="inlineStr"/>
-      <c r="BK10" s="19" t="inlineStr"/>
-      <c r="BL10" s="19" t="inlineStr"/>
+      <c r="AS10" s="18" t="inlineStr"/>
+      <c r="AT10" s="18" t="inlineStr"/>
+      <c r="AU10" s="18" t="inlineStr"/>
+      <c r="AV10" s="18" t="inlineStr"/>
+      <c r="AW10" s="18" t="inlineStr"/>
+      <c r="AX10" s="18" t="inlineStr"/>
+      <c r="AY10" s="19" t="inlineStr"/>
+      <c r="AZ10" s="19" t="inlineStr"/>
+      <c r="BA10" s="19" t="inlineStr"/>
+      <c r="BB10" s="19" t="inlineStr"/>
+      <c r="BC10" s="19" t="inlineStr"/>
+      <c r="BD10" s="19" t="inlineStr"/>
+      <c r="BE10" s="19" t="inlineStr"/>
+      <c r="BF10" s="20" t="inlineStr"/>
+      <c r="BG10" s="20" t="inlineStr"/>
+      <c r="BH10" s="20" t="inlineStr"/>
+      <c r="BI10" s="20" t="inlineStr"/>
+      <c r="BJ10" s="20" t="inlineStr"/>
+      <c r="BK10" s="20" t="inlineStr"/>
+      <c r="BL10" s="20" t="inlineStr"/>
       <c r="BM10" t="n">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="BN10" t="n">
-        <v>0.075</v>
+        <v>0.108</v>
+      </c>
+      <c r="BP10" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>C020</t>
+          <t>C007</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Mateus Machado</t>
+          <t>Simone</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Consultor Externo</t>
+          <t>Coordenador</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
@@ -2186,107 +2191,128 @@
         <v>0.05</v>
       </c>
       <c r="M11" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="N11" s="11" t="n">
-        <v>1</v>
-      </c>
-      <c r="O11" s="12" t="inlineStr"/>
-      <c r="P11" s="12" t="inlineStr"/>
-      <c r="Q11" s="12" t="inlineStr"/>
-      <c r="R11" s="12" t="inlineStr"/>
-      <c r="S11" s="12" t="inlineStr"/>
-      <c r="T11" s="12" t="inlineStr"/>
-      <c r="U11" s="13" t="inlineStr"/>
-      <c r="V11" s="13" t="inlineStr"/>
-      <c r="W11" s="13" t="inlineStr"/>
-      <c r="X11" s="13" t="inlineStr"/>
-      <c r="Y11" s="13" t="inlineStr"/>
-      <c r="Z11" s="13" t="inlineStr"/>
-      <c r="AA11" s="14" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="N11" s="12" t="n">
+        <v>0.5600000000000001</v>
+      </c>
+      <c r="O11" s="13" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="P11" s="13" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q11" s="13" t="n">
+        <v>100</v>
+      </c>
+      <c r="R11" s="13" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="S11" s="13" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="T11" s="13" t="n">
+        <v>0.3200000000000001</v>
+      </c>
+      <c r="U11" s="14" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="V11" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="W11" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="X11" s="14" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Y11" s="14" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Z11" s="14" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="AA11" s="15" t="inlineStr"/>
+      <c r="AB11" s="15" t="inlineStr"/>
+      <c r="AC11" s="15" t="inlineStr"/>
+      <c r="AD11" s="15" t="inlineStr"/>
+      <c r="AE11" s="15" t="inlineStr"/>
+      <c r="AF11" s="15" t="inlineStr"/>
+      <c r="AG11" s="16" t="inlineStr"/>
+      <c r="AH11" s="16" t="inlineStr"/>
+      <c r="AI11" s="16" t="inlineStr"/>
+      <c r="AJ11" s="16" t="inlineStr"/>
+      <c r="AK11" s="16" t="inlineStr"/>
+      <c r="AL11" s="16" t="inlineStr"/>
+      <c r="AM11" s="17" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="AN11" s="17" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="AO11" s="17" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AP11" s="17" t="n">
         <v>0.6</v>
       </c>
-      <c r="AB11" s="14" t="n">
-        <v>80</v>
-      </c>
-      <c r="AC11" s="14" t="inlineStr"/>
-      <c r="AD11" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="AE11" s="14" t="n">
-        <v>1</v>
-      </c>
-      <c r="AF11" s="14" t="n">
+      <c r="AQ11" s="17" t="n">
         <v>0.6</v>
       </c>
-      <c r="AG11" s="15" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="AH11" s="15" t="n">
-        <v>30</v>
-      </c>
-      <c r="AI11" s="15" t="inlineStr"/>
-      <c r="AJ11" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK11" s="15" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL11" s="15" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="AM11" s="16" t="inlineStr"/>
-      <c r="AN11" s="16" t="inlineStr"/>
-      <c r="AO11" s="16" t="inlineStr"/>
-      <c r="AP11" s="16" t="inlineStr"/>
-      <c r="AQ11" s="16" t="inlineStr"/>
-      <c r="AR11" s="16" t="inlineStr"/>
-      <c r="AS11" s="17" t="inlineStr"/>
-      <c r="AT11" s="17" t="inlineStr"/>
-      <c r="AU11" s="17" t="inlineStr"/>
-      <c r="AV11" s="17" t="inlineStr"/>
-      <c r="AW11" s="17" t="inlineStr"/>
-      <c r="AX11" s="17" t="inlineStr"/>
-      <c r="AY11" s="18" t="inlineStr"/>
-      <c r="AZ11" s="18" t="inlineStr"/>
-      <c r="BA11" s="18" t="inlineStr"/>
-      <c r="BB11" s="18" t="inlineStr"/>
-      <c r="BC11" s="18" t="inlineStr"/>
-      <c r="BD11" s="18" t="inlineStr"/>
-      <c r="BE11" s="18" t="inlineStr"/>
-      <c r="BF11" s="19" t="inlineStr"/>
-      <c r="BG11" s="19" t="inlineStr"/>
-      <c r="BH11" s="19" t="inlineStr"/>
-      <c r="BI11" s="19" t="inlineStr"/>
-      <c r="BJ11" s="19" t="inlineStr"/>
-      <c r="BK11" s="19" t="inlineStr"/>
-      <c r="BL11" s="19" t="inlineStr"/>
+      <c r="AR11" s="17" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="AS11" s="18" t="inlineStr"/>
+      <c r="AT11" s="18" t="inlineStr"/>
+      <c r="AU11" s="18" t="inlineStr"/>
+      <c r="AV11" s="18" t="inlineStr"/>
+      <c r="AW11" s="18" t="inlineStr"/>
+      <c r="AX11" s="18" t="inlineStr"/>
+      <c r="AY11" s="19" t="inlineStr"/>
+      <c r="AZ11" s="19" t="inlineStr"/>
+      <c r="BA11" s="19" t="inlineStr"/>
+      <c r="BB11" s="19" t="inlineStr"/>
+      <c r="BC11" s="19" t="inlineStr"/>
+      <c r="BD11" s="19" t="inlineStr"/>
+      <c r="BE11" s="19" t="inlineStr"/>
+      <c r="BF11" s="20" t="inlineStr"/>
+      <c r="BG11" s="20" t="inlineStr"/>
+      <c r="BH11" s="20" t="inlineStr"/>
+      <c r="BI11" s="20" t="inlineStr"/>
+      <c r="BJ11" s="20" t="inlineStr"/>
+      <c r="BK11" s="20" t="inlineStr"/>
+      <c r="BL11" s="20" t="inlineStr"/>
       <c r="BM11" t="n">
-        <v>0.15</v>
+        <v>0.2</v>
       </c>
       <c r="BN11" t="n">
-        <v>0.15</v>
+        <v>0.112</v>
+      </c>
+      <c r="BP11" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>C001</t>
+          <t>C010</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Paulo Negrão</t>
+          <t>Samanta</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Diretor</t>
+          <t>Consultor Interno</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>TESTE2</t>
+          <t>TESTE</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
@@ -2296,12 +2322,12 @@
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>Sonda Serie EXO</t>
+          <t>Medidor de Vazão Fixo</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>EXO</t>
+          <t>IQ Standard</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -2310,129 +2336,122 @@
         </is>
       </c>
       <c r="K12" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="L12" t="n">
         <v>0.05</v>
       </c>
       <c r="M12" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="N12" s="11" t="n">
-        <v>0.65</v>
-      </c>
-      <c r="O12" s="12" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="N12" s="12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="O12" s="13" t="inlineStr"/>
+      <c r="P12" s="13" t="inlineStr"/>
+      <c r="Q12" s="13" t="inlineStr"/>
+      <c r="R12" s="13" t="inlineStr"/>
+      <c r="S12" s="13" t="inlineStr"/>
+      <c r="T12" s="13" t="inlineStr"/>
+      <c r="U12" s="14" t="inlineStr"/>
+      <c r="V12" s="14" t="inlineStr"/>
+      <c r="W12" s="14" t="inlineStr"/>
+      <c r="X12" s="14" t="inlineStr"/>
+      <c r="Y12" s="14" t="inlineStr"/>
+      <c r="Z12" s="14" t="inlineStr"/>
+      <c r="AA12" s="15" t="n">
         <v>0.4</v>
       </c>
-      <c r="P12" s="12" t="n">
+      <c r="AB12" s="15" t="n">
         <v>80</v>
       </c>
-      <c r="Q12" s="12" t="n">
+      <c r="AC12" s="15" t="n">
         <v>100</v>
       </c>
-      <c r="R12" s="12" t="n">
+      <c r="AD12" s="15" t="n">
         <v>0.8</v>
       </c>
-      <c r="S12" s="12" t="n">
+      <c r="AE12" s="15" t="n">
         <v>0.8</v>
       </c>
-      <c r="T12" s="12" t="n">
+      <c r="AF12" s="15" t="n">
         <v>0.3200000000000001</v>
       </c>
-      <c r="U12" s="13" t="n">
+      <c r="AG12" s="16" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="AH12" s="16" t="n">
+        <v>30</v>
+      </c>
+      <c r="AI12" s="16" t="n">
+        <v>100</v>
+      </c>
+      <c r="AJ12" s="16" t="n">
         <v>0.3</v>
       </c>
-      <c r="V12" s="13" t="n">
-        <v>30</v>
-      </c>
-      <c r="W12" s="13" t="n">
-        <v>100</v>
-      </c>
-      <c r="X12" s="13" t="n">
+      <c r="AK12" s="16" t="n">
         <v>0.3</v>
       </c>
-      <c r="Y12" s="13" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="Z12" s="13" t="n">
-        <v>0.09</v>
-      </c>
-      <c r="AA12" s="14" t="inlineStr"/>
-      <c r="AB12" s="14" t="inlineStr"/>
-      <c r="AC12" s="14" t="inlineStr"/>
-      <c r="AD12" s="14" t="inlineStr"/>
-      <c r="AE12" s="14" t="inlineStr"/>
-      <c r="AF12" s="14" t="inlineStr"/>
-      <c r="AG12" s="15" t="inlineStr"/>
-      <c r="AH12" s="15" t="inlineStr"/>
-      <c r="AI12" s="15" t="inlineStr"/>
-      <c r="AJ12" s="15" t="inlineStr"/>
-      <c r="AK12" s="15" t="inlineStr"/>
-      <c r="AL12" s="15" t="inlineStr"/>
-      <c r="AM12" s="16" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="AN12" s="16" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="AO12" s="16" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AP12" s="16" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AQ12" s="16" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AR12" s="16" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="AS12" s="17" t="inlineStr"/>
-      <c r="AT12" s="17" t="inlineStr"/>
-      <c r="AU12" s="17" t="inlineStr"/>
-      <c r="AV12" s="17" t="inlineStr"/>
-      <c r="AW12" s="17" t="inlineStr"/>
-      <c r="AX12" s="17" t="inlineStr"/>
-      <c r="AY12" s="18" t="inlineStr"/>
-      <c r="AZ12" s="18" t="inlineStr"/>
-      <c r="BA12" s="18" t="inlineStr"/>
-      <c r="BB12" s="18" t="inlineStr"/>
-      <c r="BC12" s="18" t="inlineStr"/>
-      <c r="BD12" s="18" t="inlineStr"/>
-      <c r="BE12" s="18" t="inlineStr"/>
-      <c r="BF12" s="19" t="inlineStr"/>
-      <c r="BG12" s="19" t="inlineStr"/>
-      <c r="BH12" s="19" t="inlineStr"/>
-      <c r="BI12" s="19" t="inlineStr"/>
-      <c r="BJ12" s="19" t="inlineStr"/>
-      <c r="BK12" s="19" t="inlineStr"/>
-      <c r="BL12" s="19" t="inlineStr"/>
+      <c r="AL12" s="16" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="AM12" s="17" t="inlineStr"/>
+      <c r="AN12" s="17" t="inlineStr"/>
+      <c r="AO12" s="17" t="inlineStr"/>
+      <c r="AP12" s="17" t="inlineStr"/>
+      <c r="AQ12" s="17" t="inlineStr"/>
+      <c r="AR12" s="17" t="inlineStr"/>
+      <c r="AS12" s="18" t="inlineStr"/>
+      <c r="AT12" s="18" t="inlineStr"/>
+      <c r="AU12" s="18" t="inlineStr"/>
+      <c r="AV12" s="18" t="inlineStr"/>
+      <c r="AW12" s="18" t="inlineStr"/>
+      <c r="AX12" s="18" t="inlineStr"/>
+      <c r="AY12" s="19" t="inlineStr"/>
+      <c r="AZ12" s="19" t="inlineStr"/>
+      <c r="BA12" s="19" t="inlineStr"/>
+      <c r="BB12" s="19" t="inlineStr"/>
+      <c r="BC12" s="19" t="inlineStr"/>
+      <c r="BD12" s="19" t="inlineStr"/>
+      <c r="BE12" s="19" t="inlineStr"/>
+      <c r="BF12" s="20" t="inlineStr"/>
+      <c r="BG12" s="20" t="inlineStr"/>
+      <c r="BH12" s="20" t="inlineStr"/>
+      <c r="BI12" s="20" t="inlineStr"/>
+      <c r="BJ12" s="20" t="inlineStr"/>
+      <c r="BK12" s="20" t="inlineStr"/>
+      <c r="BL12" s="20" t="inlineStr"/>
       <c r="BM12" t="n">
         <v>0.15</v>
       </c>
       <c r="BN12" t="n">
-        <v>0.09750000000000002</v>
+        <v>0.075</v>
+      </c>
+      <c r="BP12" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>C002</t>
+          <t>C020</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Antônio Rosa</t>
+          <t>Mateus Machado</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Gerente Geral</t>
+          <t>Consultor Externo</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>TESTE2</t>
+          <t>TESTE</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
@@ -2442,12 +2461,12 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>Sonda Serie EXO</t>
+          <t>Medidor de Vazão Fixo</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>EXO</t>
+          <t>IQ Standard</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -2456,124 +2475,113 @@
         </is>
       </c>
       <c r="K13" t="n">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="L13" t="n">
         <v>0.05</v>
       </c>
       <c r="M13" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="N13" s="11" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="N13" s="12" t="n">
+        <v>1</v>
+      </c>
+      <c r="O13" s="13" t="inlineStr"/>
+      <c r="P13" s="13" t="inlineStr"/>
+      <c r="Q13" s="13" t="inlineStr"/>
+      <c r="R13" s="13" t="inlineStr"/>
+      <c r="S13" s="13" t="inlineStr"/>
+      <c r="T13" s="13" t="inlineStr"/>
+      <c r="U13" s="14" t="inlineStr"/>
+      <c r="V13" s="14" t="inlineStr"/>
+      <c r="W13" s="14" t="inlineStr"/>
+      <c r="X13" s="14" t="inlineStr"/>
+      <c r="Y13" s="14" t="inlineStr"/>
+      <c r="Z13" s="14" t="inlineStr"/>
+      <c r="AA13" s="15" t="n">
         <v>0.6</v>
       </c>
-      <c r="O13" s="12" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="P13" s="12" t="n">
+      <c r="AB13" s="15" t="n">
         <v>80</v>
       </c>
-      <c r="Q13" s="12" t="n">
-        <v>100</v>
-      </c>
-      <c r="R13" s="12" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="S13" s="12" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="T13" s="12" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="U13" s="13" t="n">
+      <c r="AC13" s="15" t="inlineStr"/>
+      <c r="AD13" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AE13" s="15" t="n">
+        <v>1</v>
+      </c>
+      <c r="AF13" s="15" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="AG13" s="16" t="n">
         <v>0.4</v>
       </c>
-      <c r="V13" s="13" t="n">
+      <c r="AH13" s="16" t="n">
         <v>30</v>
       </c>
-      <c r="W13" s="13" t="n">
-        <v>100</v>
-      </c>
-      <c r="X13" s="13" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="Y13" s="13" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="Z13" s="13" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="AA13" s="14" t="inlineStr"/>
-      <c r="AB13" s="14" t="inlineStr"/>
-      <c r="AC13" s="14" t="inlineStr"/>
-      <c r="AD13" s="14" t="inlineStr"/>
-      <c r="AE13" s="14" t="inlineStr"/>
-      <c r="AF13" s="14" t="inlineStr"/>
-      <c r="AG13" s="15" t="inlineStr"/>
-      <c r="AH13" s="15" t="inlineStr"/>
-      <c r="AI13" s="15" t="inlineStr"/>
-      <c r="AJ13" s="15" t="inlineStr"/>
-      <c r="AK13" s="15" t="inlineStr"/>
-      <c r="AL13" s="15" t="inlineStr"/>
-      <c r="AM13" s="16" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="AN13" s="16" t="n">
+      <c r="AI13" s="16" t="inlineStr"/>
+      <c r="AJ13" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AK13" s="16" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL13" s="16" t="n">
         <v>0.4</v>
       </c>
-      <c r="AO13" s="16" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="AP13" s="16" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AQ13" s="16" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="AR13" s="16" t="n">
-        <v>0.24</v>
-      </c>
-      <c r="AS13" s="17" t="inlineStr"/>
-      <c r="AT13" s="17" t="inlineStr"/>
-      <c r="AU13" s="17" t="inlineStr"/>
-      <c r="AV13" s="17" t="inlineStr"/>
-      <c r="AW13" s="17" t="inlineStr"/>
-      <c r="AX13" s="17" t="inlineStr"/>
-      <c r="AY13" s="18" t="inlineStr"/>
-      <c r="AZ13" s="18" t="inlineStr"/>
-      <c r="BA13" s="18" t="inlineStr"/>
-      <c r="BB13" s="18" t="inlineStr"/>
-      <c r="BC13" s="18" t="inlineStr"/>
-      <c r="BD13" s="18" t="inlineStr"/>
-      <c r="BE13" s="18" t="inlineStr"/>
-      <c r="BF13" s="19" t="inlineStr"/>
-      <c r="BG13" s="19" t="inlineStr"/>
-      <c r="BH13" s="19" t="inlineStr"/>
-      <c r="BI13" s="19" t="inlineStr"/>
-      <c r="BJ13" s="19" t="inlineStr"/>
-      <c r="BK13" s="19" t="inlineStr"/>
-      <c r="BL13" s="19" t="inlineStr"/>
+      <c r="AM13" s="17" t="inlineStr"/>
+      <c r="AN13" s="17" t="inlineStr"/>
+      <c r="AO13" s="17" t="inlineStr"/>
+      <c r="AP13" s="17" t="inlineStr"/>
+      <c r="AQ13" s="17" t="inlineStr"/>
+      <c r="AR13" s="17" t="inlineStr"/>
+      <c r="AS13" s="18" t="inlineStr"/>
+      <c r="AT13" s="18" t="inlineStr"/>
+      <c r="AU13" s="18" t="inlineStr"/>
+      <c r="AV13" s="18" t="inlineStr"/>
+      <c r="AW13" s="18" t="inlineStr"/>
+      <c r="AX13" s="18" t="inlineStr"/>
+      <c r="AY13" s="19" t="inlineStr"/>
+      <c r="AZ13" s="19" t="inlineStr"/>
+      <c r="BA13" s="19" t="inlineStr"/>
+      <c r="BB13" s="19" t="inlineStr"/>
+      <c r="BC13" s="19" t="inlineStr"/>
+      <c r="BD13" s="19" t="inlineStr"/>
+      <c r="BE13" s="19" t="inlineStr"/>
+      <c r="BF13" s="20" t="inlineStr"/>
+      <c r="BG13" s="20" t="inlineStr"/>
+      <c r="BH13" s="20" t="inlineStr"/>
+      <c r="BI13" s="20" t="inlineStr"/>
+      <c r="BJ13" s="20" t="inlineStr"/>
+      <c r="BK13" s="20" t="inlineStr"/>
+      <c r="BL13" s="20" t="inlineStr"/>
       <c r="BM13" t="n">
-        <v>0.3</v>
+        <v>0.15</v>
       </c>
       <c r="BN13" t="n">
-        <v>0.18</v>
+        <v>0.15</v>
+      </c>
+      <c r="BP13" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>C007</t>
+          <t>C001</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Simone</t>
+          <t>Paulo Negrão</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Coordenador</t>
+          <t>Diretor</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2608,118 +2616,118 @@
         <v>0.05</v>
       </c>
       <c r="M14" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="N14" s="11" t="n">
-        <v>0.6000000000000001</v>
-      </c>
-      <c r="O14" s="12" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="N14" s="12" t="n">
+        <v>0.65</v>
+      </c>
+      <c r="O14" s="13" t="n">
         <v>0.4</v>
       </c>
-      <c r="P14" s="12" t="n">
+      <c r="P14" s="13" t="n">
         <v>80</v>
       </c>
-      <c r="Q14" s="12" t="n">
+      <c r="Q14" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="R14" s="12" t="n">
+      <c r="R14" s="13" t="n">
         <v>0.8</v>
       </c>
-      <c r="S14" s="12" t="n">
+      <c r="S14" s="13" t="n">
         <v>0.8</v>
       </c>
-      <c r="T14" s="12" t="n">
+      <c r="T14" s="13" t="n">
         <v>0.3200000000000001</v>
       </c>
-      <c r="U14" s="13" t="n">
+      <c r="U14" s="14" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="V14" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="W14" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="X14" s="14" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Y14" s="14" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Z14" s="14" t="n">
+        <v>0.09</v>
+      </c>
+      <c r="AA14" s="15" t="inlineStr"/>
+      <c r="AB14" s="15" t="inlineStr"/>
+      <c r="AC14" s="15" t="inlineStr"/>
+      <c r="AD14" s="15" t="inlineStr"/>
+      <c r="AE14" s="15" t="inlineStr"/>
+      <c r="AF14" s="15" t="inlineStr"/>
+      <c r="AG14" s="16" t="inlineStr"/>
+      <c r="AH14" s="16" t="inlineStr"/>
+      <c r="AI14" s="16" t="inlineStr"/>
+      <c r="AJ14" s="16" t="inlineStr"/>
+      <c r="AK14" s="16" t="inlineStr"/>
+      <c r="AL14" s="16" t="inlineStr"/>
+      <c r="AM14" s="17" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="AN14" s="17" t="n">
         <v>0.4</v>
       </c>
-      <c r="V14" s="13" t="n">
-        <v>30</v>
-      </c>
-      <c r="W14" s="13" t="n">
-        <v>100</v>
-      </c>
-      <c r="X14" s="13" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="Y14" s="13" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="Z14" s="13" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="AA14" s="14" t="inlineStr"/>
-      <c r="AB14" s="14" t="inlineStr"/>
-      <c r="AC14" s="14" t="inlineStr"/>
-      <c r="AD14" s="14" t="inlineStr"/>
-      <c r="AE14" s="14" t="inlineStr"/>
-      <c r="AF14" s="14" t="inlineStr"/>
-      <c r="AG14" s="15" t="inlineStr"/>
-      <c r="AH14" s="15" t="inlineStr"/>
-      <c r="AI14" s="15" t="inlineStr"/>
-      <c r="AJ14" s="15" t="inlineStr"/>
-      <c r="AK14" s="15" t="inlineStr"/>
-      <c r="AL14" s="15" t="inlineStr"/>
-      <c r="AM14" s="16" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="AN14" s="16" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="AO14" s="16" t="n">
+      <c r="AO14" s="17" t="n">
         <v>0.5</v>
       </c>
-      <c r="AP14" s="16" t="n">
+      <c r="AP14" s="17" t="n">
         <v>0.8</v>
       </c>
-      <c r="AQ14" s="16" t="n">
+      <c r="AQ14" s="17" t="n">
         <v>0.8</v>
       </c>
-      <c r="AR14" s="16" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="AS14" s="17" t="inlineStr"/>
-      <c r="AT14" s="17" t="inlineStr"/>
-      <c r="AU14" s="17" t="inlineStr"/>
-      <c r="AV14" s="17" t="inlineStr"/>
-      <c r="AW14" s="17" t="inlineStr"/>
-      <c r="AX14" s="17" t="inlineStr"/>
-      <c r="AY14" s="18" t="inlineStr"/>
-      <c r="AZ14" s="18" t="inlineStr"/>
-      <c r="BA14" s="18" t="inlineStr"/>
-      <c r="BB14" s="18" t="inlineStr"/>
-      <c r="BC14" s="18" t="inlineStr"/>
-      <c r="BD14" s="18" t="inlineStr"/>
-      <c r="BE14" s="18" t="inlineStr"/>
-      <c r="BF14" s="19" t="inlineStr"/>
-      <c r="BG14" s="19" t="inlineStr"/>
-      <c r="BH14" s="19" t="inlineStr"/>
-      <c r="BI14" s="19" t="inlineStr"/>
-      <c r="BJ14" s="19" t="inlineStr"/>
-      <c r="BK14" s="19" t="inlineStr"/>
-      <c r="BL14" s="19" t="inlineStr"/>
+      <c r="AR14" s="17" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="AS14" s="18" t="inlineStr"/>
+      <c r="AT14" s="18" t="inlineStr"/>
+      <c r="AU14" s="18" t="inlineStr"/>
+      <c r="AV14" s="18" t="inlineStr"/>
+      <c r="AW14" s="18" t="inlineStr"/>
+      <c r="AX14" s="18" t="inlineStr"/>
+      <c r="AY14" s="19" t="inlineStr"/>
+      <c r="AZ14" s="19" t="inlineStr"/>
+      <c r="BA14" s="19" t="inlineStr"/>
+      <c r="BB14" s="19" t="inlineStr"/>
+      <c r="BC14" s="19" t="inlineStr"/>
+      <c r="BD14" s="19" t="inlineStr"/>
+      <c r="BE14" s="19" t="inlineStr"/>
+      <c r="BF14" s="20" t="inlineStr"/>
+      <c r="BG14" s="20" t="inlineStr"/>
+      <c r="BH14" s="20" t="inlineStr"/>
+      <c r="BI14" s="20" t="inlineStr"/>
+      <c r="BJ14" s="20" t="inlineStr"/>
+      <c r="BK14" s="20" t="inlineStr"/>
+      <c r="BL14" s="20" t="inlineStr"/>
       <c r="BM14" t="n">
-        <v>0.3</v>
+        <v>0.15</v>
       </c>
       <c r="BN14" t="n">
-        <v>0.18</v>
+        <v>0.09750000000000002</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>C010</t>
+          <t>C002</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Samanta</t>
+          <t>Antônio Rosa</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Consultor Interno</t>
+          <t>Gerente Geral</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -2754,106 +2762,118 @@
         <v>0.05</v>
       </c>
       <c r="M15" t="n">
-        <v>0.15</v>
-      </c>
-      <c r="N15" s="11" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="N15" s="12" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="O15" s="13" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="P15" s="13" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q15" s="13" t="n">
+        <v>100</v>
+      </c>
+      <c r="R15" s="13" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="S15" s="13" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="T15" s="13" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="U15" s="14" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="V15" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="W15" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="X15" s="14" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Y15" s="14" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Z15" s="14" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="AA15" s="15" t="inlineStr"/>
+      <c r="AB15" s="15" t="inlineStr"/>
+      <c r="AC15" s="15" t="inlineStr"/>
+      <c r="AD15" s="15" t="inlineStr"/>
+      <c r="AE15" s="15" t="inlineStr"/>
+      <c r="AF15" s="15" t="inlineStr"/>
+      <c r="AG15" s="16" t="inlineStr"/>
+      <c r="AH15" s="16" t="inlineStr"/>
+      <c r="AI15" s="16" t="inlineStr"/>
+      <c r="AJ15" s="16" t="inlineStr"/>
+      <c r="AK15" s="16" t="inlineStr"/>
+      <c r="AL15" s="16" t="inlineStr"/>
+      <c r="AM15" s="17" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="AN15" s="17" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="AO15" s="17" t="n">
         <v>0.5</v>
       </c>
-      <c r="O15" s="12" t="inlineStr"/>
-      <c r="P15" s="12" t="inlineStr"/>
-      <c r="Q15" s="12" t="inlineStr"/>
-      <c r="R15" s="12" t="inlineStr"/>
-      <c r="S15" s="12" t="inlineStr"/>
-      <c r="T15" s="12" t="inlineStr"/>
-      <c r="U15" s="13" t="inlineStr"/>
-      <c r="V15" s="13" t="inlineStr"/>
-      <c r="W15" s="13" t="inlineStr"/>
-      <c r="X15" s="13" t="inlineStr"/>
-      <c r="Y15" s="13" t="inlineStr"/>
-      <c r="Z15" s="13" t="inlineStr"/>
-      <c r="AA15" s="14" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="AB15" s="14" t="n">
-        <v>80</v>
-      </c>
-      <c r="AC15" s="14" t="n">
-        <v>100</v>
-      </c>
-      <c r="AD15" s="14" t="n">
+      <c r="AP15" s="17" t="n">
         <v>0.8</v>
       </c>
-      <c r="AE15" s="14" t="n">
+      <c r="AQ15" s="17" t="n">
         <v>0.8</v>
       </c>
-      <c r="AF15" s="14" t="n">
-        <v>0.3200000000000001</v>
-      </c>
-      <c r="AG15" s="15" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="AH15" s="15" t="n">
-        <v>30</v>
-      </c>
-      <c r="AI15" s="15" t="n">
-        <v>100</v>
-      </c>
-      <c r="AJ15" s="15" t="n">
+      <c r="AR15" s="17" t="n">
+        <v>0.24</v>
+      </c>
+      <c r="AS15" s="18" t="inlineStr"/>
+      <c r="AT15" s="18" t="inlineStr"/>
+      <c r="AU15" s="18" t="inlineStr"/>
+      <c r="AV15" s="18" t="inlineStr"/>
+      <c r="AW15" s="18" t="inlineStr"/>
+      <c r="AX15" s="18" t="inlineStr"/>
+      <c r="AY15" s="19" t="inlineStr"/>
+      <c r="AZ15" s="19" t="inlineStr"/>
+      <c r="BA15" s="19" t="inlineStr"/>
+      <c r="BB15" s="19" t="inlineStr"/>
+      <c r="BC15" s="19" t="inlineStr"/>
+      <c r="BD15" s="19" t="inlineStr"/>
+      <c r="BE15" s="19" t="inlineStr"/>
+      <c r="BF15" s="20" t="inlineStr"/>
+      <c r="BG15" s="20" t="inlineStr"/>
+      <c r="BH15" s="20" t="inlineStr"/>
+      <c r="BI15" s="20" t="inlineStr"/>
+      <c r="BJ15" s="20" t="inlineStr"/>
+      <c r="BK15" s="20" t="inlineStr"/>
+      <c r="BL15" s="20" t="inlineStr"/>
+      <c r="BM15" t="n">
         <v>0.3</v>
       </c>
-      <c r="AK15" s="15" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="AL15" s="15" t="n">
+      <c r="BN15" t="n">
         <v>0.18</v>
-      </c>
-      <c r="AM15" s="16" t="inlineStr"/>
-      <c r="AN15" s="16" t="inlineStr"/>
-      <c r="AO15" s="16" t="inlineStr"/>
-      <c r="AP15" s="16" t="inlineStr"/>
-      <c r="AQ15" s="16" t="inlineStr"/>
-      <c r="AR15" s="16" t="inlineStr"/>
-      <c r="AS15" s="17" t="inlineStr"/>
-      <c r="AT15" s="17" t="inlineStr"/>
-      <c r="AU15" s="17" t="inlineStr"/>
-      <c r="AV15" s="17" t="inlineStr"/>
-      <c r="AW15" s="17" t="inlineStr"/>
-      <c r="AX15" s="17" t="inlineStr"/>
-      <c r="AY15" s="18" t="inlineStr"/>
-      <c r="AZ15" s="18" t="inlineStr"/>
-      <c r="BA15" s="18" t="inlineStr"/>
-      <c r="BB15" s="18" t="inlineStr"/>
-      <c r="BC15" s="18" t="inlineStr"/>
-      <c r="BD15" s="18" t="inlineStr"/>
-      <c r="BE15" s="18" t="inlineStr"/>
-      <c r="BF15" s="19" t="inlineStr"/>
-      <c r="BG15" s="19" t="inlineStr"/>
-      <c r="BH15" s="19" t="inlineStr"/>
-      <c r="BI15" s="19" t="inlineStr"/>
-      <c r="BJ15" s="19" t="inlineStr"/>
-      <c r="BK15" s="19" t="inlineStr"/>
-      <c r="BL15" s="19" t="inlineStr"/>
-      <c r="BM15" t="n">
-        <v>0.225</v>
-      </c>
-      <c r="BN15" t="n">
-        <v>0.1125</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>C020</t>
+          <t>C007</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Mateus Machado</t>
+          <t>Simone</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>Consultor Externo</t>
+          <t>Coordenador</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -2888,85 +2908,365 @@
         <v>0.05</v>
       </c>
       <c r="M16" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="N16" s="12" t="n">
+        <v>0.6000000000000001</v>
+      </c>
+      <c r="O16" s="13" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="P16" s="13" t="n">
+        <v>80</v>
+      </c>
+      <c r="Q16" s="13" t="n">
+        <v>100</v>
+      </c>
+      <c r="R16" s="13" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="S16" s="13" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="T16" s="13" t="n">
+        <v>0.3200000000000001</v>
+      </c>
+      <c r="U16" s="14" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="V16" s="14" t="n">
+        <v>30</v>
+      </c>
+      <c r="W16" s="14" t="n">
+        <v>100</v>
+      </c>
+      <c r="X16" s="14" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Y16" s="14" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="Z16" s="14" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="AA16" s="15" t="inlineStr"/>
+      <c r="AB16" s="15" t="inlineStr"/>
+      <c r="AC16" s="15" t="inlineStr"/>
+      <c r="AD16" s="15" t="inlineStr"/>
+      <c r="AE16" s="15" t="inlineStr"/>
+      <c r="AF16" s="15" t="inlineStr"/>
+      <c r="AG16" s="16" t="inlineStr"/>
+      <c r="AH16" s="16" t="inlineStr"/>
+      <c r="AI16" s="16" t="inlineStr"/>
+      <c r="AJ16" s="16" t="inlineStr"/>
+      <c r="AK16" s="16" t="inlineStr"/>
+      <c r="AL16" s="16" t="inlineStr"/>
+      <c r="AM16" s="17" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="AN16" s="17" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="AO16" s="17" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="AP16" s="17" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AQ16" s="17" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AR16" s="17" t="n">
+        <v>0.16</v>
+      </c>
+      <c r="AS16" s="18" t="inlineStr"/>
+      <c r="AT16" s="18" t="inlineStr"/>
+      <c r="AU16" s="18" t="inlineStr"/>
+      <c r="AV16" s="18" t="inlineStr"/>
+      <c r="AW16" s="18" t="inlineStr"/>
+      <c r="AX16" s="18" t="inlineStr"/>
+      <c r="AY16" s="19" t="inlineStr"/>
+      <c r="AZ16" s="19" t="inlineStr"/>
+      <c r="BA16" s="19" t="inlineStr"/>
+      <c r="BB16" s="19" t="inlineStr"/>
+      <c r="BC16" s="19" t="inlineStr"/>
+      <c r="BD16" s="19" t="inlineStr"/>
+      <c r="BE16" s="19" t="inlineStr"/>
+      <c r="BF16" s="20" t="inlineStr"/>
+      <c r="BG16" s="20" t="inlineStr"/>
+      <c r="BH16" s="20" t="inlineStr"/>
+      <c r="BI16" s="20" t="inlineStr"/>
+      <c r="BJ16" s="20" t="inlineStr"/>
+      <c r="BK16" s="20" t="inlineStr"/>
+      <c r="BL16" s="20" t="inlineStr"/>
+      <c r="BM16" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="BN16" t="n">
+        <v>0.18</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>C010</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Samanta</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Consultor Interno</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>TESTE2</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Hidrologia</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>Sonda Serie EXO</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>EXO</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Produto</t>
+        </is>
+      </c>
+      <c r="K17" t="n">
+        <v>30</v>
+      </c>
+      <c r="L17" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M17" t="n">
         <v>0.15</v>
       </c>
-      <c r="N16" s="11" t="n">
+      <c r="N17" s="12" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="O17" s="13" t="inlineStr"/>
+      <c r="P17" s="13" t="inlineStr"/>
+      <c r="Q17" s="13" t="inlineStr"/>
+      <c r="R17" s="13" t="inlineStr"/>
+      <c r="S17" s="13" t="inlineStr"/>
+      <c r="T17" s="13" t="inlineStr"/>
+      <c r="U17" s="14" t="inlineStr"/>
+      <c r="V17" s="14" t="inlineStr"/>
+      <c r="W17" s="14" t="inlineStr"/>
+      <c r="X17" s="14" t="inlineStr"/>
+      <c r="Y17" s="14" t="inlineStr"/>
+      <c r="Z17" s="14" t="inlineStr"/>
+      <c r="AA17" s="15" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="AB17" s="15" t="n">
+        <v>80</v>
+      </c>
+      <c r="AC17" s="15" t="n">
+        <v>100</v>
+      </c>
+      <c r="AD17" s="15" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AE17" s="15" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="AF17" s="15" t="n">
+        <v>0.3200000000000001</v>
+      </c>
+      <c r="AG17" s="16" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="AH17" s="16" t="n">
+        <v>30</v>
+      </c>
+      <c r="AI17" s="16" t="n">
+        <v>100</v>
+      </c>
+      <c r="AJ17" s="16" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="AK17" s="16" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="AL17" s="16" t="n">
+        <v>0.18</v>
+      </c>
+      <c r="AM17" s="17" t="inlineStr"/>
+      <c r="AN17" s="17" t="inlineStr"/>
+      <c r="AO17" s="17" t="inlineStr"/>
+      <c r="AP17" s="17" t="inlineStr"/>
+      <c r="AQ17" s="17" t="inlineStr"/>
+      <c r="AR17" s="17" t="inlineStr"/>
+      <c r="AS17" s="18" t="inlineStr"/>
+      <c r="AT17" s="18" t="inlineStr"/>
+      <c r="AU17" s="18" t="inlineStr"/>
+      <c r="AV17" s="18" t="inlineStr"/>
+      <c r="AW17" s="18" t="inlineStr"/>
+      <c r="AX17" s="18" t="inlineStr"/>
+      <c r="AY17" s="19" t="inlineStr"/>
+      <c r="AZ17" s="19" t="inlineStr"/>
+      <c r="BA17" s="19" t="inlineStr"/>
+      <c r="BB17" s="19" t="inlineStr"/>
+      <c r="BC17" s="19" t="inlineStr"/>
+      <c r="BD17" s="19" t="inlineStr"/>
+      <c r="BE17" s="19" t="inlineStr"/>
+      <c r="BF17" s="20" t="inlineStr"/>
+      <c r="BG17" s="20" t="inlineStr"/>
+      <c r="BH17" s="20" t="inlineStr"/>
+      <c r="BI17" s="20" t="inlineStr"/>
+      <c r="BJ17" s="20" t="inlineStr"/>
+      <c r="BK17" s="20" t="inlineStr"/>
+      <c r="BL17" s="20" t="inlineStr"/>
+      <c r="BM17" t="n">
+        <v>0.225</v>
+      </c>
+      <c r="BN17" t="n">
+        <v>0.1125</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>C020</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Mateus Machado</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Consultor Externo</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>TESTE2</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Hidrologia</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>Sonda Serie EXO</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>EXO</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Produto</t>
+        </is>
+      </c>
+      <c r="K18" t="n">
+        <v>30</v>
+      </c>
+      <c r="L18" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="M18" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="N18" s="12" t="n">
         <v>1</v>
       </c>
-      <c r="O16" s="12" t="inlineStr"/>
-      <c r="P16" s="12" t="inlineStr"/>
-      <c r="Q16" s="12" t="inlineStr"/>
-      <c r="R16" s="12" t="inlineStr"/>
-      <c r="S16" s="12" t="inlineStr"/>
-      <c r="T16" s="12" t="inlineStr"/>
-      <c r="U16" s="13" t="inlineStr"/>
-      <c r="V16" s="13" t="inlineStr"/>
-      <c r="W16" s="13" t="inlineStr"/>
-      <c r="X16" s="13" t="inlineStr"/>
-      <c r="Y16" s="13" t="inlineStr"/>
-      <c r="Z16" s="13" t="inlineStr"/>
-      <c r="AA16" s="14" t="n">
+      <c r="O18" s="13" t="inlineStr"/>
+      <c r="P18" s="13" t="inlineStr"/>
+      <c r="Q18" s="13" t="inlineStr"/>
+      <c r="R18" s="13" t="inlineStr"/>
+      <c r="S18" s="13" t="inlineStr"/>
+      <c r="T18" s="13" t="inlineStr"/>
+      <c r="U18" s="14" t="inlineStr"/>
+      <c r="V18" s="14" t="inlineStr"/>
+      <c r="W18" s="14" t="inlineStr"/>
+      <c r="X18" s="14" t="inlineStr"/>
+      <c r="Y18" s="14" t="inlineStr"/>
+      <c r="Z18" s="14" t="inlineStr"/>
+      <c r="AA18" s="15" t="n">
         <v>0.6</v>
       </c>
-      <c r="AB16" s="14" t="n">
+      <c r="AB18" s="15" t="n">
         <v>80</v>
       </c>
-      <c r="AC16" s="14" t="inlineStr"/>
-      <c r="AD16" s="14" t="n">
+      <c r="AC18" s="15" t="inlineStr"/>
+      <c r="AD18" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="AE16" s="14" t="n">
+      <c r="AE18" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="AF16" s="14" t="n">
+      <c r="AF18" s="15" t="n">
         <v>0.6</v>
       </c>
-      <c r="AG16" s="15" t="n">
+      <c r="AG18" s="16" t="n">
         <v>0.4</v>
       </c>
-      <c r="AH16" s="15" t="n">
+      <c r="AH18" s="16" t="n">
         <v>30</v>
       </c>
-      <c r="AI16" s="15" t="inlineStr"/>
-      <c r="AJ16" s="15" t="n">
+      <c r="AI18" s="16" t="inlineStr"/>
+      <c r="AJ18" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="AK16" s="15" t="n">
+      <c r="AK18" s="16" t="n">
         <v>1</v>
       </c>
-      <c r="AL16" s="15" t="n">
+      <c r="AL18" s="16" t="n">
         <v>0.4</v>
       </c>
-      <c r="AM16" s="16" t="inlineStr"/>
-      <c r="AN16" s="16" t="inlineStr"/>
-      <c r="AO16" s="16" t="inlineStr"/>
-      <c r="AP16" s="16" t="inlineStr"/>
-      <c r="AQ16" s="16" t="inlineStr"/>
-      <c r="AR16" s="16" t="inlineStr"/>
-      <c r="AS16" s="17" t="inlineStr"/>
-      <c r="AT16" s="17" t="inlineStr"/>
-      <c r="AU16" s="17" t="inlineStr"/>
-      <c r="AV16" s="17" t="inlineStr"/>
-      <c r="AW16" s="17" t="inlineStr"/>
-      <c r="AX16" s="17" t="inlineStr"/>
-      <c r="AY16" s="18" t="inlineStr"/>
-      <c r="AZ16" s="18" t="inlineStr"/>
-      <c r="BA16" s="18" t="inlineStr"/>
-      <c r="BB16" s="18" t="inlineStr"/>
-      <c r="BC16" s="18" t="inlineStr"/>
-      <c r="BD16" s="18" t="inlineStr"/>
-      <c r="BE16" s="18" t="inlineStr"/>
-      <c r="BF16" s="19" t="inlineStr"/>
-      <c r="BG16" s="19" t="inlineStr"/>
-      <c r="BH16" s="19" t="inlineStr"/>
-      <c r="BI16" s="19" t="inlineStr"/>
-      <c r="BJ16" s="19" t="inlineStr"/>
-      <c r="BK16" s="19" t="inlineStr"/>
-      <c r="BL16" s="19" t="inlineStr"/>
-      <c r="BM16" t="n">
+      <c r="AM18" s="17" t="inlineStr"/>
+      <c r="AN18" s="17" t="inlineStr"/>
+      <c r="AO18" s="17" t="inlineStr"/>
+      <c r="AP18" s="17" t="inlineStr"/>
+      <c r="AQ18" s="17" t="inlineStr"/>
+      <c r="AR18" s="17" t="inlineStr"/>
+      <c r="AS18" s="18" t="inlineStr"/>
+      <c r="AT18" s="18" t="inlineStr"/>
+      <c r="AU18" s="18" t="inlineStr"/>
+      <c r="AV18" s="18" t="inlineStr"/>
+      <c r="AW18" s="18" t="inlineStr"/>
+      <c r="AX18" s="18" t="inlineStr"/>
+      <c r="AY18" s="19" t="inlineStr"/>
+      <c r="AZ18" s="19" t="inlineStr"/>
+      <c r="BA18" s="19" t="inlineStr"/>
+      <c r="BB18" s="19" t="inlineStr"/>
+      <c r="BC18" s="19" t="inlineStr"/>
+      <c r="BD18" s="19" t="inlineStr"/>
+      <c r="BE18" s="19" t="inlineStr"/>
+      <c r="BF18" s="20" t="inlineStr"/>
+      <c r="BG18" s="20" t="inlineStr"/>
+      <c r="BH18" s="20" t="inlineStr"/>
+      <c r="BI18" s="20" t="inlineStr"/>
+      <c r="BJ18" s="20" t="inlineStr"/>
+      <c r="BK18" s="20" t="inlineStr"/>
+      <c r="BL18" s="20" t="inlineStr"/>
+      <c r="BM18" t="n">
         <v>0.225</v>
       </c>
-      <c r="BN16" t="n">
+      <c r="BN18" t="n">
         <v>0.225</v>
       </c>
     </row>
@@ -2976,6 +3276,363 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AC3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>PROCESSO</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>VALOR_TOTAL_PROCESSO</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL_ANTECIPACOES</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL_PAGAMENTOS_REGULARES</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL_PAGO_ACUMULADO</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>SALDO_A_RECEBER</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL_COMISSAO_ANTECIPACOES</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL_COMISSAO_REGULARES</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL_COMISSAO_ACUMULADA</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>STATUS_PROCESSO</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>STATUS_PAGAMENTO</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>STATUS_CALCULO_MEDIAS</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>MES_ANO_FATURAMENTO</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>TCMP_JSON</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>FCMP_JSON</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>TCMP_DETALHES_JSON</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>FCMP_DETALHES_JSON</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>COLABORADORES_ENVOLVIDOS</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>DATA_PRIMEIRO_PAGAMENTO</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>DATA_ULTIMO_PAGAMENTO</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>QUANTIDADE_PAGAMENTOS</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>ULTIMA_ATUALIZACAO</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>COMISSOES_ADIANTADAS_JSON</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>STATUS_RECONCILIACAO</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>OBSERVACOES</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>TOTAL_ADIANTADO_COMISSAO</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>STATUS_PROCESSO_ANALISE</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>TCMP</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>FCMP</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TESTE</t>
+        </is>
+      </c>
+      <c r="B2" t="n">
+        <v>50</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0</v>
+      </c>
+      <c r="D2" t="n">
+        <v>80</v>
+      </c>
+      <c r="E2" t="n">
+        <v>80</v>
+      </c>
+      <c r="F2" t="n">
+        <v>-30</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.3632</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.3632</v>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>FATURADO</t>
+        </is>
+      </c>
+      <c r="K2" t="inlineStr">
+        <is>
+          <t>COMPLETO</t>
+        </is>
+      </c>
+      <c r="L2" t="inlineStr">
+        <is>
+          <t>CALCULADO</t>
+        </is>
+      </c>
+      <c r="M2" t="inlineStr">
+        <is>
+          <t>10/2025</t>
+        </is>
+      </c>
+      <c r="N2" t="inlineStr">
+        <is>
+          <t>{"André Caramello": 0.010000000000000002}</t>
+        </is>
+      </c>
+      <c r="O2" t="inlineStr">
+        <is>
+          <t>{"André Caramello": 0.4539999999999999}</t>
+        </is>
+      </c>
+      <c r="P2" t="inlineStr">
+        <is>
+          <t>{"André Caramello": {"itens": [{"negocio": "Hidrologia", "grupo": "Sonda Serie EXO", "subgrupo": "EXO", "tipo_mercadoria": "Produto", "valor": 30.0, "taxa": 0.010000000000000002, "fc": 0.47, "taxa_rateio": 0.05, "fatia_cargo": 0.2, "fc_detalhes": {"componentes": [{"nome_meta": "Faturamento da Linha", "peso": 0.15, "realizado": 80.0, "meta": 100.0, "atingimento": 0.8, "atingimento_cap": 0.8, "componente_fc": 0.12}, {"nome_meta": "Conversão da Linha", "peso": 0.3, "realizado": 30.0, "meta": 100.0, "atingimento": 0.3, "atingimento_cap": 0.3, "componente_fc": 0.09}, {"nome_meta": "Rentabilidade", "peso": 0.2, "realizado": 0.4, "meta": 0.5, "atingimento": 0.8, "atingimento_cap": 0.8, "componente_fc": 0.16000000000000003}, {"nome_meta": "Retenção de Clientes", "peso": 0.15, "realizado": 2.0, "meta": 3.0, "atingimento": 0.6666666666666666, "atingimento_cap": 0.6666666666666666, "componente_fc": 0.09999999999999999}, {"nome_meta": "Meta Fornecedor 1", "peso": 0.1, "realizado": 14.85573769241505, "meta": 25.0, "atingimento": 0.594229507696602, "atingimento_cap": 0.594229507696602, "componente_fc": 0.0594229507696602}, {"nome_meta": "Meta Fornecedor 2", "peso": 0.1, "realizado": 0.0, "meta": 25.0, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}], "fc_total": 0.47}}, {"negocio": "Hidrologia", "grupo": "Medidor de Vazão Fixo", "subgrupo": "IQ Standard", "tipo_mercadoria": "Produto", "valor": 20.0, "taxa": 0.010000000000000002, "fc": 0.42999999999999994, "taxa_rateio": 0.05, "fatia_cargo": 0.2, "fc_detalhes": {"componentes": [{"nome_meta": "Faturamento da Linha", "peso": 0.15, "realizado": 80.0, "meta": 100.0, "atingimento": 0.8, "atingimento_cap": 0.8, "componente_fc": 0.12}, {"nome_meta": "Conversão da Linha", "peso": 0.3, "realizado": 30.0, "meta": 100.0, "atingimento": 0.3, "atingimento_cap": 0.3, "componente_fc": 0.09}, {"nome_meta": "Rentabilidade", "peso": 0.2, "realizado": 0.3, "meta": 0.5, "atingimento": 0.6, "atingimento_cap": 0.6, "componente_fc": 0.12}, {"nome_meta": "Retenção de Clientes", "peso": 0.15, "realizado": 2.0, "meta": 3.0, "atingimento": 0.6666666666666666, "atingimento_cap": 0.6666666666666666, "componente_fc": 0.09999999999999999}, {"nome_meta": "Meta Fornecedor 1", "peso": 0.1, "realizado": 14.85573769241505, "meta": 25.0, "atingimento": 0.594229507696602, "atingimento_cap": 0.594229507696602, "componente_fc": 0.0594229507696602}, {"nome_meta": "Meta Fornecedor 2", "peso": 0.1, "realizado": 0.0, "meta": 25.0, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}], "fc_total": 0.42999999999999994}}], "total_valor": 50.0, "soma_ponderada": 0.5000000000000001, "tcmp_final": 0.010000000000000002}}</t>
+        </is>
+      </c>
+      <c r="Q2" t="inlineStr">
+        <is>
+          <t>{"André Caramello": {"itens": [{"negocio": "Hidrologia", "grupo": "Sonda Serie EXO", "subgrupo": "EXO", "tipo_mercadoria": "Produto", "valor": 30.0, "taxa": 0.010000000000000002, "fc": 0.47, "taxa_rateio": 0.05, "fatia_cargo": 0.2, "fc_detalhes": {"componentes": [{"nome_meta": "Faturamento da Linha", "peso": 0.15, "realizado": 80.0, "meta": 100.0, "atingimento": 0.8, "atingimento_cap": 0.8, "componente_fc": 0.12}, {"nome_meta": "Conversão da Linha", "peso": 0.3, "realizado": 30.0, "meta": 100.0, "atingimento": 0.3, "atingimento_cap": 0.3, "componente_fc": 0.09}, {"nome_meta": "Rentabilidade", "peso": 0.2, "realizado": 0.4, "meta": 0.5, "atingimento": 0.8, "atingimento_cap": 0.8, "componente_fc": 0.16000000000000003}, {"nome_meta": "Retenção de Clientes", "peso": 0.15, "realizado": 2.0, "meta": 3.0, "atingimento": 0.6666666666666666, "atingimento_cap": 0.6666666666666666, "componente_fc": 0.09999999999999999}, {"nome_meta": "Meta Fornecedor 1", "peso": 0.1, "realizado": 14.85573769241505, "meta": 25.0, "atingimento": 0.594229507696602, "atingimento_cap": 0.594229507696602, "componente_fc": 0.0594229507696602}, {"nome_meta": "Meta Fornecedor 2", "peso": 0.1, "realizado": 0.0, "meta": 25.0, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}], "fc_total": 0.47}}, {"negocio": "Hidrologia", "grupo": "Medidor de Vazão Fixo", "subgrupo": "IQ Standard", "tipo_mercadoria": "Produto", "valor": 20.0, "taxa": 0.010000000000000002, "fc": 0.42999999999999994, "taxa_rateio": 0.05, "fatia_cargo": 0.2, "fc_detalhes": {"componentes": [{"nome_meta": "Faturamento da Linha", "peso": 0.15, "realizado": 80.0, "meta": 100.0, "atingimento": 0.8, "atingimento_cap": 0.8, "componente_fc": 0.12}, {"nome_meta": "Conversão da Linha", "peso": 0.3, "realizado": 30.0, "meta": 100.0, "atingimento": 0.3, "atingimento_cap": 0.3, "componente_fc": 0.09}, {"nome_meta": "Rentabilidade", "peso": 0.2, "realizado": 0.3, "meta": 0.5, "atingimento": 0.6, "atingimento_cap": 0.6, "componente_fc": 0.12}, {"nome_meta": "Retenção de Clientes", "peso": 0.15, "realizado": 2.0, "meta": 3.0, "atingimento": 0.6666666666666666, "atingimento_cap": 0.6666666666666666, "componente_fc": 0.09999999999999999}, {"nome_meta": "Meta Fornecedor 1", "peso": 0.1, "realizado": 14.85573769241505, "meta": 25.0, "atingimento": 0.594229507696602, "atingimento_cap": 0.594229507696602, "componente_fc": 0.0594229507696602}, {"nome_meta": "Meta Fornecedor 2", "peso": 0.1, "realizado": 0.0, "meta": 25.0, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}], "fc_total": 0.42999999999999994}}], "total_valor": 50.0, "soma_ponderada": 22.699999999999996, "fcmp_final": 0.4539999999999999}}</t>
+        </is>
+      </c>
+      <c r="R2" t="inlineStr">
+        <is>
+          <t>André Caramello</t>
+        </is>
+      </c>
+      <c r="S2" s="21" t="n">
+        <v>45945</v>
+      </c>
+      <c r="T2" s="21" t="n">
+        <v>45945</v>
+      </c>
+      <c r="U2" t="n">
+        <v>2</v>
+      </c>
+      <c r="V2" s="21" t="n">
+        <v>46010.41959936343</v>
+      </c>
+      <c r="W2" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="X2" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>TESTE2</t>
+        </is>
+      </c>
+      <c r="B3" t="n">
+        <v>30</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0</v>
+      </c>
+      <c r="D3" t="n">
+        <v>60</v>
+      </c>
+      <c r="E3" t="n">
+        <v>60</v>
+      </c>
+      <c r="F3" t="n">
+        <v>-30</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.282</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>FATURADO</t>
+        </is>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>COMPLETO</t>
+        </is>
+      </c>
+      <c r="L3" t="inlineStr">
+        <is>
+          <t>CALCULADO</t>
+        </is>
+      </c>
+      <c r="M3" t="inlineStr">
+        <is>
+          <t>10/2025</t>
+        </is>
+      </c>
+      <c r="N3" t="inlineStr">
+        <is>
+          <t>{"André Caramello": 0.010000000000000002}</t>
+        </is>
+      </c>
+      <c r="O3" t="inlineStr">
+        <is>
+          <t>{"André Caramello": 0.47}</t>
+        </is>
+      </c>
+      <c r="P3" t="inlineStr">
+        <is>
+          <t>{"André Caramello": {"itens": [{"negocio": "Hidrologia", "grupo": "Sonda Serie EXO", "subgrupo": "EXO", "tipo_mercadoria": "Produto", "valor": 30.0, "taxa": 0.010000000000000002, "fc": 0.47, "taxa_rateio": 0.05, "fatia_cargo": 0.2, "fc_detalhes": {"componentes": [{"nome_meta": "Faturamento da Linha", "peso": 0.15, "realizado": 80.0, "meta": 100.0, "atingimento": 0.8, "atingimento_cap": 0.8, "componente_fc": 0.12}, {"nome_meta": "Conversão da Linha", "peso": 0.3, "realizado": 30.0, "meta": 100.0, "atingimento": 0.3, "atingimento_cap": 0.3, "componente_fc": 0.09}, {"nome_meta": "Rentabilidade", "peso": 0.2, "realizado": 0.4, "meta": 0.5, "atingimento": 0.8, "atingimento_cap": 0.8, "componente_fc": 0.16000000000000003}, {"nome_meta": "Retenção de Clientes", "peso": 0.15, "realizado": 2.0, "meta": 3.0, "atingimento": 0.6666666666666666, "atingimento_cap": 0.6666666666666666, "componente_fc": 0.09999999999999999}, {"nome_meta": "Meta Fornecedor 1", "peso": 0.1, "realizado": 14.85573769241505, "meta": 25.0, "atingimento": 0.594229507696602, "atingimento_cap": 0.594229507696602, "componente_fc": 0.0594229507696602}, {"nome_meta": "Meta Fornecedor 2", "peso": 0.1, "realizado": 0.0, "meta": 25.0, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}], "fc_total": 0.47}}], "total_valor": 30.0, "soma_ponderada": 0.30000000000000004, "tcmp_final": 0.010000000000000002}}</t>
+        </is>
+      </c>
+      <c r="Q3" t="inlineStr">
+        <is>
+          <t>{"André Caramello": {"itens": [{"negocio": "Hidrologia", "grupo": "Sonda Serie EXO", "subgrupo": "EXO", "tipo_mercadoria": "Produto", "valor": 30.0, "taxa": 0.010000000000000002, "fc": 0.47, "taxa_rateio": 0.05, "fatia_cargo": 0.2, "fc_detalhes": {"componentes": [{"nome_meta": "Faturamento da Linha", "peso": 0.15, "realizado": 80.0, "meta": 100.0, "atingimento": 0.8, "atingimento_cap": 0.8, "componente_fc": 0.12}, {"nome_meta": "Conversão da Linha", "peso": 0.3, "realizado": 30.0, "meta": 100.0, "atingimento": 0.3, "atingimento_cap": 0.3, "componente_fc": 0.09}, {"nome_meta": "Rentabilidade", "peso": 0.2, "realizado": 0.4, "meta": 0.5, "atingimento": 0.8, "atingimento_cap": 0.8, "componente_fc": 0.16000000000000003}, {"nome_meta": "Retenção de Clientes", "peso": 0.15, "realizado": 2.0, "meta": 3.0, "atingimento": 0.6666666666666666, "atingimento_cap": 0.6666666666666666, "componente_fc": 0.09999999999999999}, {"nome_meta": "Meta Fornecedor 1", "peso": 0.1, "realizado": 14.85573769241505, "meta": 25.0, "atingimento": 0.594229507696602, "atingimento_cap": 0.594229507696602, "componente_fc": 0.0594229507696602}, {"nome_meta": "Meta Fornecedor 2", "peso": 0.1, "realizado": 0.0, "meta": 25.0, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}], "fc_total": 0.47}}], "total_valor": 30.0, "soma_ponderada": 14.1, "fcmp_final": 0.47}}</t>
+        </is>
+      </c>
+      <c r="R3" t="inlineStr">
+        <is>
+          <t>André Caramello</t>
+        </is>
+      </c>
+      <c r="S3" s="21" t="n">
+        <v>45950</v>
+      </c>
+      <c r="T3" s="21" t="n">
+        <v>45950</v>
+      </c>
+      <c r="U3" t="n">
+        <v>2</v>
+      </c>
+      <c r="V3" s="21" t="n">
+        <v>46010.41959958334</v>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>{}</t>
+        </is>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>PENDENTE</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3334,7 +3991,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="16">
@@ -4208,243 +4865,68 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AU1"/>
+  <dimension ref="A1:F2"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>id_colaborador</t>
+          <t>processo</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>nome_colaborador</t>
+          <t>consultor</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>cargo</t>
+          <t>linha</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>cod_produto</t>
+          <t>taxa_pct</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>descricao_produto</t>
+          <t>decision</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>processo</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
-        <is>
-          <t>linha</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>grupo</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>subgrupo</t>
-        </is>
-      </c>
-      <c r="J1" s="1" t="inlineStr">
-        <is>
-          <t>tipo_mercadoria</t>
-        </is>
-      </c>
-      <c r="K1" s="1" t="inlineStr">
-        <is>
-          <t>faturamento_item</t>
-        </is>
-      </c>
-      <c r="L1" s="1" t="inlineStr">
-        <is>
-          <t>taxa_rateio_aplicada</t>
-        </is>
-      </c>
-      <c r="M1" s="2" t="inlineStr">
-        <is>
-          <t>fator_correcao_fc</t>
-        </is>
-      </c>
-      <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>percentual_elegibilidade_pe</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>comissao_potencial_maxima</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>comissao_calculada</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>cross_selling_decision</t>
-        </is>
-      </c>
-      <c r="R1" s="3" t="inlineStr">
-        <is>
-          <t>peso_fat_linha</t>
-        </is>
-      </c>
-      <c r="S1" s="3" t="inlineStr">
-        <is>
-          <t>realizado_fat_linha</t>
-        </is>
-      </c>
-      <c r="T1" s="3" t="inlineStr">
-        <is>
-          <t>meta_fat_linha</t>
-        </is>
-      </c>
-      <c r="U1" s="3" t="inlineStr">
-        <is>
-          <t>ating_fat_linha</t>
-        </is>
-      </c>
-      <c r="V1" s="3" t="inlineStr">
-        <is>
-          <t>ating_cap_fat_linha</t>
-        </is>
-      </c>
-      <c r="W1" s="3" t="inlineStr">
-        <is>
-          <t>comp_fc_fat_linha</t>
-        </is>
-      </c>
-      <c r="X1" s="4" t="inlineStr">
-        <is>
-          <t>peso_conv_linha</t>
-        </is>
-      </c>
-      <c r="Y1" s="4" t="inlineStr">
-        <is>
-          <t>realizado_conv_linha</t>
-        </is>
-      </c>
-      <c r="Z1" s="4" t="inlineStr">
-        <is>
-          <t>meta_conv_linha</t>
-        </is>
-      </c>
-      <c r="AA1" s="4" t="inlineStr">
-        <is>
-          <t>ating_conv_linha</t>
-        </is>
-      </c>
-      <c r="AB1" s="4" t="inlineStr">
-        <is>
-          <t>ating_cap_conv_linha</t>
-        </is>
-      </c>
-      <c r="AC1" s="4" t="inlineStr">
-        <is>
-          <t>comp_fc_conv_linha</t>
-        </is>
-      </c>
-      <c r="AD1" s="5" t="inlineStr">
-        <is>
-          <t>peso_fat_ind</t>
-        </is>
-      </c>
-      <c r="AE1" s="5" t="inlineStr">
-        <is>
-          <t>realizado_fat_ind</t>
-        </is>
-      </c>
-      <c r="AF1" s="5" t="inlineStr">
-        <is>
-          <t>meta_fat_ind</t>
-        </is>
-      </c>
-      <c r="AG1" s="5" t="inlineStr">
-        <is>
-          <t>ating_fat_ind</t>
-        </is>
-      </c>
-      <c r="AH1" s="5" t="inlineStr">
-        <is>
-          <t>ating_cap_fat_ind</t>
-        </is>
-      </c>
-      <c r="AI1" s="5" t="inlineStr">
-        <is>
-          <t>comp_fc_fat_ind</t>
-        </is>
-      </c>
-      <c r="AJ1" s="6" t="inlineStr">
-        <is>
-          <t>peso_conv_ind</t>
-        </is>
-      </c>
-      <c r="AK1" s="6" t="inlineStr">
-        <is>
-          <t>realizado_conv_ind</t>
-        </is>
-      </c>
-      <c r="AL1" s="6" t="inlineStr">
-        <is>
-          <t>meta_conv_ind</t>
-        </is>
-      </c>
-      <c r="AM1" s="6" t="inlineStr">
-        <is>
-          <t>ating_conv_ind</t>
-        </is>
-      </c>
-      <c r="AN1" s="6" t="inlineStr">
-        <is>
-          <t>ating_cap_conv_ind</t>
-        </is>
-      </c>
-      <c r="AO1" s="6" t="inlineStr">
-        <is>
-          <t>comp_fc_conv_ind</t>
-        </is>
-      </c>
-      <c r="AP1" s="9" t="inlineStr">
-        <is>
-          <t>peso_rentab</t>
-        </is>
-      </c>
-      <c r="AQ1" s="9" t="inlineStr">
-        <is>
-          <t>realizado_rentab</t>
-        </is>
-      </c>
-      <c r="AR1" s="9" t="inlineStr">
-        <is>
-          <t>meta_rentab</t>
-        </is>
-      </c>
-      <c r="AS1" s="9" t="inlineStr">
-        <is>
-          <t>ating_rentab</t>
-        </is>
-      </c>
-      <c r="AT1" s="9" t="inlineStr">
-        <is>
-          <t>ating_cap_rentab</t>
-        </is>
-      </c>
-      <c r="AU1" s="9" t="inlineStr">
-        <is>
-          <t>comp_fc_rentab</t>
+          <t>timestamp</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>TESTE</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>André Camargo</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Hidrologia</t>
+        </is>
+      </c>
+      <c r="D2" t="n">
+        <v>1</v>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>B</t>
+        </is>
+      </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>2025-12-19T10:05:47.864506</t>
         </is>
       </c>
     </row>
@@ -4459,78 +4941,248 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N1"/>
+  <dimension ref="A1:AV1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>PROCESSO</t>
+          <t>id_colaborador</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>VALOR_TOTAL_PROCESSO</t>
+          <t>nome_colaborador</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>TOTAL_ANTECIPACOES</t>
+          <t>cargo</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>TOTAL_PAGAMENTOS_REGULARES</t>
+          <t>cod_produto</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>TOTAL_PAGO_ACUMULADO</t>
+          <t>descricao_produto</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>TOTAL_ADIANTADO_COMISSAO</t>
+          <t>processo</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>STATUS_PAGAMENTO</t>
+          <t>linha</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>STATUS_RECONCILIACAO</t>
+          <t>grupo</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>STATUS_PROCESSO_ANALISE</t>
+          <t>subgrupo</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>STATUS_CALCULO_MEDIAS</t>
+          <t>tipo_mercadoria</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>MES_ANO_FATURAMENTO</t>
+          <t>faturamento_item</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>TCMP</t>
-        </is>
-      </c>
-      <c r="M1" s="1" t="inlineStr">
-        <is>
-          <t>FCMP</t>
+          <t>taxa_rateio_aplicada</t>
+        </is>
+      </c>
+      <c r="M1" s="3" t="inlineStr">
+        <is>
+          <t>fator_correcao_fc</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>ULTIMA_ATUALIZACAO</t>
+          <t>percentual_elegibilidade_pe</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>comissao_potencial_maxima</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>comissao_calculada</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>observacao</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>cross_selling_decision</t>
+        </is>
+      </c>
+      <c r="S1" s="4" t="inlineStr">
+        <is>
+          <t>peso_fat_linha</t>
+        </is>
+      </c>
+      <c r="T1" s="4" t="inlineStr">
+        <is>
+          <t>realizado_fat_linha</t>
+        </is>
+      </c>
+      <c r="U1" s="4" t="inlineStr">
+        <is>
+          <t>meta_fat_linha</t>
+        </is>
+      </c>
+      <c r="V1" s="4" t="inlineStr">
+        <is>
+          <t>ating_fat_linha</t>
+        </is>
+      </c>
+      <c r="W1" s="4" t="inlineStr">
+        <is>
+          <t>ating_cap_fat_linha</t>
+        </is>
+      </c>
+      <c r="X1" s="4" t="inlineStr">
+        <is>
+          <t>comp_fc_fat_linha</t>
+        </is>
+      </c>
+      <c r="Y1" s="5" t="inlineStr">
+        <is>
+          <t>peso_conv_linha</t>
+        </is>
+      </c>
+      <c r="Z1" s="5" t="inlineStr">
+        <is>
+          <t>realizado_conv_linha</t>
+        </is>
+      </c>
+      <c r="AA1" s="5" t="inlineStr">
+        <is>
+          <t>meta_conv_linha</t>
+        </is>
+      </c>
+      <c r="AB1" s="5" t="inlineStr">
+        <is>
+          <t>ating_conv_linha</t>
+        </is>
+      </c>
+      <c r="AC1" s="5" t="inlineStr">
+        <is>
+          <t>ating_cap_conv_linha</t>
+        </is>
+      </c>
+      <c r="AD1" s="5" t="inlineStr">
+        <is>
+          <t>comp_fc_conv_linha</t>
+        </is>
+      </c>
+      <c r="AE1" s="6" t="inlineStr">
+        <is>
+          <t>peso_fat_ind</t>
+        </is>
+      </c>
+      <c r="AF1" s="6" t="inlineStr">
+        <is>
+          <t>realizado_fat_ind</t>
+        </is>
+      </c>
+      <c r="AG1" s="6" t="inlineStr">
+        <is>
+          <t>meta_fat_ind</t>
+        </is>
+      </c>
+      <c r="AH1" s="6" t="inlineStr">
+        <is>
+          <t>ating_fat_ind</t>
+        </is>
+      </c>
+      <c r="AI1" s="6" t="inlineStr">
+        <is>
+          <t>ating_cap_fat_ind</t>
+        </is>
+      </c>
+      <c r="AJ1" s="6" t="inlineStr">
+        <is>
+          <t>comp_fc_fat_ind</t>
+        </is>
+      </c>
+      <c r="AK1" s="7" t="inlineStr">
+        <is>
+          <t>peso_conv_ind</t>
+        </is>
+      </c>
+      <c r="AL1" s="7" t="inlineStr">
+        <is>
+          <t>realizado_conv_ind</t>
+        </is>
+      </c>
+      <c r="AM1" s="7" t="inlineStr">
+        <is>
+          <t>meta_conv_ind</t>
+        </is>
+      </c>
+      <c r="AN1" s="7" t="inlineStr">
+        <is>
+          <t>ating_conv_ind</t>
+        </is>
+      </c>
+      <c r="AO1" s="7" t="inlineStr">
+        <is>
+          <t>ating_cap_conv_ind</t>
+        </is>
+      </c>
+      <c r="AP1" s="7" t="inlineStr">
+        <is>
+          <t>comp_fc_conv_ind</t>
+        </is>
+      </c>
+      <c r="AQ1" s="10" t="inlineStr">
+        <is>
+          <t>peso_rentab</t>
+        </is>
+      </c>
+      <c r="AR1" s="10" t="inlineStr">
+        <is>
+          <t>realizado_rentab</t>
+        </is>
+      </c>
+      <c r="AS1" s="10" t="inlineStr">
+        <is>
+          <t>meta_rentab</t>
+        </is>
+      </c>
+      <c r="AT1" s="10" t="inlineStr">
+        <is>
+          <t>ating_rentab</t>
+        </is>
+      </c>
+      <c r="AU1" s="10" t="inlineStr">
+        <is>
+          <t>ating_cap_rentab</t>
+        </is>
+      </c>
+      <c r="AV1" s="10" t="inlineStr">
+        <is>
+          <t>comp_fc_rentab</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Modificação no Frontend (mais bonito visualmente) e inicio da implementação da lógica de devoluções
</commit_message>
<xml_diff>
--- a/Calculo_Comissoes_10_2025.xlsx
+++ b/Calculo_Comissoes_10_2025.xlsx
@@ -990,7 +990,7 @@
       </c>
       <c r="BP2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -1039,7 +1039,7 @@
         <v>30</v>
       </c>
       <c r="L3" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="M3" t="n">
         <v>0.1</v>
@@ -1134,14 +1134,14 @@
       <c r="BK3" s="20" t="inlineStr"/>
       <c r="BL3" s="20" t="inlineStr"/>
       <c r="BM3" t="n">
-        <v>0.15</v>
+        <v>0.12</v>
       </c>
       <c r="BN3" t="n">
-        <v>0.09750000000000002</v>
+        <v>0.078</v>
       </c>
       <c r="BP3" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -1190,7 +1190,7 @@
         <v>30</v>
       </c>
       <c r="L4" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="M4" t="n">
         <v>0.2</v>
@@ -1285,14 +1285,14 @@
       <c r="BK4" s="20" t="inlineStr"/>
       <c r="BL4" s="20" t="inlineStr"/>
       <c r="BM4" t="n">
-        <v>0.3</v>
+        <v>0.24</v>
       </c>
       <c r="BN4" t="n">
-        <v>0.18</v>
+        <v>0.144</v>
       </c>
       <c r="BP4" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1341,7 @@
         <v>30</v>
       </c>
       <c r="L5" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="M5" t="n">
         <v>0.2</v>
@@ -1436,14 +1436,14 @@
       <c r="BK5" s="20" t="inlineStr"/>
       <c r="BL5" s="20" t="inlineStr"/>
       <c r="BM5" t="n">
-        <v>0.3</v>
+        <v>0.24</v>
       </c>
       <c r="BN5" t="n">
-        <v>0.18</v>
+        <v>0.144</v>
       </c>
       <c r="BP5" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -1492,7 +1492,7 @@
         <v>30</v>
       </c>
       <c r="L6" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="M6" t="n">
         <v>0.15</v>
@@ -1575,14 +1575,14 @@
       <c r="BK6" s="20" t="inlineStr"/>
       <c r="BL6" s="20" t="inlineStr"/>
       <c r="BM6" t="n">
-        <v>0.225</v>
+        <v>0.18</v>
       </c>
       <c r="BN6" t="n">
-        <v>0.1125</v>
+        <v>0.09</v>
       </c>
       <c r="BP6" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -1631,7 +1631,7 @@
         <v>30</v>
       </c>
       <c r="L7" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="M7" t="n">
         <v>0.15</v>
@@ -1710,14 +1710,14 @@
       <c r="BK7" s="20" t="inlineStr"/>
       <c r="BL7" s="20" t="inlineStr"/>
       <c r="BM7" t="n">
-        <v>0.225</v>
+        <v>0.18</v>
       </c>
       <c r="BN7" t="n">
-        <v>0.225</v>
+        <v>0.18</v>
       </c>
       <c r="BP7" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -1837,7 +1837,7 @@
       </c>
       <c r="BP8" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -1886,7 +1886,7 @@
         <v>20</v>
       </c>
       <c r="L9" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="M9" t="n">
         <v>0.1</v>
@@ -1981,14 +1981,14 @@
       <c r="BK9" s="20" t="inlineStr"/>
       <c r="BL9" s="20" t="inlineStr"/>
       <c r="BM9" t="n">
-        <v>0.1</v>
+        <v>0.08000000000000002</v>
       </c>
       <c r="BN9" t="n">
-        <v>0.05900000000000001</v>
+        <v>0.04720000000000001</v>
       </c>
       <c r="BP9" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -2037,7 +2037,7 @@
         <v>20</v>
       </c>
       <c r="L10" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="M10" t="n">
         <v>0.2</v>
@@ -2132,14 +2132,14 @@
       <c r="BK10" s="20" t="inlineStr"/>
       <c r="BL10" s="20" t="inlineStr"/>
       <c r="BM10" t="n">
-        <v>0.2</v>
+        <v>0.16</v>
       </c>
       <c r="BN10" t="n">
-        <v>0.108</v>
+        <v>0.08640000000000002</v>
       </c>
       <c r="BP10" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -2188,7 +2188,7 @@
         <v>20</v>
       </c>
       <c r="L11" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="M11" t="n">
         <v>0.2</v>
@@ -2283,14 +2283,14 @@
       <c r="BK11" s="20" t="inlineStr"/>
       <c r="BL11" s="20" t="inlineStr"/>
       <c r="BM11" t="n">
-        <v>0.2</v>
+        <v>0.16</v>
       </c>
       <c r="BN11" t="n">
-        <v>0.112</v>
+        <v>0.08960000000000003</v>
       </c>
       <c r="BP11" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -2339,7 +2339,7 @@
         <v>20</v>
       </c>
       <c r="L12" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="M12" t="n">
         <v>0.15</v>
@@ -2422,14 +2422,14 @@
       <c r="BK12" s="20" t="inlineStr"/>
       <c r="BL12" s="20" t="inlineStr"/>
       <c r="BM12" t="n">
-        <v>0.15</v>
+        <v>0.12</v>
       </c>
       <c r="BN12" t="n">
-        <v>0.075</v>
+        <v>0.06</v>
       </c>
       <c r="BP12" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -2478,7 +2478,7 @@
         <v>20</v>
       </c>
       <c r="L13" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="M13" t="n">
         <v>0.15</v>
@@ -2557,14 +2557,14 @@
       <c r="BK13" s="20" t="inlineStr"/>
       <c r="BL13" s="20" t="inlineStr"/>
       <c r="BM13" t="n">
-        <v>0.15</v>
+        <v>0.12</v>
       </c>
       <c r="BN13" t="n">
-        <v>0.15</v>
+        <v>0.12</v>
       </c>
       <c r="BP13" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
     </row>
@@ -3444,22 +3444,22 @@
         <v>0</v>
       </c>
       <c r="D2" t="n">
-        <v>80</v>
+        <v>160</v>
       </c>
       <c r="E2" t="n">
-        <v>80</v>
+        <v>160</v>
       </c>
       <c r="F2" t="n">
-        <v>-30</v>
+        <v>-110</v>
       </c>
       <c r="G2" t="n">
         <v>0</v>
       </c>
       <c r="H2" t="n">
-        <v>0.3632</v>
+        <v>0.7263999999999999</v>
       </c>
       <c r="I2" t="n">
-        <v>0.3632</v>
+        <v>0.7263999999999999</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -3513,10 +3513,10 @@
         <v>45945</v>
       </c>
       <c r="U2" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V2" s="21" t="n">
-        <v>46010.41959936343</v>
+        <v>46010.44804940972</v>
       </c>
       <c r="W2" t="inlineStr">
         <is>
@@ -3542,22 +3542,22 @@
         <v>0</v>
       </c>
       <c r="D3" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="E3" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="F3" t="n">
-        <v>-30</v>
+        <v>-90</v>
       </c>
       <c r="G3" t="n">
         <v>0</v>
       </c>
       <c r="H3" t="n">
-        <v>0.282</v>
+        <v>0.5640000000000001</v>
       </c>
       <c r="I3" t="n">
-        <v>0.282</v>
+        <v>0.5640000000000001</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -3611,10 +3611,10 @@
         <v>45950</v>
       </c>
       <c r="U3" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="V3" s="21" t="n">
-        <v>46010.41959958334</v>
+        <v>46010.44804958333</v>
       </c>
       <c r="W3" t="inlineStr">
         <is>
@@ -3731,7 +3731,7 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>0.2540000000000001</v>
+        <v>0.2227</v>
       </c>
     </row>
     <row r="3">
@@ -3751,7 +3751,7 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>0.4680000000000001</v>
+        <v>0.4104</v>
       </c>
     </row>
     <row r="4">
@@ -3831,7 +3831,7 @@
         </is>
       </c>
       <c r="D7" t="n">
-        <v>0.4720000000000001</v>
+        <v>0.4136000000000001</v>
       </c>
     </row>
     <row r="8">
@@ -3891,7 +3891,7 @@
         </is>
       </c>
       <c r="D10" t="n">
-        <v>0.3</v>
+        <v>0.2625</v>
       </c>
     </row>
     <row r="11">
@@ -4091,7 +4091,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.6</v>
+        <v>0.5249999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -4921,12 +4921,12 @@
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2025-12-19T10:05:47.864506</t>
+          <t>2025-12-19T11:26:26.948656</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Grandes avanços antes da apresentação dia 07/01/2026. Devoluções funcionando no backend e frontend (precisa de muito mais testes), com cálculo do saldo negativo que é descontado das comissões finais. Diversas melhorias no Frontend. Junção das comissões por faturamento e recebimento em uma mesma página. Etc.
</commit_message>
<xml_diff>
--- a/Calculo_Comissoes_10_2025.xlsx
+++ b/Calculo_Comissoes_10_2025.xlsx
@@ -26,9 +26,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
-    <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
-  </numFmts>
+  <numFmts count="0"/>
   <fonts count="2">
     <font>
       <name val="Calibri"/>
@@ -121,12 +119,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="22">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -163,7 +160,6 @@
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="10" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -598,257 +594,257 @@
           <t>percentual_elegibilidade_pe</t>
         </is>
       </c>
-      <c r="N1" s="3" t="inlineStr">
+      <c r="N1" s="2" t="inlineStr">
         <is>
           <t>fator_correcao_fc</t>
         </is>
       </c>
-      <c r="O1" s="4" t="inlineStr">
+      <c r="O1" s="3" t="inlineStr">
         <is>
           <t>peso_fat_linha</t>
         </is>
       </c>
-      <c r="P1" s="4" t="inlineStr">
+      <c r="P1" s="3" t="inlineStr">
         <is>
           <t>realizado_fat_linha</t>
         </is>
       </c>
-      <c r="Q1" s="4" t="inlineStr">
+      <c r="Q1" s="3" t="inlineStr">
         <is>
           <t>meta_fat_linha</t>
         </is>
       </c>
-      <c r="R1" s="4" t="inlineStr">
+      <c r="R1" s="3" t="inlineStr">
         <is>
           <t>ating_fat_linha</t>
         </is>
       </c>
-      <c r="S1" s="4" t="inlineStr">
+      <c r="S1" s="3" t="inlineStr">
         <is>
           <t>ating_cap_fat_linha</t>
         </is>
       </c>
-      <c r="T1" s="4" t="inlineStr">
+      <c r="T1" s="3" t="inlineStr">
         <is>
           <t>comp_fc_fat_linha</t>
         </is>
       </c>
-      <c r="U1" s="5" t="inlineStr">
+      <c r="U1" s="4" t="inlineStr">
         <is>
           <t>peso_conv_linha</t>
         </is>
       </c>
-      <c r="V1" s="5" t="inlineStr">
+      <c r="V1" s="4" t="inlineStr">
         <is>
           <t>realizado_conv_linha</t>
         </is>
       </c>
-      <c r="W1" s="5" t="inlineStr">
+      <c r="W1" s="4" t="inlineStr">
         <is>
           <t>meta_conv_linha</t>
         </is>
       </c>
-      <c r="X1" s="5" t="inlineStr">
+      <c r="X1" s="4" t="inlineStr">
         <is>
           <t>ating_conv_linha</t>
         </is>
       </c>
-      <c r="Y1" s="5" t="inlineStr">
+      <c r="Y1" s="4" t="inlineStr">
         <is>
           <t>ating_cap_conv_linha</t>
         </is>
       </c>
-      <c r="Z1" s="5" t="inlineStr">
+      <c r="Z1" s="4" t="inlineStr">
         <is>
           <t>comp_fc_conv_linha</t>
         </is>
       </c>
-      <c r="AA1" s="6" t="inlineStr">
+      <c r="AA1" s="5" t="inlineStr">
         <is>
           <t>peso_fat_ind</t>
         </is>
       </c>
-      <c r="AB1" s="6" t="inlineStr">
+      <c r="AB1" s="5" t="inlineStr">
         <is>
           <t>realizado_fat_ind</t>
         </is>
       </c>
-      <c r="AC1" s="6" t="inlineStr">
+      <c r="AC1" s="5" t="inlineStr">
         <is>
           <t>meta_fat_ind</t>
         </is>
       </c>
-      <c r="AD1" s="6" t="inlineStr">
+      <c r="AD1" s="5" t="inlineStr">
         <is>
           <t>ating_fat_ind</t>
         </is>
       </c>
-      <c r="AE1" s="6" t="inlineStr">
+      <c r="AE1" s="5" t="inlineStr">
         <is>
           <t>ating_cap_fat_ind</t>
         </is>
       </c>
-      <c r="AF1" s="6" t="inlineStr">
+      <c r="AF1" s="5" t="inlineStr">
         <is>
           <t>comp_fc_fat_ind</t>
         </is>
       </c>
-      <c r="AG1" s="7" t="inlineStr">
+      <c r="AG1" s="6" t="inlineStr">
         <is>
           <t>peso_conv_ind</t>
         </is>
       </c>
-      <c r="AH1" s="7" t="inlineStr">
+      <c r="AH1" s="6" t="inlineStr">
         <is>
           <t>realizado_conv_ind</t>
         </is>
       </c>
-      <c r="AI1" s="7" t="inlineStr">
+      <c r="AI1" s="6" t="inlineStr">
         <is>
           <t>meta_conv_ind</t>
         </is>
       </c>
-      <c r="AJ1" s="7" t="inlineStr">
+      <c r="AJ1" s="6" t="inlineStr">
         <is>
           <t>ating_conv_ind</t>
         </is>
       </c>
-      <c r="AK1" s="7" t="inlineStr">
+      <c r="AK1" s="6" t="inlineStr">
         <is>
           <t>ating_cap_conv_ind</t>
         </is>
       </c>
-      <c r="AL1" s="7" t="inlineStr">
+      <c r="AL1" s="6" t="inlineStr">
         <is>
           <t>comp_fc_conv_ind</t>
         </is>
       </c>
-      <c r="AM1" s="8" t="inlineStr">
+      <c r="AM1" s="7" t="inlineStr">
         <is>
           <t>peso_rentab</t>
         </is>
       </c>
-      <c r="AN1" s="8" t="inlineStr">
+      <c r="AN1" s="7" t="inlineStr">
         <is>
           <t>realizado_rentab</t>
         </is>
       </c>
-      <c r="AO1" s="8" t="inlineStr">
+      <c r="AO1" s="7" t="inlineStr">
         <is>
           <t>meta_rentab</t>
         </is>
       </c>
-      <c r="AP1" s="8" t="inlineStr">
+      <c r="AP1" s="7" t="inlineStr">
         <is>
           <t>ating_rentab</t>
         </is>
       </c>
-      <c r="AQ1" s="8" t="inlineStr">
+      <c r="AQ1" s="7" t="inlineStr">
         <is>
           <t>ating_cap_rentab</t>
         </is>
       </c>
-      <c r="AR1" s="8" t="inlineStr">
+      <c r="AR1" s="7" t="inlineStr">
         <is>
           <t>comp_fc_rentab</t>
         </is>
       </c>
-      <c r="AS1" s="9" t="inlineStr">
+      <c r="AS1" s="8" t="inlineStr">
         <is>
           <t>peso_retencao</t>
         </is>
       </c>
-      <c r="AT1" s="9" t="inlineStr">
+      <c r="AT1" s="8" t="inlineStr">
         <is>
           <t>realizado_retencao</t>
         </is>
       </c>
-      <c r="AU1" s="9" t="inlineStr">
+      <c r="AU1" s="8" t="inlineStr">
         <is>
           <t>meta_retencao</t>
         </is>
       </c>
-      <c r="AV1" s="9" t="inlineStr">
+      <c r="AV1" s="8" t="inlineStr">
         <is>
           <t>ating_retencao</t>
         </is>
       </c>
-      <c r="AW1" s="9" t="inlineStr">
+      <c r="AW1" s="8" t="inlineStr">
         <is>
           <t>ating_cap_retencao</t>
         </is>
       </c>
-      <c r="AX1" s="9" t="inlineStr">
+      <c r="AX1" s="8" t="inlineStr">
         <is>
           <t>comp_fc_retencao</t>
         </is>
       </c>
-      <c r="AY1" s="10" t="inlineStr">
+      <c r="AY1" s="9" t="inlineStr">
         <is>
           <t>peso_forn1</t>
         </is>
       </c>
-      <c r="AZ1" s="10" t="inlineStr">
+      <c r="AZ1" s="9" t="inlineStr">
         <is>
           <t>realizado_forn1</t>
         </is>
       </c>
-      <c r="BA1" s="10" t="inlineStr">
+      <c r="BA1" s="9" t="inlineStr">
         <is>
           <t>meta_forn1</t>
         </is>
       </c>
-      <c r="BB1" s="10" t="inlineStr">
+      <c r="BB1" s="9" t="inlineStr">
         <is>
           <t>ating_forn1</t>
         </is>
       </c>
-      <c r="BC1" s="10" t="inlineStr">
+      <c r="BC1" s="9" t="inlineStr">
         <is>
           <t>ating_cap_forn1</t>
         </is>
       </c>
-      <c r="BD1" s="10" t="inlineStr">
+      <c r="BD1" s="9" t="inlineStr">
         <is>
           <t>comp_fc_forn1</t>
         </is>
       </c>
-      <c r="BE1" s="10" t="inlineStr">
+      <c r="BE1" s="9" t="inlineStr">
         <is>
           <t>moeda_forn1</t>
         </is>
       </c>
-      <c r="BF1" s="11" t="inlineStr">
+      <c r="BF1" s="10" t="inlineStr">
         <is>
           <t>peso_forn2</t>
         </is>
       </c>
-      <c r="BG1" s="11" t="inlineStr">
+      <c r="BG1" s="10" t="inlineStr">
         <is>
           <t>realizado_forn2</t>
         </is>
       </c>
-      <c r="BH1" s="11" t="inlineStr">
+      <c r="BH1" s="10" t="inlineStr">
         <is>
           <t>meta_forn2</t>
         </is>
       </c>
-      <c r="BI1" s="11" t="inlineStr">
+      <c r="BI1" s="10" t="inlineStr">
         <is>
           <t>ating_forn2</t>
         </is>
       </c>
-      <c r="BJ1" s="11" t="inlineStr">
+      <c r="BJ1" s="10" t="inlineStr">
         <is>
           <t>ating_cap_forn2</t>
         </is>
       </c>
-      <c r="BK1" s="11" t="inlineStr">
+      <c r="BK1" s="10" t="inlineStr">
         <is>
           <t>comp_fc_forn2</t>
         </is>
       </c>
-      <c r="BL1" s="11" t="inlineStr">
+      <c r="BL1" s="10" t="inlineStr">
         <is>
           <t>moeda_forn2</t>
         </is>
@@ -895,6 +891,11 @@
           <t>TESTE</t>
         </is>
       </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>AAA</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr">
         <is>
           <t>Hidrologia</t>
@@ -924,59 +925,59 @@
       <c r="M2" t="n">
         <v>1</v>
       </c>
-      <c r="N2" s="12" t="n">
+      <c r="N2" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="O2" s="13" t="inlineStr"/>
-      <c r="P2" s="13" t="inlineStr"/>
-      <c r="Q2" s="13" t="inlineStr"/>
-      <c r="R2" s="13" t="inlineStr"/>
-      <c r="S2" s="13" t="inlineStr"/>
-      <c r="T2" s="13" t="inlineStr"/>
-      <c r="U2" s="14" t="inlineStr"/>
-      <c r="V2" s="14" t="inlineStr"/>
-      <c r="W2" s="14" t="inlineStr"/>
-      <c r="X2" s="14" t="inlineStr"/>
-      <c r="Y2" s="14" t="inlineStr"/>
-      <c r="Z2" s="14" t="inlineStr"/>
-      <c r="AA2" s="15" t="inlineStr"/>
-      <c r="AB2" s="15" t="inlineStr"/>
-      <c r="AC2" s="15" t="inlineStr"/>
-      <c r="AD2" s="15" t="inlineStr"/>
-      <c r="AE2" s="15" t="inlineStr"/>
-      <c r="AF2" s="15" t="inlineStr"/>
-      <c r="AG2" s="16" t="inlineStr"/>
-      <c r="AH2" s="16" t="inlineStr"/>
-      <c r="AI2" s="16" t="inlineStr"/>
-      <c r="AJ2" s="16" t="inlineStr"/>
-      <c r="AK2" s="16" t="inlineStr"/>
-      <c r="AL2" s="16" t="inlineStr"/>
-      <c r="AM2" s="17" t="inlineStr"/>
-      <c r="AN2" s="17" t="inlineStr"/>
-      <c r="AO2" s="17" t="inlineStr"/>
-      <c r="AP2" s="17" t="inlineStr"/>
-      <c r="AQ2" s="17" t="inlineStr"/>
-      <c r="AR2" s="17" t="inlineStr"/>
-      <c r="AS2" s="18" t="inlineStr"/>
-      <c r="AT2" s="18" t="inlineStr"/>
-      <c r="AU2" s="18" t="inlineStr"/>
-      <c r="AV2" s="18" t="inlineStr"/>
-      <c r="AW2" s="18" t="inlineStr"/>
-      <c r="AX2" s="18" t="inlineStr"/>
-      <c r="AY2" s="19" t="inlineStr"/>
-      <c r="AZ2" s="19" t="inlineStr"/>
-      <c r="BA2" s="19" t="inlineStr"/>
-      <c r="BB2" s="19" t="inlineStr"/>
-      <c r="BC2" s="19" t="inlineStr"/>
-      <c r="BD2" s="19" t="inlineStr"/>
-      <c r="BE2" s="19" t="inlineStr"/>
-      <c r="BF2" s="20" t="inlineStr"/>
-      <c r="BG2" s="20" t="inlineStr"/>
-      <c r="BH2" s="20" t="inlineStr"/>
-      <c r="BI2" s="20" t="inlineStr"/>
-      <c r="BJ2" s="20" t="inlineStr"/>
-      <c r="BK2" s="20" t="inlineStr"/>
-      <c r="BL2" s="20" t="inlineStr"/>
+      <c r="O2" s="12" t="inlineStr"/>
+      <c r="P2" s="12" t="inlineStr"/>
+      <c r="Q2" s="12" t="inlineStr"/>
+      <c r="R2" s="12" t="inlineStr"/>
+      <c r="S2" s="12" t="inlineStr"/>
+      <c r="T2" s="12" t="inlineStr"/>
+      <c r="U2" s="13" t="inlineStr"/>
+      <c r="V2" s="13" t="inlineStr"/>
+      <c r="W2" s="13" t="inlineStr"/>
+      <c r="X2" s="13" t="inlineStr"/>
+      <c r="Y2" s="13" t="inlineStr"/>
+      <c r="Z2" s="13" t="inlineStr"/>
+      <c r="AA2" s="14" t="inlineStr"/>
+      <c r="AB2" s="14" t="inlineStr"/>
+      <c r="AC2" s="14" t="inlineStr"/>
+      <c r="AD2" s="14" t="inlineStr"/>
+      <c r="AE2" s="14" t="inlineStr"/>
+      <c r="AF2" s="14" t="inlineStr"/>
+      <c r="AG2" s="15" t="inlineStr"/>
+      <c r="AH2" s="15" t="inlineStr"/>
+      <c r="AI2" s="15" t="inlineStr"/>
+      <c r="AJ2" s="15" t="inlineStr"/>
+      <c r="AK2" s="15" t="inlineStr"/>
+      <c r="AL2" s="15" t="inlineStr"/>
+      <c r="AM2" s="16" t="inlineStr"/>
+      <c r="AN2" s="16" t="inlineStr"/>
+      <c r="AO2" s="16" t="inlineStr"/>
+      <c r="AP2" s="16" t="inlineStr"/>
+      <c r="AQ2" s="16" t="inlineStr"/>
+      <c r="AR2" s="16" t="inlineStr"/>
+      <c r="AS2" s="17" t="inlineStr"/>
+      <c r="AT2" s="17" t="inlineStr"/>
+      <c r="AU2" s="17" t="inlineStr"/>
+      <c r="AV2" s="17" t="inlineStr"/>
+      <c r="AW2" s="17" t="inlineStr"/>
+      <c r="AX2" s="17" t="inlineStr"/>
+      <c r="AY2" s="18" t="inlineStr"/>
+      <c r="AZ2" s="18" t="inlineStr"/>
+      <c r="BA2" s="18" t="inlineStr"/>
+      <c r="BB2" s="18" t="inlineStr"/>
+      <c r="BC2" s="18" t="inlineStr"/>
+      <c r="BD2" s="18" t="inlineStr"/>
+      <c r="BE2" s="18" t="inlineStr"/>
+      <c r="BF2" s="19" t="inlineStr"/>
+      <c r="BG2" s="19" t="inlineStr"/>
+      <c r="BH2" s="19" t="inlineStr"/>
+      <c r="BI2" s="19" t="inlineStr"/>
+      <c r="BJ2" s="19" t="inlineStr"/>
+      <c r="BK2" s="19" t="inlineStr"/>
+      <c r="BL2" s="19" t="inlineStr"/>
       <c r="BM2" t="n">
         <v>0.3</v>
       </c>
@@ -1015,6 +1016,11 @@
           <t>TESTE</t>
         </is>
       </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>AAA</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr">
         <is>
           <t>Hidrologia</t>
@@ -1044,95 +1050,95 @@
       <c r="M3" t="n">
         <v>0.1</v>
       </c>
-      <c r="N3" s="12" t="n">
+      <c r="N3" s="11" t="n">
         <v>0.65</v>
       </c>
-      <c r="O3" s="13" t="n">
+      <c r="O3" s="12" t="n">
         <v>0.4</v>
       </c>
-      <c r="P3" s="13" t="n">
+      <c r="P3" s="12" t="n">
         <v>80</v>
       </c>
-      <c r="Q3" s="13" t="n">
+      <c r="Q3" s="12" t="n">
         <v>100</v>
       </c>
-      <c r="R3" s="13" t="n">
+      <c r="R3" s="12" t="n">
         <v>0.8</v>
       </c>
-      <c r="S3" s="13" t="n">
+      <c r="S3" s="12" t="n">
         <v>0.8</v>
       </c>
-      <c r="T3" s="13" t="n">
+      <c r="T3" s="12" t="n">
         <v>0.3200000000000001</v>
       </c>
-      <c r="U3" s="14" t="n">
+      <c r="U3" s="13" t="n">
         <v>0.3</v>
       </c>
-      <c r="V3" s="14" t="n">
+      <c r="V3" s="13" t="n">
         <v>30</v>
       </c>
-      <c r="W3" s="14" t="n">
+      <c r="W3" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="X3" s="14" t="n">
+      <c r="X3" s="13" t="n">
         <v>0.3</v>
       </c>
-      <c r="Y3" s="14" t="n">
+      <c r="Y3" s="13" t="n">
         <v>0.3</v>
       </c>
-      <c r="Z3" s="14" t="n">
+      <c r="Z3" s="13" t="n">
         <v>0.09</v>
       </c>
-      <c r="AA3" s="15" t="inlineStr"/>
-      <c r="AB3" s="15" t="inlineStr"/>
-      <c r="AC3" s="15" t="inlineStr"/>
-      <c r="AD3" s="15" t="inlineStr"/>
-      <c r="AE3" s="15" t="inlineStr"/>
-      <c r="AF3" s="15" t="inlineStr"/>
-      <c r="AG3" s="16" t="inlineStr"/>
-      <c r="AH3" s="16" t="inlineStr"/>
-      <c r="AI3" s="16" t="inlineStr"/>
-      <c r="AJ3" s="16" t="inlineStr"/>
-      <c r="AK3" s="16" t="inlineStr"/>
-      <c r="AL3" s="16" t="inlineStr"/>
-      <c r="AM3" s="17" t="n">
+      <c r="AA3" s="14" t="inlineStr"/>
+      <c r="AB3" s="14" t="inlineStr"/>
+      <c r="AC3" s="14" t="inlineStr"/>
+      <c r="AD3" s="14" t="inlineStr"/>
+      <c r="AE3" s="14" t="inlineStr"/>
+      <c r="AF3" s="14" t="inlineStr"/>
+      <c r="AG3" s="15" t="inlineStr"/>
+      <c r="AH3" s="15" t="inlineStr"/>
+      <c r="AI3" s="15" t="inlineStr"/>
+      <c r="AJ3" s="15" t="inlineStr"/>
+      <c r="AK3" s="15" t="inlineStr"/>
+      <c r="AL3" s="15" t="inlineStr"/>
+      <c r="AM3" s="16" t="n">
         <v>0.3</v>
       </c>
-      <c r="AN3" s="17" t="n">
+      <c r="AN3" s="16" t="n">
         <v>0.4</v>
       </c>
-      <c r="AO3" s="17" t="n">
+      <c r="AO3" s="16" t="n">
         <v>0.5</v>
       </c>
-      <c r="AP3" s="17" t="n">
+      <c r="AP3" s="16" t="n">
         <v>0.8</v>
       </c>
-      <c r="AQ3" s="17" t="n">
+      <c r="AQ3" s="16" t="n">
         <v>0.8</v>
       </c>
-      <c r="AR3" s="17" t="n">
+      <c r="AR3" s="16" t="n">
         <v>0.24</v>
       </c>
-      <c r="AS3" s="18" t="inlineStr"/>
-      <c r="AT3" s="18" t="inlineStr"/>
-      <c r="AU3" s="18" t="inlineStr"/>
-      <c r="AV3" s="18" t="inlineStr"/>
-      <c r="AW3" s="18" t="inlineStr"/>
-      <c r="AX3" s="18" t="inlineStr"/>
-      <c r="AY3" s="19" t="inlineStr"/>
-      <c r="AZ3" s="19" t="inlineStr"/>
-      <c r="BA3" s="19" t="inlineStr"/>
-      <c r="BB3" s="19" t="inlineStr"/>
-      <c r="BC3" s="19" t="inlineStr"/>
-      <c r="BD3" s="19" t="inlineStr"/>
-      <c r="BE3" s="19" t="inlineStr"/>
-      <c r="BF3" s="20" t="inlineStr"/>
-      <c r="BG3" s="20" t="inlineStr"/>
-      <c r="BH3" s="20" t="inlineStr"/>
-      <c r="BI3" s="20" t="inlineStr"/>
-      <c r="BJ3" s="20" t="inlineStr"/>
-      <c r="BK3" s="20" t="inlineStr"/>
-      <c r="BL3" s="20" t="inlineStr"/>
+      <c r="AS3" s="17" t="inlineStr"/>
+      <c r="AT3" s="17" t="inlineStr"/>
+      <c r="AU3" s="17" t="inlineStr"/>
+      <c r="AV3" s="17" t="inlineStr"/>
+      <c r="AW3" s="17" t="inlineStr"/>
+      <c r="AX3" s="17" t="inlineStr"/>
+      <c r="AY3" s="18" t="inlineStr"/>
+      <c r="AZ3" s="18" t="inlineStr"/>
+      <c r="BA3" s="18" t="inlineStr"/>
+      <c r="BB3" s="18" t="inlineStr"/>
+      <c r="BC3" s="18" t="inlineStr"/>
+      <c r="BD3" s="18" t="inlineStr"/>
+      <c r="BE3" s="18" t="inlineStr"/>
+      <c r="BF3" s="19" t="inlineStr"/>
+      <c r="BG3" s="19" t="inlineStr"/>
+      <c r="BH3" s="19" t="inlineStr"/>
+      <c r="BI3" s="19" t="inlineStr"/>
+      <c r="BJ3" s="19" t="inlineStr"/>
+      <c r="BK3" s="19" t="inlineStr"/>
+      <c r="BL3" s="19" t="inlineStr"/>
       <c r="BM3" t="n">
         <v>0.12</v>
       </c>
@@ -1166,6 +1172,11 @@
           <t>TESTE</t>
         </is>
       </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>AAA</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr">
         <is>
           <t>Hidrologia</t>
@@ -1195,95 +1206,95 @@
       <c r="M4" t="n">
         <v>0.2</v>
       </c>
-      <c r="N4" s="12" t="n">
+      <c r="N4" s="11" t="n">
         <v>0.6</v>
       </c>
-      <c r="O4" s="13" t="n">
+      <c r="O4" s="12" t="n">
         <v>0.3</v>
       </c>
-      <c r="P4" s="13" t="n">
+      <c r="P4" s="12" t="n">
         <v>80</v>
       </c>
-      <c r="Q4" s="13" t="n">
+      <c r="Q4" s="12" t="n">
         <v>100</v>
       </c>
-      <c r="R4" s="13" t="n">
+      <c r="R4" s="12" t="n">
         <v>0.8</v>
       </c>
-      <c r="S4" s="13" t="n">
+      <c r="S4" s="12" t="n">
         <v>0.8</v>
       </c>
-      <c r="T4" s="13" t="n">
+      <c r="T4" s="12" t="n">
         <v>0.24</v>
       </c>
-      <c r="U4" s="14" t="n">
+      <c r="U4" s="13" t="n">
         <v>0.4</v>
       </c>
-      <c r="V4" s="14" t="n">
+      <c r="V4" s="13" t="n">
         <v>30</v>
       </c>
-      <c r="W4" s="14" t="n">
+      <c r="W4" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="X4" s="14" t="n">
+      <c r="X4" s="13" t="n">
         <v>0.3</v>
       </c>
-      <c r="Y4" s="14" t="n">
+      <c r="Y4" s="13" t="n">
         <v>0.3</v>
       </c>
-      <c r="Z4" s="14" t="n">
+      <c r="Z4" s="13" t="n">
         <v>0.12</v>
       </c>
-      <c r="AA4" s="15" t="inlineStr"/>
-      <c r="AB4" s="15" t="inlineStr"/>
-      <c r="AC4" s="15" t="inlineStr"/>
-      <c r="AD4" s="15" t="inlineStr"/>
-      <c r="AE4" s="15" t="inlineStr"/>
-      <c r="AF4" s="15" t="inlineStr"/>
-      <c r="AG4" s="16" t="inlineStr"/>
-      <c r="AH4" s="16" t="inlineStr"/>
-      <c r="AI4" s="16" t="inlineStr"/>
-      <c r="AJ4" s="16" t="inlineStr"/>
-      <c r="AK4" s="16" t="inlineStr"/>
-      <c r="AL4" s="16" t="inlineStr"/>
-      <c r="AM4" s="17" t="n">
+      <c r="AA4" s="14" t="inlineStr"/>
+      <c r="AB4" s="14" t="inlineStr"/>
+      <c r="AC4" s="14" t="inlineStr"/>
+      <c r="AD4" s="14" t="inlineStr"/>
+      <c r="AE4" s="14" t="inlineStr"/>
+      <c r="AF4" s="14" t="inlineStr"/>
+      <c r="AG4" s="15" t="inlineStr"/>
+      <c r="AH4" s="15" t="inlineStr"/>
+      <c r="AI4" s="15" t="inlineStr"/>
+      <c r="AJ4" s="15" t="inlineStr"/>
+      <c r="AK4" s="15" t="inlineStr"/>
+      <c r="AL4" s="15" t="inlineStr"/>
+      <c r="AM4" s="16" t="n">
         <v>0.3</v>
       </c>
-      <c r="AN4" s="17" t="n">
+      <c r="AN4" s="16" t="n">
         <v>0.4</v>
       </c>
-      <c r="AO4" s="17" t="n">
+      <c r="AO4" s="16" t="n">
         <v>0.5</v>
       </c>
-      <c r="AP4" s="17" t="n">
+      <c r="AP4" s="16" t="n">
         <v>0.8</v>
       </c>
-      <c r="AQ4" s="17" t="n">
+      <c r="AQ4" s="16" t="n">
         <v>0.8</v>
       </c>
-      <c r="AR4" s="17" t="n">
+      <c r="AR4" s="16" t="n">
         <v>0.24</v>
       </c>
-      <c r="AS4" s="18" t="inlineStr"/>
-      <c r="AT4" s="18" t="inlineStr"/>
-      <c r="AU4" s="18" t="inlineStr"/>
-      <c r="AV4" s="18" t="inlineStr"/>
-      <c r="AW4" s="18" t="inlineStr"/>
-      <c r="AX4" s="18" t="inlineStr"/>
-      <c r="AY4" s="19" t="inlineStr"/>
-      <c r="AZ4" s="19" t="inlineStr"/>
-      <c r="BA4" s="19" t="inlineStr"/>
-      <c r="BB4" s="19" t="inlineStr"/>
-      <c r="BC4" s="19" t="inlineStr"/>
-      <c r="BD4" s="19" t="inlineStr"/>
-      <c r="BE4" s="19" t="inlineStr"/>
-      <c r="BF4" s="20" t="inlineStr"/>
-      <c r="BG4" s="20" t="inlineStr"/>
-      <c r="BH4" s="20" t="inlineStr"/>
-      <c r="BI4" s="20" t="inlineStr"/>
-      <c r="BJ4" s="20" t="inlineStr"/>
-      <c r="BK4" s="20" t="inlineStr"/>
-      <c r="BL4" s="20" t="inlineStr"/>
+      <c r="AS4" s="17" t="inlineStr"/>
+      <c r="AT4" s="17" t="inlineStr"/>
+      <c r="AU4" s="17" t="inlineStr"/>
+      <c r="AV4" s="17" t="inlineStr"/>
+      <c r="AW4" s="17" t="inlineStr"/>
+      <c r="AX4" s="17" t="inlineStr"/>
+      <c r="AY4" s="18" t="inlineStr"/>
+      <c r="AZ4" s="18" t="inlineStr"/>
+      <c r="BA4" s="18" t="inlineStr"/>
+      <c r="BB4" s="18" t="inlineStr"/>
+      <c r="BC4" s="18" t="inlineStr"/>
+      <c r="BD4" s="18" t="inlineStr"/>
+      <c r="BE4" s="18" t="inlineStr"/>
+      <c r="BF4" s="19" t="inlineStr"/>
+      <c r="BG4" s="19" t="inlineStr"/>
+      <c r="BH4" s="19" t="inlineStr"/>
+      <c r="BI4" s="19" t="inlineStr"/>
+      <c r="BJ4" s="19" t="inlineStr"/>
+      <c r="BK4" s="19" t="inlineStr"/>
+      <c r="BL4" s="19" t="inlineStr"/>
       <c r="BM4" t="n">
         <v>0.24</v>
       </c>
@@ -1317,6 +1328,11 @@
           <t>TESTE</t>
         </is>
       </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>AAA</t>
+        </is>
+      </c>
       <c r="G5" t="inlineStr">
         <is>
           <t>Hidrologia</t>
@@ -1346,95 +1362,95 @@
       <c r="M5" t="n">
         <v>0.2</v>
       </c>
-      <c r="N5" s="12" t="n">
+      <c r="N5" s="11" t="n">
         <v>0.6000000000000001</v>
       </c>
-      <c r="O5" s="13" t="n">
+      <c r="O5" s="12" t="n">
         <v>0.4</v>
       </c>
-      <c r="P5" s="13" t="n">
+      <c r="P5" s="12" t="n">
         <v>80</v>
       </c>
-      <c r="Q5" s="13" t="n">
+      <c r="Q5" s="12" t="n">
         <v>100</v>
       </c>
-      <c r="R5" s="13" t="n">
+      <c r="R5" s="12" t="n">
         <v>0.8</v>
       </c>
-      <c r="S5" s="13" t="n">
+      <c r="S5" s="12" t="n">
         <v>0.8</v>
       </c>
-      <c r="T5" s="13" t="n">
+      <c r="T5" s="12" t="n">
         <v>0.3200000000000001</v>
       </c>
-      <c r="U5" s="14" t="n">
+      <c r="U5" s="13" t="n">
         <v>0.4</v>
       </c>
-      <c r="V5" s="14" t="n">
+      <c r="V5" s="13" t="n">
         <v>30</v>
       </c>
-      <c r="W5" s="14" t="n">
+      <c r="W5" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="X5" s="14" t="n">
+      <c r="X5" s="13" t="n">
         <v>0.3</v>
       </c>
-      <c r="Y5" s="14" t="n">
+      <c r="Y5" s="13" t="n">
         <v>0.3</v>
       </c>
-      <c r="Z5" s="14" t="n">
+      <c r="Z5" s="13" t="n">
         <v>0.12</v>
       </c>
-      <c r="AA5" s="15" t="inlineStr"/>
-      <c r="AB5" s="15" t="inlineStr"/>
-      <c r="AC5" s="15" t="inlineStr"/>
-      <c r="AD5" s="15" t="inlineStr"/>
-      <c r="AE5" s="15" t="inlineStr"/>
-      <c r="AF5" s="15" t="inlineStr"/>
-      <c r="AG5" s="16" t="inlineStr"/>
-      <c r="AH5" s="16" t="inlineStr"/>
-      <c r="AI5" s="16" t="inlineStr"/>
-      <c r="AJ5" s="16" t="inlineStr"/>
-      <c r="AK5" s="16" t="inlineStr"/>
-      <c r="AL5" s="16" t="inlineStr"/>
-      <c r="AM5" s="17" t="n">
+      <c r="AA5" s="14" t="inlineStr"/>
+      <c r="AB5" s="14" t="inlineStr"/>
+      <c r="AC5" s="14" t="inlineStr"/>
+      <c r="AD5" s="14" t="inlineStr"/>
+      <c r="AE5" s="14" t="inlineStr"/>
+      <c r="AF5" s="14" t="inlineStr"/>
+      <c r="AG5" s="15" t="inlineStr"/>
+      <c r="AH5" s="15" t="inlineStr"/>
+      <c r="AI5" s="15" t="inlineStr"/>
+      <c r="AJ5" s="15" t="inlineStr"/>
+      <c r="AK5" s="15" t="inlineStr"/>
+      <c r="AL5" s="15" t="inlineStr"/>
+      <c r="AM5" s="16" t="n">
         <v>0.2</v>
       </c>
-      <c r="AN5" s="17" t="n">
+      <c r="AN5" s="16" t="n">
         <v>0.4</v>
       </c>
-      <c r="AO5" s="17" t="n">
+      <c r="AO5" s="16" t="n">
         <v>0.5</v>
       </c>
-      <c r="AP5" s="17" t="n">
+      <c r="AP5" s="16" t="n">
         <v>0.8</v>
       </c>
-      <c r="AQ5" s="17" t="n">
+      <c r="AQ5" s="16" t="n">
         <v>0.8</v>
       </c>
-      <c r="AR5" s="17" t="n">
+      <c r="AR5" s="16" t="n">
         <v>0.16</v>
       </c>
-      <c r="AS5" s="18" t="inlineStr"/>
-      <c r="AT5" s="18" t="inlineStr"/>
-      <c r="AU5" s="18" t="inlineStr"/>
-      <c r="AV5" s="18" t="inlineStr"/>
-      <c r="AW5" s="18" t="inlineStr"/>
-      <c r="AX5" s="18" t="inlineStr"/>
-      <c r="AY5" s="19" t="inlineStr"/>
-      <c r="AZ5" s="19" t="inlineStr"/>
-      <c r="BA5" s="19" t="inlineStr"/>
-      <c r="BB5" s="19" t="inlineStr"/>
-      <c r="BC5" s="19" t="inlineStr"/>
-      <c r="BD5" s="19" t="inlineStr"/>
-      <c r="BE5" s="19" t="inlineStr"/>
-      <c r="BF5" s="20" t="inlineStr"/>
-      <c r="BG5" s="20" t="inlineStr"/>
-      <c r="BH5" s="20" t="inlineStr"/>
-      <c r="BI5" s="20" t="inlineStr"/>
-      <c r="BJ5" s="20" t="inlineStr"/>
-      <c r="BK5" s="20" t="inlineStr"/>
-      <c r="BL5" s="20" t="inlineStr"/>
+      <c r="AS5" s="17" t="inlineStr"/>
+      <c r="AT5" s="17" t="inlineStr"/>
+      <c r="AU5" s="17" t="inlineStr"/>
+      <c r="AV5" s="17" t="inlineStr"/>
+      <c r="AW5" s="17" t="inlineStr"/>
+      <c r="AX5" s="17" t="inlineStr"/>
+      <c r="AY5" s="18" t="inlineStr"/>
+      <c r="AZ5" s="18" t="inlineStr"/>
+      <c r="BA5" s="18" t="inlineStr"/>
+      <c r="BB5" s="18" t="inlineStr"/>
+      <c r="BC5" s="18" t="inlineStr"/>
+      <c r="BD5" s="18" t="inlineStr"/>
+      <c r="BE5" s="18" t="inlineStr"/>
+      <c r="BF5" s="19" t="inlineStr"/>
+      <c r="BG5" s="19" t="inlineStr"/>
+      <c r="BH5" s="19" t="inlineStr"/>
+      <c r="BI5" s="19" t="inlineStr"/>
+      <c r="BJ5" s="19" t="inlineStr"/>
+      <c r="BK5" s="19" t="inlineStr"/>
+      <c r="BL5" s="19" t="inlineStr"/>
       <c r="BM5" t="n">
         <v>0.24</v>
       </c>
@@ -1468,6 +1484,11 @@
           <t>TESTE</t>
         </is>
       </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>AAA</t>
+        </is>
+      </c>
       <c r="G6" t="inlineStr">
         <is>
           <t>Hidrologia</t>
@@ -1497,83 +1518,83 @@
       <c r="M6" t="n">
         <v>0.15</v>
       </c>
-      <c r="N6" s="12" t="n">
+      <c r="N6" s="11" t="n">
         <v>0.5</v>
       </c>
-      <c r="O6" s="13" t="inlineStr"/>
-      <c r="P6" s="13" t="inlineStr"/>
-      <c r="Q6" s="13" t="inlineStr"/>
-      <c r="R6" s="13" t="inlineStr"/>
-      <c r="S6" s="13" t="inlineStr"/>
-      <c r="T6" s="13" t="inlineStr"/>
-      <c r="U6" s="14" t="inlineStr"/>
-      <c r="V6" s="14" t="inlineStr"/>
-      <c r="W6" s="14" t="inlineStr"/>
-      <c r="X6" s="14" t="inlineStr"/>
-      <c r="Y6" s="14" t="inlineStr"/>
-      <c r="Z6" s="14" t="inlineStr"/>
-      <c r="AA6" s="15" t="n">
+      <c r="O6" s="12" t="inlineStr"/>
+      <c r="P6" s="12" t="inlineStr"/>
+      <c r="Q6" s="12" t="inlineStr"/>
+      <c r="R6" s="12" t="inlineStr"/>
+      <c r="S6" s="12" t="inlineStr"/>
+      <c r="T6" s="12" t="inlineStr"/>
+      <c r="U6" s="13" t="inlineStr"/>
+      <c r="V6" s="13" t="inlineStr"/>
+      <c r="W6" s="13" t="inlineStr"/>
+      <c r="X6" s="13" t="inlineStr"/>
+      <c r="Y6" s="13" t="inlineStr"/>
+      <c r="Z6" s="13" t="inlineStr"/>
+      <c r="AA6" s="14" t="n">
         <v>0.4</v>
       </c>
-      <c r="AB6" s="15" t="n">
+      <c r="AB6" s="14" t="n">
         <v>80</v>
       </c>
-      <c r="AC6" s="15" t="n">
+      <c r="AC6" s="14" t="n">
         <v>100</v>
       </c>
-      <c r="AD6" s="15" t="n">
+      <c r="AD6" s="14" t="n">
         <v>0.8</v>
       </c>
-      <c r="AE6" s="15" t="n">
+      <c r="AE6" s="14" t="n">
         <v>0.8</v>
       </c>
-      <c r="AF6" s="15" t="n">
+      <c r="AF6" s="14" t="n">
         <v>0.3200000000000001</v>
       </c>
-      <c r="AG6" s="16" t="n">
+      <c r="AG6" s="15" t="n">
         <v>0.6</v>
       </c>
-      <c r="AH6" s="16" t="n">
+      <c r="AH6" s="15" t="n">
         <v>30</v>
       </c>
-      <c r="AI6" s="16" t="n">
+      <c r="AI6" s="15" t="n">
         <v>100</v>
       </c>
-      <c r="AJ6" s="16" t="n">
+      <c r="AJ6" s="15" t="n">
         <v>0.3</v>
       </c>
-      <c r="AK6" s="16" t="n">
+      <c r="AK6" s="15" t="n">
         <v>0.3</v>
       </c>
-      <c r="AL6" s="16" t="n">
+      <c r="AL6" s="15" t="n">
         <v>0.18</v>
       </c>
-      <c r="AM6" s="17" t="inlineStr"/>
-      <c r="AN6" s="17" t="inlineStr"/>
-      <c r="AO6" s="17" t="inlineStr"/>
-      <c r="AP6" s="17" t="inlineStr"/>
-      <c r="AQ6" s="17" t="inlineStr"/>
-      <c r="AR6" s="17" t="inlineStr"/>
-      <c r="AS6" s="18" t="inlineStr"/>
-      <c r="AT6" s="18" t="inlineStr"/>
-      <c r="AU6" s="18" t="inlineStr"/>
-      <c r="AV6" s="18" t="inlineStr"/>
-      <c r="AW6" s="18" t="inlineStr"/>
-      <c r="AX6" s="18" t="inlineStr"/>
-      <c r="AY6" s="19" t="inlineStr"/>
-      <c r="AZ6" s="19" t="inlineStr"/>
-      <c r="BA6" s="19" t="inlineStr"/>
-      <c r="BB6" s="19" t="inlineStr"/>
-      <c r="BC6" s="19" t="inlineStr"/>
-      <c r="BD6" s="19" t="inlineStr"/>
-      <c r="BE6" s="19" t="inlineStr"/>
-      <c r="BF6" s="20" t="inlineStr"/>
-      <c r="BG6" s="20" t="inlineStr"/>
-      <c r="BH6" s="20" t="inlineStr"/>
-      <c r="BI6" s="20" t="inlineStr"/>
-      <c r="BJ6" s="20" t="inlineStr"/>
-      <c r="BK6" s="20" t="inlineStr"/>
-      <c r="BL6" s="20" t="inlineStr"/>
+      <c r="AM6" s="16" t="inlineStr"/>
+      <c r="AN6" s="16" t="inlineStr"/>
+      <c r="AO6" s="16" t="inlineStr"/>
+      <c r="AP6" s="16" t="inlineStr"/>
+      <c r="AQ6" s="16" t="inlineStr"/>
+      <c r="AR6" s="16" t="inlineStr"/>
+      <c r="AS6" s="17" t="inlineStr"/>
+      <c r="AT6" s="17" t="inlineStr"/>
+      <c r="AU6" s="17" t="inlineStr"/>
+      <c r="AV6" s="17" t="inlineStr"/>
+      <c r="AW6" s="17" t="inlineStr"/>
+      <c r="AX6" s="17" t="inlineStr"/>
+      <c r="AY6" s="18" t="inlineStr"/>
+      <c r="AZ6" s="18" t="inlineStr"/>
+      <c r="BA6" s="18" t="inlineStr"/>
+      <c r="BB6" s="18" t="inlineStr"/>
+      <c r="BC6" s="18" t="inlineStr"/>
+      <c r="BD6" s="18" t="inlineStr"/>
+      <c r="BE6" s="18" t="inlineStr"/>
+      <c r="BF6" s="19" t="inlineStr"/>
+      <c r="BG6" s="19" t="inlineStr"/>
+      <c r="BH6" s="19" t="inlineStr"/>
+      <c r="BI6" s="19" t="inlineStr"/>
+      <c r="BJ6" s="19" t="inlineStr"/>
+      <c r="BK6" s="19" t="inlineStr"/>
+      <c r="BL6" s="19" t="inlineStr"/>
       <c r="BM6" t="n">
         <v>0.18</v>
       </c>
@@ -1607,6 +1628,11 @@
           <t>TESTE</t>
         </is>
       </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>AAA</t>
+        </is>
+      </c>
       <c r="G7" t="inlineStr">
         <is>
           <t>Hidrologia</t>
@@ -1636,79 +1662,79 @@
       <c r="M7" t="n">
         <v>0.15</v>
       </c>
-      <c r="N7" s="12" t="n">
+      <c r="N7" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="O7" s="13" t="inlineStr"/>
-      <c r="P7" s="13" t="inlineStr"/>
-      <c r="Q7" s="13" t="inlineStr"/>
-      <c r="R7" s="13" t="inlineStr"/>
-      <c r="S7" s="13" t="inlineStr"/>
-      <c r="T7" s="13" t="inlineStr"/>
-      <c r="U7" s="14" t="inlineStr"/>
-      <c r="V7" s="14" t="inlineStr"/>
-      <c r="W7" s="14" t="inlineStr"/>
-      <c r="X7" s="14" t="inlineStr"/>
-      <c r="Y7" s="14" t="inlineStr"/>
-      <c r="Z7" s="14" t="inlineStr"/>
-      <c r="AA7" s="15" t="n">
+      <c r="O7" s="12" t="inlineStr"/>
+      <c r="P7" s="12" t="inlineStr"/>
+      <c r="Q7" s="12" t="inlineStr"/>
+      <c r="R7" s="12" t="inlineStr"/>
+      <c r="S7" s="12" t="inlineStr"/>
+      <c r="T7" s="12" t="inlineStr"/>
+      <c r="U7" s="13" t="inlineStr"/>
+      <c r="V7" s="13" t="inlineStr"/>
+      <c r="W7" s="13" t="inlineStr"/>
+      <c r="X7" s="13" t="inlineStr"/>
+      <c r="Y7" s="13" t="inlineStr"/>
+      <c r="Z7" s="13" t="inlineStr"/>
+      <c r="AA7" s="14" t="n">
         <v>0.6</v>
       </c>
-      <c r="AB7" s="15" t="n">
+      <c r="AB7" s="14" t="n">
         <v>80</v>
       </c>
-      <c r="AC7" s="15" t="inlineStr"/>
-      <c r="AD7" s="15" t="n">
+      <c r="AC7" s="14" t="inlineStr"/>
+      <c r="AD7" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="AE7" s="15" t="n">
+      <c r="AE7" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="AF7" s="15" t="n">
+      <c r="AF7" s="14" t="n">
         <v>0.6</v>
       </c>
-      <c r="AG7" s="16" t="n">
+      <c r="AG7" s="15" t="n">
         <v>0.4</v>
       </c>
-      <c r="AH7" s="16" t="n">
+      <c r="AH7" s="15" t="n">
         <v>30</v>
       </c>
-      <c r="AI7" s="16" t="inlineStr"/>
-      <c r="AJ7" s="16" t="n">
+      <c r="AI7" s="15" t="inlineStr"/>
+      <c r="AJ7" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="AK7" s="16" t="n">
+      <c r="AK7" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="AL7" s="16" t="n">
+      <c r="AL7" s="15" t="n">
         <v>0.4</v>
       </c>
-      <c r="AM7" s="17" t="inlineStr"/>
-      <c r="AN7" s="17" t="inlineStr"/>
-      <c r="AO7" s="17" t="inlineStr"/>
-      <c r="AP7" s="17" t="inlineStr"/>
-      <c r="AQ7" s="17" t="inlineStr"/>
-      <c r="AR7" s="17" t="inlineStr"/>
-      <c r="AS7" s="18" t="inlineStr"/>
-      <c r="AT7" s="18" t="inlineStr"/>
-      <c r="AU7" s="18" t="inlineStr"/>
-      <c r="AV7" s="18" t="inlineStr"/>
-      <c r="AW7" s="18" t="inlineStr"/>
-      <c r="AX7" s="18" t="inlineStr"/>
-      <c r="AY7" s="19" t="inlineStr"/>
-      <c r="AZ7" s="19" t="inlineStr"/>
-      <c r="BA7" s="19" t="inlineStr"/>
-      <c r="BB7" s="19" t="inlineStr"/>
-      <c r="BC7" s="19" t="inlineStr"/>
-      <c r="BD7" s="19" t="inlineStr"/>
-      <c r="BE7" s="19" t="inlineStr"/>
-      <c r="BF7" s="20" t="inlineStr"/>
-      <c r="BG7" s="20" t="inlineStr"/>
-      <c r="BH7" s="20" t="inlineStr"/>
-      <c r="BI7" s="20" t="inlineStr"/>
-      <c r="BJ7" s="20" t="inlineStr"/>
-      <c r="BK7" s="20" t="inlineStr"/>
-      <c r="BL7" s="20" t="inlineStr"/>
+      <c r="AM7" s="16" t="inlineStr"/>
+      <c r="AN7" s="16" t="inlineStr"/>
+      <c r="AO7" s="16" t="inlineStr"/>
+      <c r="AP7" s="16" t="inlineStr"/>
+      <c r="AQ7" s="16" t="inlineStr"/>
+      <c r="AR7" s="16" t="inlineStr"/>
+      <c r="AS7" s="17" t="inlineStr"/>
+      <c r="AT7" s="17" t="inlineStr"/>
+      <c r="AU7" s="17" t="inlineStr"/>
+      <c r="AV7" s="17" t="inlineStr"/>
+      <c r="AW7" s="17" t="inlineStr"/>
+      <c r="AX7" s="17" t="inlineStr"/>
+      <c r="AY7" s="18" t="inlineStr"/>
+      <c r="AZ7" s="18" t="inlineStr"/>
+      <c r="BA7" s="18" t="inlineStr"/>
+      <c r="BB7" s="18" t="inlineStr"/>
+      <c r="BC7" s="18" t="inlineStr"/>
+      <c r="BD7" s="18" t="inlineStr"/>
+      <c r="BE7" s="18" t="inlineStr"/>
+      <c r="BF7" s="19" t="inlineStr"/>
+      <c r="BG7" s="19" t="inlineStr"/>
+      <c r="BH7" s="19" t="inlineStr"/>
+      <c r="BI7" s="19" t="inlineStr"/>
+      <c r="BJ7" s="19" t="inlineStr"/>
+      <c r="BK7" s="19" t="inlineStr"/>
+      <c r="BL7" s="19" t="inlineStr"/>
       <c r="BM7" t="n">
         <v>0.18</v>
       </c>
@@ -1742,6 +1768,11 @@
           <t>TESTE</t>
         </is>
       </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>BBB</t>
+        </is>
+      </c>
       <c r="G8" t="inlineStr">
         <is>
           <t>Hidrologia</t>
@@ -1771,59 +1802,59 @@
       <c r="M8" t="n">
         <v>1</v>
       </c>
-      <c r="N8" s="12" t="n">
+      <c r="N8" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="O8" s="13" t="inlineStr"/>
-      <c r="P8" s="13" t="inlineStr"/>
-      <c r="Q8" s="13" t="inlineStr"/>
-      <c r="R8" s="13" t="inlineStr"/>
-      <c r="S8" s="13" t="inlineStr"/>
-      <c r="T8" s="13" t="inlineStr"/>
-      <c r="U8" s="14" t="inlineStr"/>
-      <c r="V8" s="14" t="inlineStr"/>
-      <c r="W8" s="14" t="inlineStr"/>
-      <c r="X8" s="14" t="inlineStr"/>
-      <c r="Y8" s="14" t="inlineStr"/>
-      <c r="Z8" s="14" t="inlineStr"/>
-      <c r="AA8" s="15" t="inlineStr"/>
-      <c r="AB8" s="15" t="inlineStr"/>
-      <c r="AC8" s="15" t="inlineStr"/>
-      <c r="AD8" s="15" t="inlineStr"/>
-      <c r="AE8" s="15" t="inlineStr"/>
-      <c r="AF8" s="15" t="inlineStr"/>
-      <c r="AG8" s="16" t="inlineStr"/>
-      <c r="AH8" s="16" t="inlineStr"/>
-      <c r="AI8" s="16" t="inlineStr"/>
-      <c r="AJ8" s="16" t="inlineStr"/>
-      <c r="AK8" s="16" t="inlineStr"/>
-      <c r="AL8" s="16" t="inlineStr"/>
-      <c r="AM8" s="17" t="inlineStr"/>
-      <c r="AN8" s="17" t="inlineStr"/>
-      <c r="AO8" s="17" t="inlineStr"/>
-      <c r="AP8" s="17" t="inlineStr"/>
-      <c r="AQ8" s="17" t="inlineStr"/>
-      <c r="AR8" s="17" t="inlineStr"/>
-      <c r="AS8" s="18" t="inlineStr"/>
-      <c r="AT8" s="18" t="inlineStr"/>
-      <c r="AU8" s="18" t="inlineStr"/>
-      <c r="AV8" s="18" t="inlineStr"/>
-      <c r="AW8" s="18" t="inlineStr"/>
-      <c r="AX8" s="18" t="inlineStr"/>
-      <c r="AY8" s="19" t="inlineStr"/>
-      <c r="AZ8" s="19" t="inlineStr"/>
-      <c r="BA8" s="19" t="inlineStr"/>
-      <c r="BB8" s="19" t="inlineStr"/>
-      <c r="BC8" s="19" t="inlineStr"/>
-      <c r="BD8" s="19" t="inlineStr"/>
-      <c r="BE8" s="19" t="inlineStr"/>
-      <c r="BF8" s="20" t="inlineStr"/>
-      <c r="BG8" s="20" t="inlineStr"/>
-      <c r="BH8" s="20" t="inlineStr"/>
-      <c r="BI8" s="20" t="inlineStr"/>
-      <c r="BJ8" s="20" t="inlineStr"/>
-      <c r="BK8" s="20" t="inlineStr"/>
-      <c r="BL8" s="20" t="inlineStr"/>
+      <c r="O8" s="12" t="inlineStr"/>
+      <c r="P8" s="12" t="inlineStr"/>
+      <c r="Q8" s="12" t="inlineStr"/>
+      <c r="R8" s="12" t="inlineStr"/>
+      <c r="S8" s="12" t="inlineStr"/>
+      <c r="T8" s="12" t="inlineStr"/>
+      <c r="U8" s="13" t="inlineStr"/>
+      <c r="V8" s="13" t="inlineStr"/>
+      <c r="W8" s="13" t="inlineStr"/>
+      <c r="X8" s="13" t="inlineStr"/>
+      <c r="Y8" s="13" t="inlineStr"/>
+      <c r="Z8" s="13" t="inlineStr"/>
+      <c r="AA8" s="14" t="inlineStr"/>
+      <c r="AB8" s="14" t="inlineStr"/>
+      <c r="AC8" s="14" t="inlineStr"/>
+      <c r="AD8" s="14" t="inlineStr"/>
+      <c r="AE8" s="14" t="inlineStr"/>
+      <c r="AF8" s="14" t="inlineStr"/>
+      <c r="AG8" s="15" t="inlineStr"/>
+      <c r="AH8" s="15" t="inlineStr"/>
+      <c r="AI8" s="15" t="inlineStr"/>
+      <c r="AJ8" s="15" t="inlineStr"/>
+      <c r="AK8" s="15" t="inlineStr"/>
+      <c r="AL8" s="15" t="inlineStr"/>
+      <c r="AM8" s="16" t="inlineStr"/>
+      <c r="AN8" s="16" t="inlineStr"/>
+      <c r="AO8" s="16" t="inlineStr"/>
+      <c r="AP8" s="16" t="inlineStr"/>
+      <c r="AQ8" s="16" t="inlineStr"/>
+      <c r="AR8" s="16" t="inlineStr"/>
+      <c r="AS8" s="17" t="inlineStr"/>
+      <c r="AT8" s="17" t="inlineStr"/>
+      <c r="AU8" s="17" t="inlineStr"/>
+      <c r="AV8" s="17" t="inlineStr"/>
+      <c r="AW8" s="17" t="inlineStr"/>
+      <c r="AX8" s="17" t="inlineStr"/>
+      <c r="AY8" s="18" t="inlineStr"/>
+      <c r="AZ8" s="18" t="inlineStr"/>
+      <c r="BA8" s="18" t="inlineStr"/>
+      <c r="BB8" s="18" t="inlineStr"/>
+      <c r="BC8" s="18" t="inlineStr"/>
+      <c r="BD8" s="18" t="inlineStr"/>
+      <c r="BE8" s="18" t="inlineStr"/>
+      <c r="BF8" s="19" t="inlineStr"/>
+      <c r="BG8" s="19" t="inlineStr"/>
+      <c r="BH8" s="19" t="inlineStr"/>
+      <c r="BI8" s="19" t="inlineStr"/>
+      <c r="BJ8" s="19" t="inlineStr"/>
+      <c r="BK8" s="19" t="inlineStr"/>
+      <c r="BL8" s="19" t="inlineStr"/>
       <c r="BM8" t="n">
         <v>0.2</v>
       </c>
@@ -1862,6 +1893,11 @@
           <t>TESTE</t>
         </is>
       </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>BBB</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr">
         <is>
           <t>Hidrologia</t>
@@ -1891,95 +1927,95 @@
       <c r="M9" t="n">
         <v>0.1</v>
       </c>
-      <c r="N9" s="12" t="n">
+      <c r="N9" s="11" t="n">
         <v>0.5900000000000001</v>
       </c>
-      <c r="O9" s="13" t="n">
+      <c r="O9" s="12" t="n">
         <v>0.4</v>
       </c>
-      <c r="P9" s="13" t="n">
+      <c r="P9" s="12" t="n">
         <v>80</v>
       </c>
-      <c r="Q9" s="13" t="n">
+      <c r="Q9" s="12" t="n">
         <v>100</v>
       </c>
-      <c r="R9" s="13" t="n">
+      <c r="R9" s="12" t="n">
         <v>0.8</v>
       </c>
-      <c r="S9" s="13" t="n">
+      <c r="S9" s="12" t="n">
         <v>0.8</v>
       </c>
-      <c r="T9" s="13" t="n">
+      <c r="T9" s="12" t="n">
         <v>0.3200000000000001</v>
       </c>
-      <c r="U9" s="14" t="n">
+      <c r="U9" s="13" t="n">
         <v>0.3</v>
       </c>
-      <c r="V9" s="14" t="n">
+      <c r="V9" s="13" t="n">
         <v>30</v>
       </c>
-      <c r="W9" s="14" t="n">
+      <c r="W9" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="X9" s="14" t="n">
+      <c r="X9" s="13" t="n">
         <v>0.3</v>
       </c>
-      <c r="Y9" s="14" t="n">
+      <c r="Y9" s="13" t="n">
         <v>0.3</v>
       </c>
-      <c r="Z9" s="14" t="n">
+      <c r="Z9" s="13" t="n">
         <v>0.09</v>
       </c>
-      <c r="AA9" s="15" t="inlineStr"/>
-      <c r="AB9" s="15" t="inlineStr"/>
-      <c r="AC9" s="15" t="inlineStr"/>
-      <c r="AD9" s="15" t="inlineStr"/>
-      <c r="AE9" s="15" t="inlineStr"/>
-      <c r="AF9" s="15" t="inlineStr"/>
-      <c r="AG9" s="16" t="inlineStr"/>
-      <c r="AH9" s="16" t="inlineStr"/>
-      <c r="AI9" s="16" t="inlineStr"/>
-      <c r="AJ9" s="16" t="inlineStr"/>
-      <c r="AK9" s="16" t="inlineStr"/>
-      <c r="AL9" s="16" t="inlineStr"/>
-      <c r="AM9" s="17" t="n">
+      <c r="AA9" s="14" t="inlineStr"/>
+      <c r="AB9" s="14" t="inlineStr"/>
+      <c r="AC9" s="14" t="inlineStr"/>
+      <c r="AD9" s="14" t="inlineStr"/>
+      <c r="AE9" s="14" t="inlineStr"/>
+      <c r="AF9" s="14" t="inlineStr"/>
+      <c r="AG9" s="15" t="inlineStr"/>
+      <c r="AH9" s="15" t="inlineStr"/>
+      <c r="AI9" s="15" t="inlineStr"/>
+      <c r="AJ9" s="15" t="inlineStr"/>
+      <c r="AK9" s="15" t="inlineStr"/>
+      <c r="AL9" s="15" t="inlineStr"/>
+      <c r="AM9" s="16" t="n">
         <v>0.3</v>
       </c>
-      <c r="AN9" s="17" t="n">
+      <c r="AN9" s="16" t="n">
         <v>0.3</v>
       </c>
-      <c r="AO9" s="17" t="n">
+      <c r="AO9" s="16" t="n">
         <v>0.5</v>
       </c>
-      <c r="AP9" s="17" t="n">
+      <c r="AP9" s="16" t="n">
         <v>0.6</v>
       </c>
-      <c r="AQ9" s="17" t="n">
+      <c r="AQ9" s="16" t="n">
         <v>0.6</v>
       </c>
-      <c r="AR9" s="17" t="n">
+      <c r="AR9" s="16" t="n">
         <v>0.18</v>
       </c>
-      <c r="AS9" s="18" t="inlineStr"/>
-      <c r="AT9" s="18" t="inlineStr"/>
-      <c r="AU9" s="18" t="inlineStr"/>
-      <c r="AV9" s="18" t="inlineStr"/>
-      <c r="AW9" s="18" t="inlineStr"/>
-      <c r="AX9" s="18" t="inlineStr"/>
-      <c r="AY9" s="19" t="inlineStr"/>
-      <c r="AZ9" s="19" t="inlineStr"/>
-      <c r="BA9" s="19" t="inlineStr"/>
-      <c r="BB9" s="19" t="inlineStr"/>
-      <c r="BC9" s="19" t="inlineStr"/>
-      <c r="BD9" s="19" t="inlineStr"/>
-      <c r="BE9" s="19" t="inlineStr"/>
-      <c r="BF9" s="20" t="inlineStr"/>
-      <c r="BG9" s="20" t="inlineStr"/>
-      <c r="BH9" s="20" t="inlineStr"/>
-      <c r="BI9" s="20" t="inlineStr"/>
-      <c r="BJ9" s="20" t="inlineStr"/>
-      <c r="BK9" s="20" t="inlineStr"/>
-      <c r="BL9" s="20" t="inlineStr"/>
+      <c r="AS9" s="17" t="inlineStr"/>
+      <c r="AT9" s="17" t="inlineStr"/>
+      <c r="AU9" s="17" t="inlineStr"/>
+      <c r="AV9" s="17" t="inlineStr"/>
+      <c r="AW9" s="17" t="inlineStr"/>
+      <c r="AX9" s="17" t="inlineStr"/>
+      <c r="AY9" s="18" t="inlineStr"/>
+      <c r="AZ9" s="18" t="inlineStr"/>
+      <c r="BA9" s="18" t="inlineStr"/>
+      <c r="BB9" s="18" t="inlineStr"/>
+      <c r="BC9" s="18" t="inlineStr"/>
+      <c r="BD9" s="18" t="inlineStr"/>
+      <c r="BE9" s="18" t="inlineStr"/>
+      <c r="BF9" s="19" t="inlineStr"/>
+      <c r="BG9" s="19" t="inlineStr"/>
+      <c r="BH9" s="19" t="inlineStr"/>
+      <c r="BI9" s="19" t="inlineStr"/>
+      <c r="BJ9" s="19" t="inlineStr"/>
+      <c r="BK9" s="19" t="inlineStr"/>
+      <c r="BL9" s="19" t="inlineStr"/>
       <c r="BM9" t="n">
         <v>0.08000000000000002</v>
       </c>
@@ -2013,6 +2049,11 @@
           <t>TESTE</t>
         </is>
       </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>BBB</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr">
         <is>
           <t>Hidrologia</t>
@@ -2042,95 +2083,95 @@
       <c r="M10" t="n">
         <v>0.2</v>
       </c>
-      <c r="N10" s="12" t="n">
+      <c r="N10" s="11" t="n">
         <v>0.54</v>
       </c>
-      <c r="O10" s="13" t="n">
+      <c r="O10" s="12" t="n">
         <v>0.3</v>
       </c>
-      <c r="P10" s="13" t="n">
+      <c r="P10" s="12" t="n">
         <v>80</v>
       </c>
-      <c r="Q10" s="13" t="n">
+      <c r="Q10" s="12" t="n">
         <v>100</v>
       </c>
-      <c r="R10" s="13" t="n">
+      <c r="R10" s="12" t="n">
         <v>0.8</v>
       </c>
-      <c r="S10" s="13" t="n">
+      <c r="S10" s="12" t="n">
         <v>0.8</v>
       </c>
-      <c r="T10" s="13" t="n">
+      <c r="T10" s="12" t="n">
         <v>0.24</v>
       </c>
-      <c r="U10" s="14" t="n">
+      <c r="U10" s="13" t="n">
         <v>0.4</v>
       </c>
-      <c r="V10" s="14" t="n">
+      <c r="V10" s="13" t="n">
         <v>30</v>
       </c>
-      <c r="W10" s="14" t="n">
+      <c r="W10" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="X10" s="14" t="n">
+      <c r="X10" s="13" t="n">
         <v>0.3</v>
       </c>
-      <c r="Y10" s="14" t="n">
+      <c r="Y10" s="13" t="n">
         <v>0.3</v>
       </c>
-      <c r="Z10" s="14" t="n">
+      <c r="Z10" s="13" t="n">
         <v>0.12</v>
       </c>
-      <c r="AA10" s="15" t="inlineStr"/>
-      <c r="AB10" s="15" t="inlineStr"/>
-      <c r="AC10" s="15" t="inlineStr"/>
-      <c r="AD10" s="15" t="inlineStr"/>
-      <c r="AE10" s="15" t="inlineStr"/>
-      <c r="AF10" s="15" t="inlineStr"/>
-      <c r="AG10" s="16" t="inlineStr"/>
-      <c r="AH10" s="16" t="inlineStr"/>
-      <c r="AI10" s="16" t="inlineStr"/>
-      <c r="AJ10" s="16" t="inlineStr"/>
-      <c r="AK10" s="16" t="inlineStr"/>
-      <c r="AL10" s="16" t="inlineStr"/>
-      <c r="AM10" s="17" t="n">
+      <c r="AA10" s="14" t="inlineStr"/>
+      <c r="AB10" s="14" t="inlineStr"/>
+      <c r="AC10" s="14" t="inlineStr"/>
+      <c r="AD10" s="14" t="inlineStr"/>
+      <c r="AE10" s="14" t="inlineStr"/>
+      <c r="AF10" s="14" t="inlineStr"/>
+      <c r="AG10" s="15" t="inlineStr"/>
+      <c r="AH10" s="15" t="inlineStr"/>
+      <c r="AI10" s="15" t="inlineStr"/>
+      <c r="AJ10" s="15" t="inlineStr"/>
+      <c r="AK10" s="15" t="inlineStr"/>
+      <c r="AL10" s="15" t="inlineStr"/>
+      <c r="AM10" s="16" t="n">
         <v>0.3</v>
       </c>
-      <c r="AN10" s="17" t="n">
+      <c r="AN10" s="16" t="n">
         <v>0.3</v>
       </c>
-      <c r="AO10" s="17" t="n">
+      <c r="AO10" s="16" t="n">
         <v>0.5</v>
       </c>
-      <c r="AP10" s="17" t="n">
+      <c r="AP10" s="16" t="n">
         <v>0.6</v>
       </c>
-      <c r="AQ10" s="17" t="n">
+      <c r="AQ10" s="16" t="n">
         <v>0.6</v>
       </c>
-      <c r="AR10" s="17" t="n">
+      <c r="AR10" s="16" t="n">
         <v>0.18</v>
       </c>
-      <c r="AS10" s="18" t="inlineStr"/>
-      <c r="AT10" s="18" t="inlineStr"/>
-      <c r="AU10" s="18" t="inlineStr"/>
-      <c r="AV10" s="18" t="inlineStr"/>
-      <c r="AW10" s="18" t="inlineStr"/>
-      <c r="AX10" s="18" t="inlineStr"/>
-      <c r="AY10" s="19" t="inlineStr"/>
-      <c r="AZ10" s="19" t="inlineStr"/>
-      <c r="BA10" s="19" t="inlineStr"/>
-      <c r="BB10" s="19" t="inlineStr"/>
-      <c r="BC10" s="19" t="inlineStr"/>
-      <c r="BD10" s="19" t="inlineStr"/>
-      <c r="BE10" s="19" t="inlineStr"/>
-      <c r="BF10" s="20" t="inlineStr"/>
-      <c r="BG10" s="20" t="inlineStr"/>
-      <c r="BH10" s="20" t="inlineStr"/>
-      <c r="BI10" s="20" t="inlineStr"/>
-      <c r="BJ10" s="20" t="inlineStr"/>
-      <c r="BK10" s="20" t="inlineStr"/>
-      <c r="BL10" s="20" t="inlineStr"/>
+      <c r="AS10" s="17" t="inlineStr"/>
+      <c r="AT10" s="17" t="inlineStr"/>
+      <c r="AU10" s="17" t="inlineStr"/>
+      <c r="AV10" s="17" t="inlineStr"/>
+      <c r="AW10" s="17" t="inlineStr"/>
+      <c r="AX10" s="17" t="inlineStr"/>
+      <c r="AY10" s="18" t="inlineStr"/>
+      <c r="AZ10" s="18" t="inlineStr"/>
+      <c r="BA10" s="18" t="inlineStr"/>
+      <c r="BB10" s="18" t="inlineStr"/>
+      <c r="BC10" s="18" t="inlineStr"/>
+      <c r="BD10" s="18" t="inlineStr"/>
+      <c r="BE10" s="18" t="inlineStr"/>
+      <c r="BF10" s="19" t="inlineStr"/>
+      <c r="BG10" s="19" t="inlineStr"/>
+      <c r="BH10" s="19" t="inlineStr"/>
+      <c r="BI10" s="19" t="inlineStr"/>
+      <c r="BJ10" s="19" t="inlineStr"/>
+      <c r="BK10" s="19" t="inlineStr"/>
+      <c r="BL10" s="19" t="inlineStr"/>
       <c r="BM10" t="n">
         <v>0.16</v>
       </c>
@@ -2164,6 +2205,11 @@
           <t>TESTE</t>
         </is>
       </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>BBB</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr">
         <is>
           <t>Hidrologia</t>
@@ -2193,95 +2239,95 @@
       <c r="M11" t="n">
         <v>0.2</v>
       </c>
-      <c r="N11" s="12" t="n">
+      <c r="N11" s="11" t="n">
         <v>0.5600000000000001</v>
       </c>
-      <c r="O11" s="13" t="n">
+      <c r="O11" s="12" t="n">
         <v>0.4</v>
       </c>
-      <c r="P11" s="13" t="n">
+      <c r="P11" s="12" t="n">
         <v>80</v>
       </c>
-      <c r="Q11" s="13" t="n">
+      <c r="Q11" s="12" t="n">
         <v>100</v>
       </c>
-      <c r="R11" s="13" t="n">
+      <c r="R11" s="12" t="n">
         <v>0.8</v>
       </c>
-      <c r="S11" s="13" t="n">
+      <c r="S11" s="12" t="n">
         <v>0.8</v>
       </c>
-      <c r="T11" s="13" t="n">
+      <c r="T11" s="12" t="n">
         <v>0.3200000000000001</v>
       </c>
-      <c r="U11" s="14" t="n">
+      <c r="U11" s="13" t="n">
         <v>0.4</v>
       </c>
-      <c r="V11" s="14" t="n">
+      <c r="V11" s="13" t="n">
         <v>30</v>
       </c>
-      <c r="W11" s="14" t="n">
+      <c r="W11" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="X11" s="14" t="n">
+      <c r="X11" s="13" t="n">
         <v>0.3</v>
       </c>
-      <c r="Y11" s="14" t="n">
+      <c r="Y11" s="13" t="n">
         <v>0.3</v>
       </c>
-      <c r="Z11" s="14" t="n">
+      <c r="Z11" s="13" t="n">
         <v>0.12</v>
       </c>
-      <c r="AA11" s="15" t="inlineStr"/>
-      <c r="AB11" s="15" t="inlineStr"/>
-      <c r="AC11" s="15" t="inlineStr"/>
-      <c r="AD11" s="15" t="inlineStr"/>
-      <c r="AE11" s="15" t="inlineStr"/>
-      <c r="AF11" s="15" t="inlineStr"/>
-      <c r="AG11" s="16" t="inlineStr"/>
-      <c r="AH11" s="16" t="inlineStr"/>
-      <c r="AI11" s="16" t="inlineStr"/>
-      <c r="AJ11" s="16" t="inlineStr"/>
-      <c r="AK11" s="16" t="inlineStr"/>
-      <c r="AL11" s="16" t="inlineStr"/>
-      <c r="AM11" s="17" t="n">
+      <c r="AA11" s="14" t="inlineStr"/>
+      <c r="AB11" s="14" t="inlineStr"/>
+      <c r="AC11" s="14" t="inlineStr"/>
+      <c r="AD11" s="14" t="inlineStr"/>
+      <c r="AE11" s="14" t="inlineStr"/>
+      <c r="AF11" s="14" t="inlineStr"/>
+      <c r="AG11" s="15" t="inlineStr"/>
+      <c r="AH11" s="15" t="inlineStr"/>
+      <c r="AI11" s="15" t="inlineStr"/>
+      <c r="AJ11" s="15" t="inlineStr"/>
+      <c r="AK11" s="15" t="inlineStr"/>
+      <c r="AL11" s="15" t="inlineStr"/>
+      <c r="AM11" s="16" t="n">
         <v>0.2</v>
       </c>
-      <c r="AN11" s="17" t="n">
+      <c r="AN11" s="16" t="n">
         <v>0.3</v>
       </c>
-      <c r="AO11" s="17" t="n">
+      <c r="AO11" s="16" t="n">
         <v>0.5</v>
       </c>
-      <c r="AP11" s="17" t="n">
+      <c r="AP11" s="16" t="n">
         <v>0.6</v>
       </c>
-      <c r="AQ11" s="17" t="n">
+      <c r="AQ11" s="16" t="n">
         <v>0.6</v>
       </c>
-      <c r="AR11" s="17" t="n">
+      <c r="AR11" s="16" t="n">
         <v>0.12</v>
       </c>
-      <c r="AS11" s="18" t="inlineStr"/>
-      <c r="AT11" s="18" t="inlineStr"/>
-      <c r="AU11" s="18" t="inlineStr"/>
-      <c r="AV11" s="18" t="inlineStr"/>
-      <c r="AW11" s="18" t="inlineStr"/>
-      <c r="AX11" s="18" t="inlineStr"/>
-      <c r="AY11" s="19" t="inlineStr"/>
-      <c r="AZ11" s="19" t="inlineStr"/>
-      <c r="BA11" s="19" t="inlineStr"/>
-      <c r="BB11" s="19" t="inlineStr"/>
-      <c r="BC11" s="19" t="inlineStr"/>
-      <c r="BD11" s="19" t="inlineStr"/>
-      <c r="BE11" s="19" t="inlineStr"/>
-      <c r="BF11" s="20" t="inlineStr"/>
-      <c r="BG11" s="20" t="inlineStr"/>
-      <c r="BH11" s="20" t="inlineStr"/>
-      <c r="BI11" s="20" t="inlineStr"/>
-      <c r="BJ11" s="20" t="inlineStr"/>
-      <c r="BK11" s="20" t="inlineStr"/>
-      <c r="BL11" s="20" t="inlineStr"/>
+      <c r="AS11" s="17" t="inlineStr"/>
+      <c r="AT11" s="17" t="inlineStr"/>
+      <c r="AU11" s="17" t="inlineStr"/>
+      <c r="AV11" s="17" t="inlineStr"/>
+      <c r="AW11" s="17" t="inlineStr"/>
+      <c r="AX11" s="17" t="inlineStr"/>
+      <c r="AY11" s="18" t="inlineStr"/>
+      <c r="AZ11" s="18" t="inlineStr"/>
+      <c r="BA11" s="18" t="inlineStr"/>
+      <c r="BB11" s="18" t="inlineStr"/>
+      <c r="BC11" s="18" t="inlineStr"/>
+      <c r="BD11" s="18" t="inlineStr"/>
+      <c r="BE11" s="18" t="inlineStr"/>
+      <c r="BF11" s="19" t="inlineStr"/>
+      <c r="BG11" s="19" t="inlineStr"/>
+      <c r="BH11" s="19" t="inlineStr"/>
+      <c r="BI11" s="19" t="inlineStr"/>
+      <c r="BJ11" s="19" t="inlineStr"/>
+      <c r="BK11" s="19" t="inlineStr"/>
+      <c r="BL11" s="19" t="inlineStr"/>
       <c r="BM11" t="n">
         <v>0.16</v>
       </c>
@@ -2315,6 +2361,11 @@
           <t>TESTE</t>
         </is>
       </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>BBB</t>
+        </is>
+      </c>
       <c r="G12" t="inlineStr">
         <is>
           <t>Hidrologia</t>
@@ -2344,83 +2395,83 @@
       <c r="M12" t="n">
         <v>0.15</v>
       </c>
-      <c r="N12" s="12" t="n">
+      <c r="N12" s="11" t="n">
         <v>0.5</v>
       </c>
-      <c r="O12" s="13" t="inlineStr"/>
-      <c r="P12" s="13" t="inlineStr"/>
-      <c r="Q12" s="13" t="inlineStr"/>
-      <c r="R12" s="13" t="inlineStr"/>
-      <c r="S12" s="13" t="inlineStr"/>
-      <c r="T12" s="13" t="inlineStr"/>
-      <c r="U12" s="14" t="inlineStr"/>
-      <c r="V12" s="14" t="inlineStr"/>
-      <c r="W12" s="14" t="inlineStr"/>
-      <c r="X12" s="14" t="inlineStr"/>
-      <c r="Y12" s="14" t="inlineStr"/>
-      <c r="Z12" s="14" t="inlineStr"/>
-      <c r="AA12" s="15" t="n">
+      <c r="O12" s="12" t="inlineStr"/>
+      <c r="P12" s="12" t="inlineStr"/>
+      <c r="Q12" s="12" t="inlineStr"/>
+      <c r="R12" s="12" t="inlineStr"/>
+      <c r="S12" s="12" t="inlineStr"/>
+      <c r="T12" s="12" t="inlineStr"/>
+      <c r="U12" s="13" t="inlineStr"/>
+      <c r="V12" s="13" t="inlineStr"/>
+      <c r="W12" s="13" t="inlineStr"/>
+      <c r="X12" s="13" t="inlineStr"/>
+      <c r="Y12" s="13" t="inlineStr"/>
+      <c r="Z12" s="13" t="inlineStr"/>
+      <c r="AA12" s="14" t="n">
         <v>0.4</v>
       </c>
-      <c r="AB12" s="15" t="n">
+      <c r="AB12" s="14" t="n">
         <v>80</v>
       </c>
-      <c r="AC12" s="15" t="n">
+      <c r="AC12" s="14" t="n">
         <v>100</v>
       </c>
-      <c r="AD12" s="15" t="n">
+      <c r="AD12" s="14" t="n">
         <v>0.8</v>
       </c>
-      <c r="AE12" s="15" t="n">
+      <c r="AE12" s="14" t="n">
         <v>0.8</v>
       </c>
-      <c r="AF12" s="15" t="n">
+      <c r="AF12" s="14" t="n">
         <v>0.3200000000000001</v>
       </c>
-      <c r="AG12" s="16" t="n">
+      <c r="AG12" s="15" t="n">
         <v>0.6</v>
       </c>
-      <c r="AH12" s="16" t="n">
+      <c r="AH12" s="15" t="n">
         <v>30</v>
       </c>
-      <c r="AI12" s="16" t="n">
+      <c r="AI12" s="15" t="n">
         <v>100</v>
       </c>
-      <c r="AJ12" s="16" t="n">
+      <c r="AJ12" s="15" t="n">
         <v>0.3</v>
       </c>
-      <c r="AK12" s="16" t="n">
+      <c r="AK12" s="15" t="n">
         <v>0.3</v>
       </c>
-      <c r="AL12" s="16" t="n">
+      <c r="AL12" s="15" t="n">
         <v>0.18</v>
       </c>
-      <c r="AM12" s="17" t="inlineStr"/>
-      <c r="AN12" s="17" t="inlineStr"/>
-      <c r="AO12" s="17" t="inlineStr"/>
-      <c r="AP12" s="17" t="inlineStr"/>
-      <c r="AQ12" s="17" t="inlineStr"/>
-      <c r="AR12" s="17" t="inlineStr"/>
-      <c r="AS12" s="18" t="inlineStr"/>
-      <c r="AT12" s="18" t="inlineStr"/>
-      <c r="AU12" s="18" t="inlineStr"/>
-      <c r="AV12" s="18" t="inlineStr"/>
-      <c r="AW12" s="18" t="inlineStr"/>
-      <c r="AX12" s="18" t="inlineStr"/>
-      <c r="AY12" s="19" t="inlineStr"/>
-      <c r="AZ12" s="19" t="inlineStr"/>
-      <c r="BA12" s="19" t="inlineStr"/>
-      <c r="BB12" s="19" t="inlineStr"/>
-      <c r="BC12" s="19" t="inlineStr"/>
-      <c r="BD12" s="19" t="inlineStr"/>
-      <c r="BE12" s="19" t="inlineStr"/>
-      <c r="BF12" s="20" t="inlineStr"/>
-      <c r="BG12" s="20" t="inlineStr"/>
-      <c r="BH12" s="20" t="inlineStr"/>
-      <c r="BI12" s="20" t="inlineStr"/>
-      <c r="BJ12" s="20" t="inlineStr"/>
-      <c r="BK12" s="20" t="inlineStr"/>
-      <c r="BL12" s="20" t="inlineStr"/>
+      <c r="AM12" s="16" t="inlineStr"/>
+      <c r="AN12" s="16" t="inlineStr"/>
+      <c r="AO12" s="16" t="inlineStr"/>
+      <c r="AP12" s="16" t="inlineStr"/>
+      <c r="AQ12" s="16" t="inlineStr"/>
+      <c r="AR12" s="16" t="inlineStr"/>
+      <c r="AS12" s="17" t="inlineStr"/>
+      <c r="AT12" s="17" t="inlineStr"/>
+      <c r="AU12" s="17" t="inlineStr"/>
+      <c r="AV12" s="17" t="inlineStr"/>
+      <c r="AW12" s="17" t="inlineStr"/>
+      <c r="AX12" s="17" t="inlineStr"/>
+      <c r="AY12" s="18" t="inlineStr"/>
+      <c r="AZ12" s="18" t="inlineStr"/>
+      <c r="BA12" s="18" t="inlineStr"/>
+      <c r="BB12" s="18" t="inlineStr"/>
+      <c r="BC12" s="18" t="inlineStr"/>
+      <c r="BD12" s="18" t="inlineStr"/>
+      <c r="BE12" s="18" t="inlineStr"/>
+      <c r="BF12" s="19" t="inlineStr"/>
+      <c r="BG12" s="19" t="inlineStr"/>
+      <c r="BH12" s="19" t="inlineStr"/>
+      <c r="BI12" s="19" t="inlineStr"/>
+      <c r="BJ12" s="19" t="inlineStr"/>
+      <c r="BK12" s="19" t="inlineStr"/>
+      <c r="BL12" s="19" t="inlineStr"/>
       <c r="BM12" t="n">
         <v>0.12</v>
       </c>
@@ -2454,6 +2505,11 @@
           <t>TESTE</t>
         </is>
       </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>BBB</t>
+        </is>
+      </c>
       <c r="G13" t="inlineStr">
         <is>
           <t>Hidrologia</t>
@@ -2483,79 +2539,79 @@
       <c r="M13" t="n">
         <v>0.15</v>
       </c>
-      <c r="N13" s="12" t="n">
+      <c r="N13" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="O13" s="13" t="inlineStr"/>
-      <c r="P13" s="13" t="inlineStr"/>
-      <c r="Q13" s="13" t="inlineStr"/>
-      <c r="R13" s="13" t="inlineStr"/>
-      <c r="S13" s="13" t="inlineStr"/>
-      <c r="T13" s="13" t="inlineStr"/>
-      <c r="U13" s="14" t="inlineStr"/>
-      <c r="V13" s="14" t="inlineStr"/>
-      <c r="W13" s="14" t="inlineStr"/>
-      <c r="X13" s="14" t="inlineStr"/>
-      <c r="Y13" s="14" t="inlineStr"/>
-      <c r="Z13" s="14" t="inlineStr"/>
-      <c r="AA13" s="15" t="n">
+      <c r="O13" s="12" t="inlineStr"/>
+      <c r="P13" s="12" t="inlineStr"/>
+      <c r="Q13" s="12" t="inlineStr"/>
+      <c r="R13" s="12" t="inlineStr"/>
+      <c r="S13" s="12" t="inlineStr"/>
+      <c r="T13" s="12" t="inlineStr"/>
+      <c r="U13" s="13" t="inlineStr"/>
+      <c r="V13" s="13" t="inlineStr"/>
+      <c r="W13" s="13" t="inlineStr"/>
+      <c r="X13" s="13" t="inlineStr"/>
+      <c r="Y13" s="13" t="inlineStr"/>
+      <c r="Z13" s="13" t="inlineStr"/>
+      <c r="AA13" s="14" t="n">
         <v>0.6</v>
       </c>
-      <c r="AB13" s="15" t="n">
+      <c r="AB13" s="14" t="n">
         <v>80</v>
       </c>
-      <c r="AC13" s="15" t="inlineStr"/>
-      <c r="AD13" s="15" t="n">
+      <c r="AC13" s="14" t="inlineStr"/>
+      <c r="AD13" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="AE13" s="15" t="n">
+      <c r="AE13" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="AF13" s="15" t="n">
+      <c r="AF13" s="14" t="n">
         <v>0.6</v>
       </c>
-      <c r="AG13" s="16" t="n">
+      <c r="AG13" s="15" t="n">
         <v>0.4</v>
       </c>
-      <c r="AH13" s="16" t="n">
+      <c r="AH13" s="15" t="n">
         <v>30</v>
       </c>
-      <c r="AI13" s="16" t="inlineStr"/>
-      <c r="AJ13" s="16" t="n">
+      <c r="AI13" s="15" t="inlineStr"/>
+      <c r="AJ13" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="AK13" s="16" t="n">
+      <c r="AK13" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="AL13" s="16" t="n">
+      <c r="AL13" s="15" t="n">
         <v>0.4</v>
       </c>
-      <c r="AM13" s="17" t="inlineStr"/>
-      <c r="AN13" s="17" t="inlineStr"/>
-      <c r="AO13" s="17" t="inlineStr"/>
-      <c r="AP13" s="17" t="inlineStr"/>
-      <c r="AQ13" s="17" t="inlineStr"/>
-      <c r="AR13" s="17" t="inlineStr"/>
-      <c r="AS13" s="18" t="inlineStr"/>
-      <c r="AT13" s="18" t="inlineStr"/>
-      <c r="AU13" s="18" t="inlineStr"/>
-      <c r="AV13" s="18" t="inlineStr"/>
-      <c r="AW13" s="18" t="inlineStr"/>
-      <c r="AX13" s="18" t="inlineStr"/>
-      <c r="AY13" s="19" t="inlineStr"/>
-      <c r="AZ13" s="19" t="inlineStr"/>
-      <c r="BA13" s="19" t="inlineStr"/>
-      <c r="BB13" s="19" t="inlineStr"/>
-      <c r="BC13" s="19" t="inlineStr"/>
-      <c r="BD13" s="19" t="inlineStr"/>
-      <c r="BE13" s="19" t="inlineStr"/>
-      <c r="BF13" s="20" t="inlineStr"/>
-      <c r="BG13" s="20" t="inlineStr"/>
-      <c r="BH13" s="20" t="inlineStr"/>
-      <c r="BI13" s="20" t="inlineStr"/>
-      <c r="BJ13" s="20" t="inlineStr"/>
-      <c r="BK13" s="20" t="inlineStr"/>
-      <c r="BL13" s="20" t="inlineStr"/>
+      <c r="AM13" s="16" t="inlineStr"/>
+      <c r="AN13" s="16" t="inlineStr"/>
+      <c r="AO13" s="16" t="inlineStr"/>
+      <c r="AP13" s="16" t="inlineStr"/>
+      <c r="AQ13" s="16" t="inlineStr"/>
+      <c r="AR13" s="16" t="inlineStr"/>
+      <c r="AS13" s="17" t="inlineStr"/>
+      <c r="AT13" s="17" t="inlineStr"/>
+      <c r="AU13" s="17" t="inlineStr"/>
+      <c r="AV13" s="17" t="inlineStr"/>
+      <c r="AW13" s="17" t="inlineStr"/>
+      <c r="AX13" s="17" t="inlineStr"/>
+      <c r="AY13" s="18" t="inlineStr"/>
+      <c r="AZ13" s="18" t="inlineStr"/>
+      <c r="BA13" s="18" t="inlineStr"/>
+      <c r="BB13" s="18" t="inlineStr"/>
+      <c r="BC13" s="18" t="inlineStr"/>
+      <c r="BD13" s="18" t="inlineStr"/>
+      <c r="BE13" s="18" t="inlineStr"/>
+      <c r="BF13" s="19" t="inlineStr"/>
+      <c r="BG13" s="19" t="inlineStr"/>
+      <c r="BH13" s="19" t="inlineStr"/>
+      <c r="BI13" s="19" t="inlineStr"/>
+      <c r="BJ13" s="19" t="inlineStr"/>
+      <c r="BK13" s="19" t="inlineStr"/>
+      <c r="BL13" s="19" t="inlineStr"/>
       <c r="BM13" t="n">
         <v>0.12</v>
       </c>
@@ -2589,6 +2645,11 @@
           <t>TESTE2</t>
         </is>
       </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>AAA</t>
+        </is>
+      </c>
       <c r="G14" t="inlineStr">
         <is>
           <t>Hidrologia</t>
@@ -2618,95 +2679,95 @@
       <c r="M14" t="n">
         <v>0.1</v>
       </c>
-      <c r="N14" s="12" t="n">
+      <c r="N14" s="11" t="n">
         <v>0.65</v>
       </c>
-      <c r="O14" s="13" t="n">
+      <c r="O14" s="12" t="n">
         <v>0.4</v>
       </c>
-      <c r="P14" s="13" t="n">
+      <c r="P14" s="12" t="n">
         <v>80</v>
       </c>
-      <c r="Q14" s="13" t="n">
+      <c r="Q14" s="12" t="n">
         <v>100</v>
       </c>
-      <c r="R14" s="13" t="n">
+      <c r="R14" s="12" t="n">
         <v>0.8</v>
       </c>
-      <c r="S14" s="13" t="n">
+      <c r="S14" s="12" t="n">
         <v>0.8</v>
       </c>
-      <c r="T14" s="13" t="n">
+      <c r="T14" s="12" t="n">
         <v>0.3200000000000001</v>
       </c>
-      <c r="U14" s="14" t="n">
+      <c r="U14" s="13" t="n">
         <v>0.3</v>
       </c>
-      <c r="V14" s="14" t="n">
+      <c r="V14" s="13" t="n">
         <v>30</v>
       </c>
-      <c r="W14" s="14" t="n">
+      <c r="W14" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="X14" s="14" t="n">
+      <c r="X14" s="13" t="n">
         <v>0.3</v>
       </c>
-      <c r="Y14" s="14" t="n">
+      <c r="Y14" s="13" t="n">
         <v>0.3</v>
       </c>
-      <c r="Z14" s="14" t="n">
+      <c r="Z14" s="13" t="n">
         <v>0.09</v>
       </c>
-      <c r="AA14" s="15" t="inlineStr"/>
-      <c r="AB14" s="15" t="inlineStr"/>
-      <c r="AC14" s="15" t="inlineStr"/>
-      <c r="AD14" s="15" t="inlineStr"/>
-      <c r="AE14" s="15" t="inlineStr"/>
-      <c r="AF14" s="15" t="inlineStr"/>
-      <c r="AG14" s="16" t="inlineStr"/>
-      <c r="AH14" s="16" t="inlineStr"/>
-      <c r="AI14" s="16" t="inlineStr"/>
-      <c r="AJ14" s="16" t="inlineStr"/>
-      <c r="AK14" s="16" t="inlineStr"/>
-      <c r="AL14" s="16" t="inlineStr"/>
-      <c r="AM14" s="17" t="n">
+      <c r="AA14" s="14" t="inlineStr"/>
+      <c r="AB14" s="14" t="inlineStr"/>
+      <c r="AC14" s="14" t="inlineStr"/>
+      <c r="AD14" s="14" t="inlineStr"/>
+      <c r="AE14" s="14" t="inlineStr"/>
+      <c r="AF14" s="14" t="inlineStr"/>
+      <c r="AG14" s="15" t="inlineStr"/>
+      <c r="AH14" s="15" t="inlineStr"/>
+      <c r="AI14" s="15" t="inlineStr"/>
+      <c r="AJ14" s="15" t="inlineStr"/>
+      <c r="AK14" s="15" t="inlineStr"/>
+      <c r="AL14" s="15" t="inlineStr"/>
+      <c r="AM14" s="16" t="n">
         <v>0.3</v>
       </c>
-      <c r="AN14" s="17" t="n">
+      <c r="AN14" s="16" t="n">
         <v>0.4</v>
       </c>
-      <c r="AO14" s="17" t="n">
+      <c r="AO14" s="16" t="n">
         <v>0.5</v>
       </c>
-      <c r="AP14" s="17" t="n">
+      <c r="AP14" s="16" t="n">
         <v>0.8</v>
       </c>
-      <c r="AQ14" s="17" t="n">
+      <c r="AQ14" s="16" t="n">
         <v>0.8</v>
       </c>
-      <c r="AR14" s="17" t="n">
+      <c r="AR14" s="16" t="n">
         <v>0.24</v>
       </c>
-      <c r="AS14" s="18" t="inlineStr"/>
-      <c r="AT14" s="18" t="inlineStr"/>
-      <c r="AU14" s="18" t="inlineStr"/>
-      <c r="AV14" s="18" t="inlineStr"/>
-      <c r="AW14" s="18" t="inlineStr"/>
-      <c r="AX14" s="18" t="inlineStr"/>
-      <c r="AY14" s="19" t="inlineStr"/>
-      <c r="AZ14" s="19" t="inlineStr"/>
-      <c r="BA14" s="19" t="inlineStr"/>
-      <c r="BB14" s="19" t="inlineStr"/>
-      <c r="BC14" s="19" t="inlineStr"/>
-      <c r="BD14" s="19" t="inlineStr"/>
-      <c r="BE14" s="19" t="inlineStr"/>
-      <c r="BF14" s="20" t="inlineStr"/>
-      <c r="BG14" s="20" t="inlineStr"/>
-      <c r="BH14" s="20" t="inlineStr"/>
-      <c r="BI14" s="20" t="inlineStr"/>
-      <c r="BJ14" s="20" t="inlineStr"/>
-      <c r="BK14" s="20" t="inlineStr"/>
-      <c r="BL14" s="20" t="inlineStr"/>
+      <c r="AS14" s="17" t="inlineStr"/>
+      <c r="AT14" s="17" t="inlineStr"/>
+      <c r="AU14" s="17" t="inlineStr"/>
+      <c r="AV14" s="17" t="inlineStr"/>
+      <c r="AW14" s="17" t="inlineStr"/>
+      <c r="AX14" s="17" t="inlineStr"/>
+      <c r="AY14" s="18" t="inlineStr"/>
+      <c r="AZ14" s="18" t="inlineStr"/>
+      <c r="BA14" s="18" t="inlineStr"/>
+      <c r="BB14" s="18" t="inlineStr"/>
+      <c r="BC14" s="18" t="inlineStr"/>
+      <c r="BD14" s="18" t="inlineStr"/>
+      <c r="BE14" s="18" t="inlineStr"/>
+      <c r="BF14" s="19" t="inlineStr"/>
+      <c r="BG14" s="19" t="inlineStr"/>
+      <c r="BH14" s="19" t="inlineStr"/>
+      <c r="BI14" s="19" t="inlineStr"/>
+      <c r="BJ14" s="19" t="inlineStr"/>
+      <c r="BK14" s="19" t="inlineStr"/>
+      <c r="BL14" s="19" t="inlineStr"/>
       <c r="BM14" t="n">
         <v>0.15</v>
       </c>
@@ -2735,6 +2796,11 @@
           <t>TESTE2</t>
         </is>
       </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>AAA</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr">
         <is>
           <t>Hidrologia</t>
@@ -2764,95 +2830,95 @@
       <c r="M15" t="n">
         <v>0.2</v>
       </c>
-      <c r="N15" s="12" t="n">
+      <c r="N15" s="11" t="n">
         <v>0.6</v>
       </c>
-      <c r="O15" s="13" t="n">
+      <c r="O15" s="12" t="n">
         <v>0.3</v>
       </c>
-      <c r="P15" s="13" t="n">
+      <c r="P15" s="12" t="n">
         <v>80</v>
       </c>
-      <c r="Q15" s="13" t="n">
+      <c r="Q15" s="12" t="n">
         <v>100</v>
       </c>
-      <c r="R15" s="13" t="n">
+      <c r="R15" s="12" t="n">
         <v>0.8</v>
       </c>
-      <c r="S15" s="13" t="n">
+      <c r="S15" s="12" t="n">
         <v>0.8</v>
       </c>
-      <c r="T15" s="13" t="n">
+      <c r="T15" s="12" t="n">
         <v>0.24</v>
       </c>
-      <c r="U15" s="14" t="n">
+      <c r="U15" s="13" t="n">
         <v>0.4</v>
       </c>
-      <c r="V15" s="14" t="n">
+      <c r="V15" s="13" t="n">
         <v>30</v>
       </c>
-      <c r="W15" s="14" t="n">
+      <c r="W15" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="X15" s="14" t="n">
+      <c r="X15" s="13" t="n">
         <v>0.3</v>
       </c>
-      <c r="Y15" s="14" t="n">
+      <c r="Y15" s="13" t="n">
         <v>0.3</v>
       </c>
-      <c r="Z15" s="14" t="n">
+      <c r="Z15" s="13" t="n">
         <v>0.12</v>
       </c>
-      <c r="AA15" s="15" t="inlineStr"/>
-      <c r="AB15" s="15" t="inlineStr"/>
-      <c r="AC15" s="15" t="inlineStr"/>
-      <c r="AD15" s="15" t="inlineStr"/>
-      <c r="AE15" s="15" t="inlineStr"/>
-      <c r="AF15" s="15" t="inlineStr"/>
-      <c r="AG15" s="16" t="inlineStr"/>
-      <c r="AH15" s="16" t="inlineStr"/>
-      <c r="AI15" s="16" t="inlineStr"/>
-      <c r="AJ15" s="16" t="inlineStr"/>
-      <c r="AK15" s="16" t="inlineStr"/>
-      <c r="AL15" s="16" t="inlineStr"/>
-      <c r="AM15" s="17" t="n">
+      <c r="AA15" s="14" t="inlineStr"/>
+      <c r="AB15" s="14" t="inlineStr"/>
+      <c r="AC15" s="14" t="inlineStr"/>
+      <c r="AD15" s="14" t="inlineStr"/>
+      <c r="AE15" s="14" t="inlineStr"/>
+      <c r="AF15" s="14" t="inlineStr"/>
+      <c r="AG15" s="15" t="inlineStr"/>
+      <c r="AH15" s="15" t="inlineStr"/>
+      <c r="AI15" s="15" t="inlineStr"/>
+      <c r="AJ15" s="15" t="inlineStr"/>
+      <c r="AK15" s="15" t="inlineStr"/>
+      <c r="AL15" s="15" t="inlineStr"/>
+      <c r="AM15" s="16" t="n">
         <v>0.3</v>
       </c>
-      <c r="AN15" s="17" t="n">
+      <c r="AN15" s="16" t="n">
         <v>0.4</v>
       </c>
-      <c r="AO15" s="17" t="n">
+      <c r="AO15" s="16" t="n">
         <v>0.5</v>
       </c>
-      <c r="AP15" s="17" t="n">
+      <c r="AP15" s="16" t="n">
         <v>0.8</v>
       </c>
-      <c r="AQ15" s="17" t="n">
+      <c r="AQ15" s="16" t="n">
         <v>0.8</v>
       </c>
-      <c r="AR15" s="17" t="n">
+      <c r="AR15" s="16" t="n">
         <v>0.24</v>
       </c>
-      <c r="AS15" s="18" t="inlineStr"/>
-      <c r="AT15" s="18" t="inlineStr"/>
-      <c r="AU15" s="18" t="inlineStr"/>
-      <c r="AV15" s="18" t="inlineStr"/>
-      <c r="AW15" s="18" t="inlineStr"/>
-      <c r="AX15" s="18" t="inlineStr"/>
-      <c r="AY15" s="19" t="inlineStr"/>
-      <c r="AZ15" s="19" t="inlineStr"/>
-      <c r="BA15" s="19" t="inlineStr"/>
-      <c r="BB15" s="19" t="inlineStr"/>
-      <c r="BC15" s="19" t="inlineStr"/>
-      <c r="BD15" s="19" t="inlineStr"/>
-      <c r="BE15" s="19" t="inlineStr"/>
-      <c r="BF15" s="20" t="inlineStr"/>
-      <c r="BG15" s="20" t="inlineStr"/>
-      <c r="BH15" s="20" t="inlineStr"/>
-      <c r="BI15" s="20" t="inlineStr"/>
-      <c r="BJ15" s="20" t="inlineStr"/>
-      <c r="BK15" s="20" t="inlineStr"/>
-      <c r="BL15" s="20" t="inlineStr"/>
+      <c r="AS15" s="17" t="inlineStr"/>
+      <c r="AT15" s="17" t="inlineStr"/>
+      <c r="AU15" s="17" t="inlineStr"/>
+      <c r="AV15" s="17" t="inlineStr"/>
+      <c r="AW15" s="17" t="inlineStr"/>
+      <c r="AX15" s="17" t="inlineStr"/>
+      <c r="AY15" s="18" t="inlineStr"/>
+      <c r="AZ15" s="18" t="inlineStr"/>
+      <c r="BA15" s="18" t="inlineStr"/>
+      <c r="BB15" s="18" t="inlineStr"/>
+      <c r="BC15" s="18" t="inlineStr"/>
+      <c r="BD15" s="18" t="inlineStr"/>
+      <c r="BE15" s="18" t="inlineStr"/>
+      <c r="BF15" s="19" t="inlineStr"/>
+      <c r="BG15" s="19" t="inlineStr"/>
+      <c r="BH15" s="19" t="inlineStr"/>
+      <c r="BI15" s="19" t="inlineStr"/>
+      <c r="BJ15" s="19" t="inlineStr"/>
+      <c r="BK15" s="19" t="inlineStr"/>
+      <c r="BL15" s="19" t="inlineStr"/>
       <c r="BM15" t="n">
         <v>0.3</v>
       </c>
@@ -2881,6 +2947,11 @@
           <t>TESTE2</t>
         </is>
       </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>AAA</t>
+        </is>
+      </c>
       <c r="G16" t="inlineStr">
         <is>
           <t>Hidrologia</t>
@@ -2910,95 +2981,95 @@
       <c r="M16" t="n">
         <v>0.2</v>
       </c>
-      <c r="N16" s="12" t="n">
+      <c r="N16" s="11" t="n">
         <v>0.6000000000000001</v>
       </c>
-      <c r="O16" s="13" t="n">
+      <c r="O16" s="12" t="n">
         <v>0.4</v>
       </c>
-      <c r="P16" s="13" t="n">
+      <c r="P16" s="12" t="n">
         <v>80</v>
       </c>
-      <c r="Q16" s="13" t="n">
+      <c r="Q16" s="12" t="n">
         <v>100</v>
       </c>
-      <c r="R16" s="13" t="n">
+      <c r="R16" s="12" t="n">
         <v>0.8</v>
       </c>
-      <c r="S16" s="13" t="n">
+      <c r="S16" s="12" t="n">
         <v>0.8</v>
       </c>
-      <c r="T16" s="13" t="n">
+      <c r="T16" s="12" t="n">
         <v>0.3200000000000001</v>
       </c>
-      <c r="U16" s="14" t="n">
+      <c r="U16" s="13" t="n">
         <v>0.4</v>
       </c>
-      <c r="V16" s="14" t="n">
+      <c r="V16" s="13" t="n">
         <v>30</v>
       </c>
-      <c r="W16" s="14" t="n">
+      <c r="W16" s="13" t="n">
         <v>100</v>
       </c>
-      <c r="X16" s="14" t="n">
+      <c r="X16" s="13" t="n">
         <v>0.3</v>
       </c>
-      <c r="Y16" s="14" t="n">
+      <c r="Y16" s="13" t="n">
         <v>0.3</v>
       </c>
-      <c r="Z16" s="14" t="n">
+      <c r="Z16" s="13" t="n">
         <v>0.12</v>
       </c>
-      <c r="AA16" s="15" t="inlineStr"/>
-      <c r="AB16" s="15" t="inlineStr"/>
-      <c r="AC16" s="15" t="inlineStr"/>
-      <c r="AD16" s="15" t="inlineStr"/>
-      <c r="AE16" s="15" t="inlineStr"/>
-      <c r="AF16" s="15" t="inlineStr"/>
-      <c r="AG16" s="16" t="inlineStr"/>
-      <c r="AH16" s="16" t="inlineStr"/>
-      <c r="AI16" s="16" t="inlineStr"/>
-      <c r="AJ16" s="16" t="inlineStr"/>
-      <c r="AK16" s="16" t="inlineStr"/>
-      <c r="AL16" s="16" t="inlineStr"/>
-      <c r="AM16" s="17" t="n">
+      <c r="AA16" s="14" t="inlineStr"/>
+      <c r="AB16" s="14" t="inlineStr"/>
+      <c r="AC16" s="14" t="inlineStr"/>
+      <c r="AD16" s="14" t="inlineStr"/>
+      <c r="AE16" s="14" t="inlineStr"/>
+      <c r="AF16" s="14" t="inlineStr"/>
+      <c r="AG16" s="15" t="inlineStr"/>
+      <c r="AH16" s="15" t="inlineStr"/>
+      <c r="AI16" s="15" t="inlineStr"/>
+      <c r="AJ16" s="15" t="inlineStr"/>
+      <c r="AK16" s="15" t="inlineStr"/>
+      <c r="AL16" s="15" t="inlineStr"/>
+      <c r="AM16" s="16" t="n">
         <v>0.2</v>
       </c>
-      <c r="AN16" s="17" t="n">
+      <c r="AN16" s="16" t="n">
         <v>0.4</v>
       </c>
-      <c r="AO16" s="17" t="n">
+      <c r="AO16" s="16" t="n">
         <v>0.5</v>
       </c>
-      <c r="AP16" s="17" t="n">
+      <c r="AP16" s="16" t="n">
         <v>0.8</v>
       </c>
-      <c r="AQ16" s="17" t="n">
+      <c r="AQ16" s="16" t="n">
         <v>0.8</v>
       </c>
-      <c r="AR16" s="17" t="n">
+      <c r="AR16" s="16" t="n">
         <v>0.16</v>
       </c>
-      <c r="AS16" s="18" t="inlineStr"/>
-      <c r="AT16" s="18" t="inlineStr"/>
-      <c r="AU16" s="18" t="inlineStr"/>
-      <c r="AV16" s="18" t="inlineStr"/>
-      <c r="AW16" s="18" t="inlineStr"/>
-      <c r="AX16" s="18" t="inlineStr"/>
-      <c r="AY16" s="19" t="inlineStr"/>
-      <c r="AZ16" s="19" t="inlineStr"/>
-      <c r="BA16" s="19" t="inlineStr"/>
-      <c r="BB16" s="19" t="inlineStr"/>
-      <c r="BC16" s="19" t="inlineStr"/>
-      <c r="BD16" s="19" t="inlineStr"/>
-      <c r="BE16" s="19" t="inlineStr"/>
-      <c r="BF16" s="20" t="inlineStr"/>
-      <c r="BG16" s="20" t="inlineStr"/>
-      <c r="BH16" s="20" t="inlineStr"/>
-      <c r="BI16" s="20" t="inlineStr"/>
-      <c r="BJ16" s="20" t="inlineStr"/>
-      <c r="BK16" s="20" t="inlineStr"/>
-      <c r="BL16" s="20" t="inlineStr"/>
+      <c r="AS16" s="17" t="inlineStr"/>
+      <c r="AT16" s="17" t="inlineStr"/>
+      <c r="AU16" s="17" t="inlineStr"/>
+      <c r="AV16" s="17" t="inlineStr"/>
+      <c r="AW16" s="17" t="inlineStr"/>
+      <c r="AX16" s="17" t="inlineStr"/>
+      <c r="AY16" s="18" t="inlineStr"/>
+      <c r="AZ16" s="18" t="inlineStr"/>
+      <c r="BA16" s="18" t="inlineStr"/>
+      <c r="BB16" s="18" t="inlineStr"/>
+      <c r="BC16" s="18" t="inlineStr"/>
+      <c r="BD16" s="18" t="inlineStr"/>
+      <c r="BE16" s="18" t="inlineStr"/>
+      <c r="BF16" s="19" t="inlineStr"/>
+      <c r="BG16" s="19" t="inlineStr"/>
+      <c r="BH16" s="19" t="inlineStr"/>
+      <c r="BI16" s="19" t="inlineStr"/>
+      <c r="BJ16" s="19" t="inlineStr"/>
+      <c r="BK16" s="19" t="inlineStr"/>
+      <c r="BL16" s="19" t="inlineStr"/>
       <c r="BM16" t="n">
         <v>0.3</v>
       </c>
@@ -3027,6 +3098,11 @@
           <t>TESTE2</t>
         </is>
       </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>AAA</t>
+        </is>
+      </c>
       <c r="G17" t="inlineStr">
         <is>
           <t>Hidrologia</t>
@@ -3056,83 +3132,83 @@
       <c r="M17" t="n">
         <v>0.15</v>
       </c>
-      <c r="N17" s="12" t="n">
+      <c r="N17" s="11" t="n">
         <v>0.5</v>
       </c>
-      <c r="O17" s="13" t="inlineStr"/>
-      <c r="P17" s="13" t="inlineStr"/>
-      <c r="Q17" s="13" t="inlineStr"/>
-      <c r="R17" s="13" t="inlineStr"/>
-      <c r="S17" s="13" t="inlineStr"/>
-      <c r="T17" s="13" t="inlineStr"/>
-      <c r="U17" s="14" t="inlineStr"/>
-      <c r="V17" s="14" t="inlineStr"/>
-      <c r="W17" s="14" t="inlineStr"/>
-      <c r="X17" s="14" t="inlineStr"/>
-      <c r="Y17" s="14" t="inlineStr"/>
-      <c r="Z17" s="14" t="inlineStr"/>
-      <c r="AA17" s="15" t="n">
+      <c r="O17" s="12" t="inlineStr"/>
+      <c r="P17" s="12" t="inlineStr"/>
+      <c r="Q17" s="12" t="inlineStr"/>
+      <c r="R17" s="12" t="inlineStr"/>
+      <c r="S17" s="12" t="inlineStr"/>
+      <c r="T17" s="12" t="inlineStr"/>
+      <c r="U17" s="13" t="inlineStr"/>
+      <c r="V17" s="13" t="inlineStr"/>
+      <c r="W17" s="13" t="inlineStr"/>
+      <c r="X17" s="13" t="inlineStr"/>
+      <c r="Y17" s="13" t="inlineStr"/>
+      <c r="Z17" s="13" t="inlineStr"/>
+      <c r="AA17" s="14" t="n">
         <v>0.4</v>
       </c>
-      <c r="AB17" s="15" t="n">
+      <c r="AB17" s="14" t="n">
         <v>80</v>
       </c>
-      <c r="AC17" s="15" t="n">
+      <c r="AC17" s="14" t="n">
         <v>100</v>
       </c>
-      <c r="AD17" s="15" t="n">
+      <c r="AD17" s="14" t="n">
         <v>0.8</v>
       </c>
-      <c r="AE17" s="15" t="n">
+      <c r="AE17" s="14" t="n">
         <v>0.8</v>
       </c>
-      <c r="AF17" s="15" t="n">
+      <c r="AF17" s="14" t="n">
         <v>0.3200000000000001</v>
       </c>
-      <c r="AG17" s="16" t="n">
+      <c r="AG17" s="15" t="n">
         <v>0.6</v>
       </c>
-      <c r="AH17" s="16" t="n">
+      <c r="AH17" s="15" t="n">
         <v>30</v>
       </c>
-      <c r="AI17" s="16" t="n">
+      <c r="AI17" s="15" t="n">
         <v>100</v>
       </c>
-      <c r="AJ17" s="16" t="n">
+      <c r="AJ17" s="15" t="n">
         <v>0.3</v>
       </c>
-      <c r="AK17" s="16" t="n">
+      <c r="AK17" s="15" t="n">
         <v>0.3</v>
       </c>
-      <c r="AL17" s="16" t="n">
+      <c r="AL17" s="15" t="n">
         <v>0.18</v>
       </c>
-      <c r="AM17" s="17" t="inlineStr"/>
-      <c r="AN17" s="17" t="inlineStr"/>
-      <c r="AO17" s="17" t="inlineStr"/>
-      <c r="AP17" s="17" t="inlineStr"/>
-      <c r="AQ17" s="17" t="inlineStr"/>
-      <c r="AR17" s="17" t="inlineStr"/>
-      <c r="AS17" s="18" t="inlineStr"/>
-      <c r="AT17" s="18" t="inlineStr"/>
-      <c r="AU17" s="18" t="inlineStr"/>
-      <c r="AV17" s="18" t="inlineStr"/>
-      <c r="AW17" s="18" t="inlineStr"/>
-      <c r="AX17" s="18" t="inlineStr"/>
-      <c r="AY17" s="19" t="inlineStr"/>
-      <c r="AZ17" s="19" t="inlineStr"/>
-      <c r="BA17" s="19" t="inlineStr"/>
-      <c r="BB17" s="19" t="inlineStr"/>
-      <c r="BC17" s="19" t="inlineStr"/>
-      <c r="BD17" s="19" t="inlineStr"/>
-      <c r="BE17" s="19" t="inlineStr"/>
-      <c r="BF17" s="20" t="inlineStr"/>
-      <c r="BG17" s="20" t="inlineStr"/>
-      <c r="BH17" s="20" t="inlineStr"/>
-      <c r="BI17" s="20" t="inlineStr"/>
-      <c r="BJ17" s="20" t="inlineStr"/>
-      <c r="BK17" s="20" t="inlineStr"/>
-      <c r="BL17" s="20" t="inlineStr"/>
+      <c r="AM17" s="16" t="inlineStr"/>
+      <c r="AN17" s="16" t="inlineStr"/>
+      <c r="AO17" s="16" t="inlineStr"/>
+      <c r="AP17" s="16" t="inlineStr"/>
+      <c r="AQ17" s="16" t="inlineStr"/>
+      <c r="AR17" s="16" t="inlineStr"/>
+      <c r="AS17" s="17" t="inlineStr"/>
+      <c r="AT17" s="17" t="inlineStr"/>
+      <c r="AU17" s="17" t="inlineStr"/>
+      <c r="AV17" s="17" t="inlineStr"/>
+      <c r="AW17" s="17" t="inlineStr"/>
+      <c r="AX17" s="17" t="inlineStr"/>
+      <c r="AY17" s="18" t="inlineStr"/>
+      <c r="AZ17" s="18" t="inlineStr"/>
+      <c r="BA17" s="18" t="inlineStr"/>
+      <c r="BB17" s="18" t="inlineStr"/>
+      <c r="BC17" s="18" t="inlineStr"/>
+      <c r="BD17" s="18" t="inlineStr"/>
+      <c r="BE17" s="18" t="inlineStr"/>
+      <c r="BF17" s="19" t="inlineStr"/>
+      <c r="BG17" s="19" t="inlineStr"/>
+      <c r="BH17" s="19" t="inlineStr"/>
+      <c r="BI17" s="19" t="inlineStr"/>
+      <c r="BJ17" s="19" t="inlineStr"/>
+      <c r="BK17" s="19" t="inlineStr"/>
+      <c r="BL17" s="19" t="inlineStr"/>
       <c r="BM17" t="n">
         <v>0.225</v>
       </c>
@@ -3161,6 +3237,11 @@
           <t>TESTE2</t>
         </is>
       </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>AAA</t>
+        </is>
+      </c>
       <c r="G18" t="inlineStr">
         <is>
           <t>Hidrologia</t>
@@ -3190,79 +3271,79 @@
       <c r="M18" t="n">
         <v>0.15</v>
       </c>
-      <c r="N18" s="12" t="n">
+      <c r="N18" s="11" t="n">
         <v>1</v>
       </c>
-      <c r="O18" s="13" t="inlineStr"/>
-      <c r="P18" s="13" t="inlineStr"/>
-      <c r="Q18" s="13" t="inlineStr"/>
-      <c r="R18" s="13" t="inlineStr"/>
-      <c r="S18" s="13" t="inlineStr"/>
-      <c r="T18" s="13" t="inlineStr"/>
-      <c r="U18" s="14" t="inlineStr"/>
-      <c r="V18" s="14" t="inlineStr"/>
-      <c r="W18" s="14" t="inlineStr"/>
-      <c r="X18" s="14" t="inlineStr"/>
-      <c r="Y18" s="14" t="inlineStr"/>
-      <c r="Z18" s="14" t="inlineStr"/>
-      <c r="AA18" s="15" t="n">
+      <c r="O18" s="12" t="inlineStr"/>
+      <c r="P18" s="12" t="inlineStr"/>
+      <c r="Q18" s="12" t="inlineStr"/>
+      <c r="R18" s="12" t="inlineStr"/>
+      <c r="S18" s="12" t="inlineStr"/>
+      <c r="T18" s="12" t="inlineStr"/>
+      <c r="U18" s="13" t="inlineStr"/>
+      <c r="V18" s="13" t="inlineStr"/>
+      <c r="W18" s="13" t="inlineStr"/>
+      <c r="X18" s="13" t="inlineStr"/>
+      <c r="Y18" s="13" t="inlineStr"/>
+      <c r="Z18" s="13" t="inlineStr"/>
+      <c r="AA18" s="14" t="n">
         <v>0.6</v>
       </c>
-      <c r="AB18" s="15" t="n">
+      <c r="AB18" s="14" t="n">
         <v>80</v>
       </c>
-      <c r="AC18" s="15" t="inlineStr"/>
-      <c r="AD18" s="15" t="n">
+      <c r="AC18" s="14" t="inlineStr"/>
+      <c r="AD18" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="AE18" s="15" t="n">
+      <c r="AE18" s="14" t="n">
         <v>1</v>
       </c>
-      <c r="AF18" s="15" t="n">
+      <c r="AF18" s="14" t="n">
         <v>0.6</v>
       </c>
-      <c r="AG18" s="16" t="n">
+      <c r="AG18" s="15" t="n">
         <v>0.4</v>
       </c>
-      <c r="AH18" s="16" t="n">
+      <c r="AH18" s="15" t="n">
         <v>30</v>
       </c>
-      <c r="AI18" s="16" t="inlineStr"/>
-      <c r="AJ18" s="16" t="n">
+      <c r="AI18" s="15" t="inlineStr"/>
+      <c r="AJ18" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="AK18" s="16" t="n">
+      <c r="AK18" s="15" t="n">
         <v>1</v>
       </c>
-      <c r="AL18" s="16" t="n">
+      <c r="AL18" s="15" t="n">
         <v>0.4</v>
       </c>
-      <c r="AM18" s="17" t="inlineStr"/>
-      <c r="AN18" s="17" t="inlineStr"/>
-      <c r="AO18" s="17" t="inlineStr"/>
-      <c r="AP18" s="17" t="inlineStr"/>
-      <c r="AQ18" s="17" t="inlineStr"/>
-      <c r="AR18" s="17" t="inlineStr"/>
-      <c r="AS18" s="18" t="inlineStr"/>
-      <c r="AT18" s="18" t="inlineStr"/>
-      <c r="AU18" s="18" t="inlineStr"/>
-      <c r="AV18" s="18" t="inlineStr"/>
-      <c r="AW18" s="18" t="inlineStr"/>
-      <c r="AX18" s="18" t="inlineStr"/>
-      <c r="AY18" s="19" t="inlineStr"/>
-      <c r="AZ18" s="19" t="inlineStr"/>
-      <c r="BA18" s="19" t="inlineStr"/>
-      <c r="BB18" s="19" t="inlineStr"/>
-      <c r="BC18" s="19" t="inlineStr"/>
-      <c r="BD18" s="19" t="inlineStr"/>
-      <c r="BE18" s="19" t="inlineStr"/>
-      <c r="BF18" s="20" t="inlineStr"/>
-      <c r="BG18" s="20" t="inlineStr"/>
-      <c r="BH18" s="20" t="inlineStr"/>
-      <c r="BI18" s="20" t="inlineStr"/>
-      <c r="BJ18" s="20" t="inlineStr"/>
-      <c r="BK18" s="20" t="inlineStr"/>
-      <c r="BL18" s="20" t="inlineStr"/>
+      <c r="AM18" s="16" t="inlineStr"/>
+      <c r="AN18" s="16" t="inlineStr"/>
+      <c r="AO18" s="16" t="inlineStr"/>
+      <c r="AP18" s="16" t="inlineStr"/>
+      <c r="AQ18" s="16" t="inlineStr"/>
+      <c r="AR18" s="16" t="inlineStr"/>
+      <c r="AS18" s="17" t="inlineStr"/>
+      <c r="AT18" s="17" t="inlineStr"/>
+      <c r="AU18" s="17" t="inlineStr"/>
+      <c r="AV18" s="17" t="inlineStr"/>
+      <c r="AW18" s="17" t="inlineStr"/>
+      <c r="AX18" s="17" t="inlineStr"/>
+      <c r="AY18" s="18" t="inlineStr"/>
+      <c r="AZ18" s="18" t="inlineStr"/>
+      <c r="BA18" s="18" t="inlineStr"/>
+      <c r="BB18" s="18" t="inlineStr"/>
+      <c r="BC18" s="18" t="inlineStr"/>
+      <c r="BD18" s="18" t="inlineStr"/>
+      <c r="BE18" s="18" t="inlineStr"/>
+      <c r="BF18" s="19" t="inlineStr"/>
+      <c r="BG18" s="19" t="inlineStr"/>
+      <c r="BH18" s="19" t="inlineStr"/>
+      <c r="BI18" s="19" t="inlineStr"/>
+      <c r="BJ18" s="19" t="inlineStr"/>
+      <c r="BK18" s="19" t="inlineStr"/>
+      <c r="BL18" s="19" t="inlineStr"/>
       <c r="BM18" t="n">
         <v>0.225</v>
       </c>
@@ -3281,7 +3362,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC3"/>
+  <dimension ref="A1:N1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -3312,318 +3393,47 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>SALDO_A_RECEBER</t>
+          <t>TOTAL_ADIANTADO_COMISSAO</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>TOTAL_COMISSAO_ANTECIPACOES</t>
+          <t>STATUS_PAGAMENTO</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>TOTAL_COMISSAO_REGULARES</t>
+          <t>STATUS_RECONCILIACAO</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>TOTAL_COMISSAO_ACUMULADA</t>
+          <t>STATUS_PROCESSO_ANALISE</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>STATUS_PROCESSO</t>
+          <t>STATUS_CALCULO_MEDIAS</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>STATUS_PAGAMENTO</t>
+          <t>MES_ANO_FATURAMENTO</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>STATUS_CALCULO_MEDIAS</t>
+          <t>TCMP</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>MES_ANO_FATURAMENTO</t>
+          <t>FCMP</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
         <is>
-          <t>TCMP_JSON</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>FCMP_JSON</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>TCMP_DETALHES_JSON</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>FCMP_DETALHES_JSON</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>COLABORADORES_ENVOLVIDOS</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>DATA_PRIMEIRO_PAGAMENTO</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>DATA_ULTIMO_PAGAMENTO</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>QUANTIDADE_PAGAMENTOS</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
           <t>ULTIMA_ATUALIZACAO</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>COMISSOES_ADIANTADAS_JSON</t>
-        </is>
-      </c>
-      <c r="X1" s="1" t="inlineStr">
-        <is>
-          <t>STATUS_RECONCILIACAO</t>
-        </is>
-      </c>
-      <c r="Y1" s="1" t="inlineStr">
-        <is>
-          <t>OBSERVACOES</t>
-        </is>
-      </c>
-      <c r="Z1" s="1" t="inlineStr">
-        <is>
-          <t>TOTAL_ADIANTADO_COMISSAO</t>
-        </is>
-      </c>
-      <c r="AA1" s="1" t="inlineStr">
-        <is>
-          <t>STATUS_PROCESSO_ANALISE</t>
-        </is>
-      </c>
-      <c r="AB1" s="1" t="inlineStr">
-        <is>
-          <t>TCMP</t>
-        </is>
-      </c>
-      <c r="AC1" s="1" t="inlineStr">
-        <is>
-          <t>FCMP</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" t="inlineStr">
-        <is>
-          <t>TESTE</t>
-        </is>
-      </c>
-      <c r="B2" t="n">
-        <v>50</v>
-      </c>
-      <c r="C2" t="n">
-        <v>0</v>
-      </c>
-      <c r="D2" t="n">
-        <v>160</v>
-      </c>
-      <c r="E2" t="n">
-        <v>160</v>
-      </c>
-      <c r="F2" t="n">
-        <v>-110</v>
-      </c>
-      <c r="G2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H2" t="n">
-        <v>0.7263999999999999</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0.7263999999999999</v>
-      </c>
-      <c r="J2" t="inlineStr">
-        <is>
-          <t>FATURADO</t>
-        </is>
-      </c>
-      <c r="K2" t="inlineStr">
-        <is>
-          <t>COMPLETO</t>
-        </is>
-      </c>
-      <c r="L2" t="inlineStr">
-        <is>
-          <t>CALCULADO</t>
-        </is>
-      </c>
-      <c r="M2" t="inlineStr">
-        <is>
-          <t>10/2025</t>
-        </is>
-      </c>
-      <c r="N2" t="inlineStr">
-        <is>
-          <t>{"André Caramello": 0.010000000000000002}</t>
-        </is>
-      </c>
-      <c r="O2" t="inlineStr">
-        <is>
-          <t>{"André Caramello": 0.4539999999999999}</t>
-        </is>
-      </c>
-      <c r="P2" t="inlineStr">
-        <is>
-          <t>{"André Caramello": {"itens": [{"negocio": "Hidrologia", "grupo": "Sonda Serie EXO", "subgrupo": "EXO", "tipo_mercadoria": "Produto", "valor": 30.0, "taxa": 0.010000000000000002, "fc": 0.47, "taxa_rateio": 0.05, "fatia_cargo": 0.2, "fc_detalhes": {"componentes": [{"nome_meta": "Faturamento da Linha", "peso": 0.15, "realizado": 80.0, "meta": 100.0, "atingimento": 0.8, "atingimento_cap": 0.8, "componente_fc": 0.12}, {"nome_meta": "Conversão da Linha", "peso": 0.3, "realizado": 30.0, "meta": 100.0, "atingimento": 0.3, "atingimento_cap": 0.3, "componente_fc": 0.09}, {"nome_meta": "Rentabilidade", "peso": 0.2, "realizado": 0.4, "meta": 0.5, "atingimento": 0.8, "atingimento_cap": 0.8, "componente_fc": 0.16000000000000003}, {"nome_meta": "Retenção de Clientes", "peso": 0.15, "realizado": 2.0, "meta": 3.0, "atingimento": 0.6666666666666666, "atingimento_cap": 0.6666666666666666, "componente_fc": 0.09999999999999999}, {"nome_meta": "Meta Fornecedor 1", "peso": 0.1, "realizado": 14.85573769241505, "meta": 25.0, "atingimento": 0.594229507696602, "atingimento_cap": 0.594229507696602, "componente_fc": 0.0594229507696602}, {"nome_meta": "Meta Fornecedor 2", "peso": 0.1, "realizado": 0.0, "meta": 25.0, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}], "fc_total": 0.47}}, {"negocio": "Hidrologia", "grupo": "Medidor de Vazão Fixo", "subgrupo": "IQ Standard", "tipo_mercadoria": "Produto", "valor": 20.0, "taxa": 0.010000000000000002, "fc": 0.42999999999999994, "taxa_rateio": 0.05, "fatia_cargo": 0.2, "fc_detalhes": {"componentes": [{"nome_meta": "Faturamento da Linha", "peso": 0.15, "realizado": 80.0, "meta": 100.0, "atingimento": 0.8, "atingimento_cap": 0.8, "componente_fc": 0.12}, {"nome_meta": "Conversão da Linha", "peso": 0.3, "realizado": 30.0, "meta": 100.0, "atingimento": 0.3, "atingimento_cap": 0.3, "componente_fc": 0.09}, {"nome_meta": "Rentabilidade", "peso": 0.2, "realizado": 0.3, "meta": 0.5, "atingimento": 0.6, "atingimento_cap": 0.6, "componente_fc": 0.12}, {"nome_meta": "Retenção de Clientes", "peso": 0.15, "realizado": 2.0, "meta": 3.0, "atingimento": 0.6666666666666666, "atingimento_cap": 0.6666666666666666, "componente_fc": 0.09999999999999999}, {"nome_meta": "Meta Fornecedor 1", "peso": 0.1, "realizado": 14.85573769241505, "meta": 25.0, "atingimento": 0.594229507696602, "atingimento_cap": 0.594229507696602, "componente_fc": 0.0594229507696602}, {"nome_meta": "Meta Fornecedor 2", "peso": 0.1, "realizado": 0.0, "meta": 25.0, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}], "fc_total": 0.42999999999999994}}], "total_valor": 50.0, "soma_ponderada": 0.5000000000000001, "tcmp_final": 0.010000000000000002}}</t>
-        </is>
-      </c>
-      <c r="Q2" t="inlineStr">
-        <is>
-          <t>{"André Caramello": {"itens": [{"negocio": "Hidrologia", "grupo": "Sonda Serie EXO", "subgrupo": "EXO", "tipo_mercadoria": "Produto", "valor": 30.0, "taxa": 0.010000000000000002, "fc": 0.47, "taxa_rateio": 0.05, "fatia_cargo": 0.2, "fc_detalhes": {"componentes": [{"nome_meta": "Faturamento da Linha", "peso": 0.15, "realizado": 80.0, "meta": 100.0, "atingimento": 0.8, "atingimento_cap": 0.8, "componente_fc": 0.12}, {"nome_meta": "Conversão da Linha", "peso": 0.3, "realizado": 30.0, "meta": 100.0, "atingimento": 0.3, "atingimento_cap": 0.3, "componente_fc": 0.09}, {"nome_meta": "Rentabilidade", "peso": 0.2, "realizado": 0.4, "meta": 0.5, "atingimento": 0.8, "atingimento_cap": 0.8, "componente_fc": 0.16000000000000003}, {"nome_meta": "Retenção de Clientes", "peso": 0.15, "realizado": 2.0, "meta": 3.0, "atingimento": 0.6666666666666666, "atingimento_cap": 0.6666666666666666, "componente_fc": 0.09999999999999999}, {"nome_meta": "Meta Fornecedor 1", "peso": 0.1, "realizado": 14.85573769241505, "meta": 25.0, "atingimento": 0.594229507696602, "atingimento_cap": 0.594229507696602, "componente_fc": 0.0594229507696602}, {"nome_meta": "Meta Fornecedor 2", "peso": 0.1, "realizado": 0.0, "meta": 25.0, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}], "fc_total": 0.47}}, {"negocio": "Hidrologia", "grupo": "Medidor de Vazão Fixo", "subgrupo": "IQ Standard", "tipo_mercadoria": "Produto", "valor": 20.0, "taxa": 0.010000000000000002, "fc": 0.42999999999999994, "taxa_rateio": 0.05, "fatia_cargo": 0.2, "fc_detalhes": {"componentes": [{"nome_meta": "Faturamento da Linha", "peso": 0.15, "realizado": 80.0, "meta": 100.0, "atingimento": 0.8, "atingimento_cap": 0.8, "componente_fc": 0.12}, {"nome_meta": "Conversão da Linha", "peso": 0.3, "realizado": 30.0, "meta": 100.0, "atingimento": 0.3, "atingimento_cap": 0.3, "componente_fc": 0.09}, {"nome_meta": "Rentabilidade", "peso": 0.2, "realizado": 0.3, "meta": 0.5, "atingimento": 0.6, "atingimento_cap": 0.6, "componente_fc": 0.12}, {"nome_meta": "Retenção de Clientes", "peso": 0.15, "realizado": 2.0, "meta": 3.0, "atingimento": 0.6666666666666666, "atingimento_cap": 0.6666666666666666, "componente_fc": 0.09999999999999999}, {"nome_meta": "Meta Fornecedor 1", "peso": 0.1, "realizado": 14.85573769241505, "meta": 25.0, "atingimento": 0.594229507696602, "atingimento_cap": 0.594229507696602, "componente_fc": 0.0594229507696602}, {"nome_meta": "Meta Fornecedor 2", "peso": 0.1, "realizado": 0.0, "meta": 25.0, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}], "fc_total": 0.42999999999999994}}], "total_valor": 50.0, "soma_ponderada": 22.699999999999996, "fcmp_final": 0.4539999999999999}}</t>
-        </is>
-      </c>
-      <c r="R2" t="inlineStr">
-        <is>
-          <t>André Caramello</t>
-        </is>
-      </c>
-      <c r="S2" s="21" t="n">
-        <v>45945</v>
-      </c>
-      <c r="T2" s="21" t="n">
-        <v>45945</v>
-      </c>
-      <c r="U2" t="n">
-        <v>4</v>
-      </c>
-      <c r="V2" s="21" t="n">
-        <v>46010.44804940972</v>
-      </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="X2" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>TESTE2</t>
-        </is>
-      </c>
-      <c r="B3" t="n">
-        <v>30</v>
-      </c>
-      <c r="C3" t="n">
-        <v>0</v>
-      </c>
-      <c r="D3" t="n">
-        <v>120</v>
-      </c>
-      <c r="E3" t="n">
-        <v>120</v>
-      </c>
-      <c r="F3" t="n">
-        <v>-90</v>
-      </c>
-      <c r="G3" t="n">
-        <v>0</v>
-      </c>
-      <c r="H3" t="n">
-        <v>0.5640000000000001</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0.5640000000000001</v>
-      </c>
-      <c r="J3" t="inlineStr">
-        <is>
-          <t>FATURADO</t>
-        </is>
-      </c>
-      <c r="K3" t="inlineStr">
-        <is>
-          <t>COMPLETO</t>
-        </is>
-      </c>
-      <c r="L3" t="inlineStr">
-        <is>
-          <t>CALCULADO</t>
-        </is>
-      </c>
-      <c r="M3" t="inlineStr">
-        <is>
-          <t>10/2025</t>
-        </is>
-      </c>
-      <c r="N3" t="inlineStr">
-        <is>
-          <t>{"André Caramello": 0.010000000000000002}</t>
-        </is>
-      </c>
-      <c r="O3" t="inlineStr">
-        <is>
-          <t>{"André Caramello": 0.47}</t>
-        </is>
-      </c>
-      <c r="P3" t="inlineStr">
-        <is>
-          <t>{"André Caramello": {"itens": [{"negocio": "Hidrologia", "grupo": "Sonda Serie EXO", "subgrupo": "EXO", "tipo_mercadoria": "Produto", "valor": 30.0, "taxa": 0.010000000000000002, "fc": 0.47, "taxa_rateio": 0.05, "fatia_cargo": 0.2, "fc_detalhes": {"componentes": [{"nome_meta": "Faturamento da Linha", "peso": 0.15, "realizado": 80.0, "meta": 100.0, "atingimento": 0.8, "atingimento_cap": 0.8, "componente_fc": 0.12}, {"nome_meta": "Conversão da Linha", "peso": 0.3, "realizado": 30.0, "meta": 100.0, "atingimento": 0.3, "atingimento_cap": 0.3, "componente_fc": 0.09}, {"nome_meta": "Rentabilidade", "peso": 0.2, "realizado": 0.4, "meta": 0.5, "atingimento": 0.8, "atingimento_cap": 0.8, "componente_fc": 0.16000000000000003}, {"nome_meta": "Retenção de Clientes", "peso": 0.15, "realizado": 2.0, "meta": 3.0, "atingimento": 0.6666666666666666, "atingimento_cap": 0.6666666666666666, "componente_fc": 0.09999999999999999}, {"nome_meta": "Meta Fornecedor 1", "peso": 0.1, "realizado": 14.85573769241505, "meta": 25.0, "atingimento": 0.594229507696602, "atingimento_cap": 0.594229507696602, "componente_fc": 0.0594229507696602}, {"nome_meta": "Meta Fornecedor 2", "peso": 0.1, "realizado": 0.0, "meta": 25.0, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}], "fc_total": 0.47}}], "total_valor": 30.0, "soma_ponderada": 0.30000000000000004, "tcmp_final": 0.010000000000000002}}</t>
-        </is>
-      </c>
-      <c r="Q3" t="inlineStr">
-        <is>
-          <t>{"André Caramello": {"itens": [{"negocio": "Hidrologia", "grupo": "Sonda Serie EXO", "subgrupo": "EXO", "tipo_mercadoria": "Produto", "valor": 30.0, "taxa": 0.010000000000000002, "fc": 0.47, "taxa_rateio": 0.05, "fatia_cargo": 0.2, "fc_detalhes": {"componentes": [{"nome_meta": "Faturamento da Linha", "peso": 0.15, "realizado": 80.0, "meta": 100.0, "atingimento": 0.8, "atingimento_cap": 0.8, "componente_fc": 0.12}, {"nome_meta": "Conversão da Linha", "peso": 0.3, "realizado": 30.0, "meta": 100.0, "atingimento": 0.3, "atingimento_cap": 0.3, "componente_fc": 0.09}, {"nome_meta": "Rentabilidade", "peso": 0.2, "realizado": 0.4, "meta": 0.5, "atingimento": 0.8, "atingimento_cap": 0.8, "componente_fc": 0.16000000000000003}, {"nome_meta": "Retenção de Clientes", "peso": 0.15, "realizado": 2.0, "meta": 3.0, "atingimento": 0.6666666666666666, "atingimento_cap": 0.6666666666666666, "componente_fc": 0.09999999999999999}, {"nome_meta": "Meta Fornecedor 1", "peso": 0.1, "realizado": 14.85573769241505, "meta": 25.0, "atingimento": 0.594229507696602, "atingimento_cap": 0.594229507696602, "componente_fc": 0.0594229507696602}, {"nome_meta": "Meta Fornecedor 2", "peso": 0.1, "realizado": 0.0, "meta": 25.0, "atingimento": 0.0, "atingimento_cap": 0.0, "componente_fc": 0.0}], "fc_total": 0.47}}], "total_valor": 30.0, "soma_ponderada": 14.1, "fcmp_final": 0.47}}</t>
-        </is>
-      </c>
-      <c r="R3" t="inlineStr">
-        <is>
-          <t>André Caramello</t>
-        </is>
-      </c>
-      <c r="S3" s="21" t="n">
-        <v>45950</v>
-      </c>
-      <c r="T3" s="21" t="n">
-        <v>45950</v>
-      </c>
-      <c r="U3" t="n">
-        <v>4</v>
-      </c>
-      <c r="V3" s="21" t="n">
-        <v>46010.44804958333</v>
-      </c>
-      <c r="W3" t="inlineStr">
-        <is>
-          <t>{}</t>
-        </is>
-      </c>
-      <c r="X3" t="inlineStr">
-        <is>
-          <t>PENDENTE</t>
         </is>
       </c>
     </row>
@@ -4721,6 +4531,11 @@
           <t>Gerente Linha</t>
         </is>
       </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>AAA</t>
+        </is>
+      </c>
       <c r="D2" t="inlineStr">
         <is>
           <t>Hidrologia</t>
@@ -4791,6 +4606,11 @@
       <c r="B3" t="inlineStr">
         <is>
           <t>Gerente Linha</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>AAA</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -4926,7 +4746,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>2025-12-19T11:26:26.948656</t>
+          <t>2026-01-06T23:03:40.156194</t>
         </is>
       </c>
     </row>
@@ -4941,7 +4761,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AV1"/>
+  <dimension ref="A1:AW1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5005,7 +4825,7 @@
           <t>taxa_rateio_aplicada</t>
         </is>
       </c>
-      <c r="M1" s="3" t="inlineStr">
+      <c r="M1" s="2" t="inlineStr">
         <is>
           <t>fator_correcao_fc</t>
         </is>
@@ -5035,152 +4855,157 @@
           <t>cross_selling_decision</t>
         </is>
       </c>
-      <c r="S1" s="4" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>numero_nf</t>
+        </is>
+      </c>
+      <c r="T1" s="3" t="inlineStr">
         <is>
           <t>peso_fat_linha</t>
         </is>
       </c>
-      <c r="T1" s="4" t="inlineStr">
+      <c r="U1" s="3" t="inlineStr">
         <is>
           <t>realizado_fat_linha</t>
         </is>
       </c>
-      <c r="U1" s="4" t="inlineStr">
+      <c r="V1" s="3" t="inlineStr">
         <is>
           <t>meta_fat_linha</t>
         </is>
       </c>
-      <c r="V1" s="4" t="inlineStr">
+      <c r="W1" s="3" t="inlineStr">
         <is>
           <t>ating_fat_linha</t>
         </is>
       </c>
-      <c r="W1" s="4" t="inlineStr">
+      <c r="X1" s="3" t="inlineStr">
         <is>
           <t>ating_cap_fat_linha</t>
         </is>
       </c>
-      <c r="X1" s="4" t="inlineStr">
+      <c r="Y1" s="3" t="inlineStr">
         <is>
           <t>comp_fc_fat_linha</t>
         </is>
       </c>
-      <c r="Y1" s="5" t="inlineStr">
+      <c r="Z1" s="4" t="inlineStr">
         <is>
           <t>peso_conv_linha</t>
         </is>
       </c>
-      <c r="Z1" s="5" t="inlineStr">
+      <c r="AA1" s="4" t="inlineStr">
         <is>
           <t>realizado_conv_linha</t>
         </is>
       </c>
-      <c r="AA1" s="5" t="inlineStr">
+      <c r="AB1" s="4" t="inlineStr">
         <is>
           <t>meta_conv_linha</t>
         </is>
       </c>
-      <c r="AB1" s="5" t="inlineStr">
+      <c r="AC1" s="4" t="inlineStr">
         <is>
           <t>ating_conv_linha</t>
         </is>
       </c>
-      <c r="AC1" s="5" t="inlineStr">
+      <c r="AD1" s="4" t="inlineStr">
         <is>
           <t>ating_cap_conv_linha</t>
         </is>
       </c>
-      <c r="AD1" s="5" t="inlineStr">
+      <c r="AE1" s="4" t="inlineStr">
         <is>
           <t>comp_fc_conv_linha</t>
         </is>
       </c>
-      <c r="AE1" s="6" t="inlineStr">
+      <c r="AF1" s="5" t="inlineStr">
         <is>
           <t>peso_fat_ind</t>
         </is>
       </c>
-      <c r="AF1" s="6" t="inlineStr">
+      <c r="AG1" s="5" t="inlineStr">
         <is>
           <t>realizado_fat_ind</t>
         </is>
       </c>
-      <c r="AG1" s="6" t="inlineStr">
+      <c r="AH1" s="5" t="inlineStr">
         <is>
           <t>meta_fat_ind</t>
         </is>
       </c>
-      <c r="AH1" s="6" t="inlineStr">
+      <c r="AI1" s="5" t="inlineStr">
         <is>
           <t>ating_fat_ind</t>
         </is>
       </c>
-      <c r="AI1" s="6" t="inlineStr">
+      <c r="AJ1" s="5" t="inlineStr">
         <is>
           <t>ating_cap_fat_ind</t>
         </is>
       </c>
-      <c r="AJ1" s="6" t="inlineStr">
+      <c r="AK1" s="5" t="inlineStr">
         <is>
           <t>comp_fc_fat_ind</t>
         </is>
       </c>
-      <c r="AK1" s="7" t="inlineStr">
+      <c r="AL1" s="6" t="inlineStr">
         <is>
           <t>peso_conv_ind</t>
         </is>
       </c>
-      <c r="AL1" s="7" t="inlineStr">
+      <c r="AM1" s="6" t="inlineStr">
         <is>
           <t>realizado_conv_ind</t>
         </is>
       </c>
-      <c r="AM1" s="7" t="inlineStr">
+      <c r="AN1" s="6" t="inlineStr">
         <is>
           <t>meta_conv_ind</t>
         </is>
       </c>
-      <c r="AN1" s="7" t="inlineStr">
+      <c r="AO1" s="6" t="inlineStr">
         <is>
           <t>ating_conv_ind</t>
         </is>
       </c>
-      <c r="AO1" s="7" t="inlineStr">
+      <c r="AP1" s="6" t="inlineStr">
         <is>
           <t>ating_cap_conv_ind</t>
         </is>
       </c>
-      <c r="AP1" s="7" t="inlineStr">
+      <c r="AQ1" s="6" t="inlineStr">
         <is>
           <t>comp_fc_conv_ind</t>
         </is>
       </c>
-      <c r="AQ1" s="10" t="inlineStr">
+      <c r="AR1" s="9" t="inlineStr">
         <is>
           <t>peso_rentab</t>
         </is>
       </c>
-      <c r="AR1" s="10" t="inlineStr">
+      <c r="AS1" s="9" t="inlineStr">
         <is>
           <t>realizado_rentab</t>
         </is>
       </c>
-      <c r="AS1" s="10" t="inlineStr">
+      <c r="AT1" s="9" t="inlineStr">
         <is>
           <t>meta_rentab</t>
         </is>
       </c>
-      <c r="AT1" s="10" t="inlineStr">
+      <c r="AU1" s="9" t="inlineStr">
         <is>
           <t>ating_rentab</t>
         </is>
       </c>
-      <c r="AU1" s="10" t="inlineStr">
+      <c r="AV1" s="9" t="inlineStr">
         <is>
           <t>ating_cap_rentab</t>
         </is>
       </c>
-      <c r="AV1" s="10" t="inlineStr">
+      <c r="AW1" s="9" t="inlineStr">
         <is>
           <t>comp_fc_rentab</t>
         </is>

</xml_diff>

<commit_message>
Adicão de documentação completa do robô de comissões e geração de diversos testes unitários e de integração da lógica do robô de comissões
</commit_message>
<xml_diff>
--- a/Calculo_Comissoes_10_2025.xlsx
+++ b/Calculo_Comissoes_10_2025.xlsx
@@ -919,6 +919,11 @@
           <t>AAA</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>ITEM 5</t>
+        </is>
+      </c>
       <c r="G2" t="inlineStr">
         <is>
           <t>Hidrologia</t>
@@ -1063,6 +1068,11 @@
           <t>AAA</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>ITEM 5</t>
+        </is>
+      </c>
       <c r="G3" t="inlineStr">
         <is>
           <t>Hidrologia</t>
@@ -1207,6 +1217,11 @@
           <t>AAA</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>ITEM 5</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr">
         <is>
           <t>Hidrologia</t>
@@ -1351,6 +1366,11 @@
           <t>AAA</t>
         </is>
       </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>ITEM 5</t>
+        </is>
+      </c>
       <c r="G5" t="inlineStr">
         <is>
           <t>Hidrologia</t>
@@ -1495,6 +1515,11 @@
           <t>AAA</t>
         </is>
       </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>ITEM 5</t>
+        </is>
+      </c>
       <c r="G6" t="inlineStr">
         <is>
           <t>Hidrologia</t>
@@ -1639,6 +1664,11 @@
           <t>AAA</t>
         </is>
       </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>ITEM 5</t>
+        </is>
+      </c>
       <c r="G7" t="inlineStr">
         <is>
           <t>Hidrologia</t>
@@ -1783,6 +1813,11 @@
           <t>BBB</t>
         </is>
       </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>ITEM 6</t>
+        </is>
+      </c>
       <c r="G8" t="inlineStr">
         <is>
           <t>Hidrologia</t>
@@ -1927,6 +1962,11 @@
           <t>BBB</t>
         </is>
       </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>ITEM 6</t>
+        </is>
+      </c>
       <c r="G9" t="inlineStr">
         <is>
           <t>Hidrologia</t>
@@ -2071,6 +2111,11 @@
           <t>BBB</t>
         </is>
       </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>ITEM 6</t>
+        </is>
+      </c>
       <c r="G10" t="inlineStr">
         <is>
           <t>Hidrologia</t>
@@ -2215,6 +2260,11 @@
           <t>BBB</t>
         </is>
       </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>ITEM 6</t>
+        </is>
+      </c>
       <c r="G11" t="inlineStr">
         <is>
           <t>Hidrologia</t>
@@ -2359,6 +2409,11 @@
           <t>BBB</t>
         </is>
       </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>ITEM 6</t>
+        </is>
+      </c>
       <c r="G12" t="inlineStr">
         <is>
           <t>Hidrologia</t>
@@ -2503,6 +2558,11 @@
           <t>BBB</t>
         </is>
       </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>ITEM 6</t>
+        </is>
+      </c>
       <c r="G13" t="inlineStr">
         <is>
           <t>Hidrologia</t>
@@ -2647,6 +2707,11 @@
           <t>AAA</t>
         </is>
       </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>ITEM 7</t>
+        </is>
+      </c>
       <c r="G14" t="inlineStr">
         <is>
           <t>Hidrologia</t>
@@ -2791,6 +2856,11 @@
           <t>AAA</t>
         </is>
       </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>ITEM 7</t>
+        </is>
+      </c>
       <c r="G15" t="inlineStr">
         <is>
           <t>Hidrologia</t>
@@ -2935,6 +3005,11 @@
           <t>AAA</t>
         </is>
       </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>ITEM 7</t>
+        </is>
+      </c>
       <c r="G16" t="inlineStr">
         <is>
           <t>Hidrologia</t>
@@ -3079,6 +3154,11 @@
           <t>AAA</t>
         </is>
       </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>ITEM 7</t>
+        </is>
+      </c>
       <c r="G17" t="inlineStr">
         <is>
           <t>Hidrologia</t>
@@ -3223,6 +3303,11 @@
           <t>AAA</t>
         </is>
       </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>ITEM 7</t>
+        </is>
+      </c>
       <c r="G18" t="inlineStr">
         <is>
           <t>Hidrologia</t>
@@ -3367,6 +3452,11 @@
           <t>AAA</t>
         </is>
       </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>ITEM 7</t>
+        </is>
+      </c>
       <c r="G19" t="inlineStr">
         <is>
           <t>Hidrologia</t>

</xml_diff>